<commit_message>
Update odds files - Sat May 30 05:36:25 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -1736,32 +1736,32 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Jahmai Jones</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>+420</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>19.2%</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>19.2%</t>
         </is>
@@ -1785,17 +1785,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+410</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
+          <t>19.6%</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
           <t>19.2%</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>19.0%</t>
         </is>
       </c>
     </row>
@@ -1834,27 +1834,27 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+493</t>
+          <t>+435</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>+390</t>
+          <t>+440</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -1866,17 +1866,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+435</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -1962,7 +1962,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Luke Raley</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2058,64 +2058,64 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+462</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+462</t>
+          <t>+493</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+410</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
@@ -2216,32 +2216,32 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Colby Thomas</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>+470</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>17.5%</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>17.5%</t>
         </is>
@@ -2794,27 +2794,27 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+576</t>
+          <t>+518</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -2826,17 +2826,17 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+518</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2851,14 +2851,14 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2890,7 +2890,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Austin Wells</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Dillon Dingler</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3018,32 +3018,32 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Austin Wells</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+596</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
@@ -3530,27 +3530,27 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Jorge Soler</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+545</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -3562,32 +3562,32 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Jorge Soler</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+545</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
@@ -3626,39 +3626,39 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Taylor Trammell</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Will Smith</t>
+          <t>Randy Arozarena</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -3690,7 +3690,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Taylor Trammell</t>
+          <t>Will Smith</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3722,27 +3722,27 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Randy Arozarena</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -3754,32 +3754,32 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>+552</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
@@ -3914,27 +3914,27 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -3944,32 +3944,32 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="inlineStr">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>Rhys Hoskins</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>+610</t>
         </is>
       </c>
-      <c r="C110" s="3" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
       </c>
-      <c r="D110" s="3" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>+570</t>
         </is>
       </c>
-      <c r="E110" s="3" t="inlineStr">
+      <c r="E110" s="2" t="inlineStr">
         <is>
           <t>14.9%</t>
         </is>
       </c>
-      <c r="F110" s="3" t="inlineStr">
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>14.5%</t>
         </is>
@@ -4921,34 +4921,34 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.1%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -4963,14 +4963,14 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.9%</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Hao-Yu Lee</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -5002,7 +5002,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Hao-Yu Lee</t>
+          <t>Wenceel Perez</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -5034,7 +5034,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Wenceel Perez</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -5066,32 +5066,32 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
@@ -6216,32 +6216,32 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="3" t="inlineStr">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>Andrew Benintendi</t>
         </is>
       </c>
-      <c r="B181" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C181" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>+790</t>
         </is>
       </c>
-      <c r="E181" s="3" t="inlineStr">
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>11.2%</t>
         </is>
       </c>
-      <c r="F181" s="3" t="inlineStr">
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>11.2%</t>
         </is>
@@ -6602,17 +6602,17 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vilade</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -6627,34 +6627,34 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.7%</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
@@ -6666,17 +6666,17 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Sandy Leon</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -6691,34 +6691,34 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>10.7%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Sandy Leon</t>
+          <t>Ryan Vilade</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F196" s="2" t="inlineStr">
@@ -7114,7 +7114,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Braden Shewmake</t>
+          <t>Carson Williams</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -7146,7 +7146,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Braden Shewmake</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -7242,27 +7242,27 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F213" s="2" t="inlineStr">
@@ -7274,59 +7274,59 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
           <t>10.2%</t>
-        </is>
-      </c>
-      <c r="F214" s="2" t="inlineStr">
-        <is>
-          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F215" s="2" t="inlineStr">
@@ -7338,27 +7338,27 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
@@ -7370,59 +7370,59 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Andruw Monasterio</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Andruw Monasterio</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
@@ -7434,17 +7434,17 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -7459,56 +7459,56 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Edgar Quero</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Edgar Quero</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -7530,17 +7530,17 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Carson Williams</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -7754,27 +7754,27 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Rodolfo Duran</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="F229" s="2" t="inlineStr">
@@ -7786,39 +7786,39 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Rodolfo Duran</t>
+          <t>Ryan Waldschmidt</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Ildemaro Vargas</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -7850,7 +7850,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -7882,7 +7882,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Ryan Waldschmidt</t>
+          <t>Ildemaro Vargas</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -8010,17 +8010,17 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -8035,39 +8035,39 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
           <t>9.1%</t>
-        </is>
-      </c>
-      <c r="D238" s="2" t="inlineStr">
-        <is>
-          <t>+980</t>
-        </is>
-      </c>
-      <c r="E238" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
-      <c r="F238" s="2" t="inlineStr">
-        <is>
-          <t>9.2%</t>
         </is>
       </c>
     </row>
@@ -8170,49 +8170,49 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Luisangel Acuna</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -8227,46 +8227,46 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Luisangel Acuna</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.7%</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -9034,27 +9034,27 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>Victor Scott II</t>
+          <t>Nico Hoerner</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1260</t>
         </is>
       </c>
       <c r="E269" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="F269" s="2" t="inlineStr">
@@ -9066,59 +9066,59 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Victor Scott II</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1280</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1300</t>
         </is>
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>Jorbit Vivas</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1340</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1260</t>
         </is>
       </c>
       <c r="E271" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="F271" s="2" t="inlineStr">
@@ -9130,7 +9130,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Jorbit Vivas</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -9290,17 +9290,17 @@
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>+1860</t>
+          <t>+1880</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update odds files - Sat May 30 13:51:55 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -559,27 +559,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>+269</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>27.1%</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>+270</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>27.0%</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>+270</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>27.0%</t>
-        </is>
-      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>27.0%</t>
+          <t>27.1%</t>
         </is>
       </c>
     </row>
@@ -714,64 +714,64 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
+          <t>+318</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>23.9%</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>+320</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>23.8%</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>+320</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>23.8%</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>+318</t>
+          <t>+320</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>+320</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.8%</t>
         </is>
       </c>
     </row>
@@ -842,96 +842,96 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+335</t>
+          <t>+336</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>22.9%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+330</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Brandon Lowe</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+335</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>22.7%</t>
+          <t>23.0%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Ben Rice</t>
+          <t>Brandon Lowe</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>+336</t>
+          <t>+350</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>22.9%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+330</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.7%</t>
         </is>
       </c>
     </row>
@@ -970,17 +970,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Trent Grisham</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+365</t>
+          <t>+374</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -995,56 +995,56 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>21.7%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Juan Soto</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+374</t>
+          <t>+369</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>21.5%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+369</t>
+          <t>+373</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1059,34 +1059,34 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Trent Grisham</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+373</t>
+          <t>+365</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.5%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+370</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1113,17 +1113,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>+370</t>
+          <t>+390</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>21.0%</t>
         </is>
       </c>
     </row>
@@ -1354,27 +1354,27 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+397</t>
+          <t>+438</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>+410</t>
+          <t>+370</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1386,27 +1386,27 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Pete Alonso</t>
+          <t>Hunter Goodman</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+418</t>
+          <t>+397</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>+390</t>
+          <t>+410</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1418,17 +1418,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+438</t>
+          <t>+418</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
@@ -1642,27 +1642,27 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+465</t>
+          <t>+432</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>+410</t>
+          <t>+440</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1674,155 +1674,155 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+458</t>
+          <t>+465</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+410</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.7%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>Kazuma Okamoto</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>+458</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>17.9%</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>Ozzie Albies</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>+448</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>18.2%</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>+430</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>18.9%</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>18.6%</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>Bobby Witt Jr.</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>+461</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>17.8%</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>+420</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>19.2%</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>18.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Dominic Canzone</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>+445</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>18.3%</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>+440</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>18.5%</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+458</t>
+          <t>+445</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+440</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1834,94 +1834,94 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Randal Grichuk</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+420</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+453</t>
+          <t>+458</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Mike Yastrzemski</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>+427</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>19.0%</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>+470</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>17.5%</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Randal Grichuk</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>+461</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>+430</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>18.9%</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t>18.3%</t>
         </is>
@@ -1930,17 +1930,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+458</t>
+          <t>+453</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1955,66 +1955,66 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>+427</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+432</t>
+          <t>+458</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+440</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2058,17 +2058,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+469</t>
+          <t>+487</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2083,78 +2083,78 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>Colby Thomas</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>+479</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>17.3%</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>+440</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>18.5%</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>17.9%</t>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Bryce Eldridge</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>+461</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>17.5%</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+477</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Luke Raley</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2186,27 +2186,27 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+459</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2218,59 +2218,59 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>+459</t>
+          <t>+486</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>+486</t>
+          <t>+536</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2344,32 +2344,32 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Spencer Steer</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>+536</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>15.7%</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>+440</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>18.5%</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Colby Thomas</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>+479</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>17.3%</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>17.1%</t>
         </is>
@@ -2504,32 +2504,32 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Jahmai Jones</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>+501</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>16.6%</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>+490</t>
         </is>
       </c>
-      <c r="E65" s="3" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>16.9%</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>16.8%</t>
         </is>
@@ -2570,7 +2570,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Jorge Soler</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2602,7 +2602,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Jorge Soler</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2858,39 +2858,39 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Ryan McMahon</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+514</t>
+          <t>+500</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
           <t>16.1%</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Ryan McMahon</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2922,27 +2922,27 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -2954,27 +2954,27 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+556</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -2986,27 +2986,27 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+525</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -3018,59 +3018,59 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Vinnie Pasquantino</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+525</t>
+          <t>+531</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
+          <t>15.8%</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>+520</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>16.1%</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
           <t>16.0%</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>+520</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>16.1%</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Vinnie Pasquantino</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+531</t>
+          <t>+514</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3178,27 +3178,27 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
+          <t>16.1%</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
           <t>15.6%</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>+520</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>16.1%</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3210,27 +3210,27 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Jonah Heim</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+523</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -3242,113 +3242,113 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Jonah Heim</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+505</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>C.J. Abrams</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+505</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+559</t>
+          <t>+543</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>C.J. Abrams</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+545</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -3370,44 +3370,44 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Dillon Dingler</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>+545</t>
+          <t>+569</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
+          <t>14.9%</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>+520</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>16.1%</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
           <t>15.5%</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>+540</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>15.6%</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Marcell Ozuna</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>+569</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -3417,17 +3417,17 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
@@ -3466,44 +3466,44 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Marcell Ozuna</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
+          <t>+548</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
           <t>+570</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr">
+      <c r="E95" s="2" t="inlineStr">
         <is>
           <t>14.9%</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>+540</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>15.6%</t>
-        </is>
-      </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+549</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -3530,44 +3530,44 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Coby Mayo</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+549</t>
+          <t>+583</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+583</t>
+          <t>+587</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -3594,91 +3594,91 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Jose Ramirez</t>
+          <t>Will Smith (LAD)</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+565</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Will Smith (LAD)</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>+565</t>
+          <t>+558</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>+558</t>
+          <t>+578</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -3690,27 +3690,27 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Rhys Hoskins</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>+578</t>
+          <t>+559</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -3946,7 +3946,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Adrian Del Castillo</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -3978,7 +3978,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Adrian Del Castillo</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -4042,7 +4042,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Brice Matthews</t>
+          <t>Harrison Bader</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -4057,17 +4057,17 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Harrison Bader</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -4138,7 +4138,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Brice Matthews</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -4170,7 +4170,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Ramon Laureano</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -4202,7 +4202,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Ramon Laureano</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -4458,7 +4458,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Nolan Gorman</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -4490,7 +4490,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Nolan Gorman</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -4650,7 +4650,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -4682,7 +4682,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -4842,7 +4842,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -5130,17 +5130,17 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>TJ Rumfield</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -5162,7 +5162,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -5194,17 +5194,17 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>TJ Rumfield</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -5322,7 +5322,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -5354,7 +5354,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -5386,7 +5386,7 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -5770,7 +5770,7 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Nick Castellanos</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
@@ -5802,7 +5802,7 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -5866,7 +5866,7 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Nick Castellanos</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -5994,7 +5994,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -6026,7 +6026,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -6090,7 +6090,7 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Crooks</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -6122,7 +6122,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Jhostynxon Garcia</t>
+          <t>Braden Shewmake</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -6154,17 +6154,17 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Jhostynxon Garcia</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -6186,7 +6186,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Jimmy Crooks</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -6218,17 +6218,17 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Braden Shewmake</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -6282,27 +6282,27 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
           <t>+820</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="E183" s="2" t="inlineStr">
         <is>
           <t>10.9%</t>
-        </is>
-      </c>
-      <c r="D183" s="2" t="inlineStr">
-        <is>
-          <t>+790</t>
-        </is>
-      </c>
-      <c r="E183" s="2" t="inlineStr">
-        <is>
-          <t>11.2%</t>
         </is>
       </c>
       <c r="F183" s="2" t="inlineStr">
@@ -6314,27 +6314,27 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
           <t>+790</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="E184" s="2" t="inlineStr">
         <is>
           <t>11.2%</t>
-        </is>
-      </c>
-      <c r="D184" s="2" t="inlineStr">
-        <is>
-          <t>+820</t>
-        </is>
-      </c>
-      <c r="E184" s="2" t="inlineStr">
-        <is>
-          <t>10.9%</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -6506,7 +6506,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -6521,12 +6521,12 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
@@ -6538,7 +6538,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Angel Martinez</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -6570,7 +6570,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Angel Martinez</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -6617,12 +6617,12 @@
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F193" s="2" t="inlineStr">
@@ -6666,7 +6666,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Connor Norby</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -6698,7 +6698,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Connor Norby</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -6730,17 +6730,17 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Sterlin Thompson</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -6755,34 +6755,34 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Sandy Leon</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F198" s="2" t="inlineStr">
@@ -6794,59 +6794,59 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Sandy Leon</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F200" s="2" t="inlineStr">
@@ -6858,96 +6858,96 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Sterlin Thompson</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
           <t>10.4%</t>
-        </is>
-      </c>
-      <c r="D203" s="2" t="inlineStr">
-        <is>
-          <t>+880</t>
-        </is>
-      </c>
-      <c r="E203" s="2" t="inlineStr">
-        <is>
-          <t>10.2%</t>
-        </is>
-      </c>
-      <c r="F203" s="2" t="inlineStr">
-        <is>
-          <t>10.3%</t>
         </is>
       </c>
     </row>
@@ -7018,27 +7018,27 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F206" s="2" t="inlineStr">
@@ -7050,27 +7050,27 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F207" s="2" t="inlineStr">
@@ -7082,7 +7082,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -7146,32 +7146,32 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Daniel Susac</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
           <t>10.1%</t>
-        </is>
-      </c>
-      <c r="D210" s="2" t="inlineStr">
-        <is>
-          <t>+880</t>
-        </is>
-      </c>
-      <c r="E210" s="2" t="inlineStr">
-        <is>
-          <t>10.2%</t>
-        </is>
-      </c>
-      <c r="F210" s="2" t="inlineStr">
-        <is>
-          <t>10.2%</t>
         </is>
       </c>
     </row>
@@ -7338,59 +7338,59 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Carlos Narvaez</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
           <t>10.0%</t>
-        </is>
-      </c>
-      <c r="D216" s="2" t="inlineStr">
-        <is>
-          <t>+920</t>
-        </is>
-      </c>
-      <c r="E216" s="2" t="inlineStr">
-        <is>
-          <t>9.8%</t>
-        </is>
-      </c>
-      <c r="F216" s="2" t="inlineStr">
-        <is>
-          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Carlos Narvaez</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
@@ -7466,91 +7466,91 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Edgar Quero</t>
+          <t>Rodolfo Duran</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
+          <t>+910</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
           <t>+920</t>
         </is>
       </c>
-      <c r="C221" s="2" t="inlineStr">
+      <c r="E221" s="2" t="inlineStr">
         <is>
           <t>9.8%</t>
         </is>
       </c>
-      <c r="D221" s="2" t="inlineStr">
-        <is>
-          <t>+920</t>
-        </is>
-      </c>
-      <c r="E221" s="2" t="inlineStr">
-        <is>
-          <t>9.8%</t>
-        </is>
-      </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="F222" s="2" t="inlineStr">
@@ -7562,17 +7562,17 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Edgar Quero</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -7594,145 +7594,145 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Luisangel Acuna</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
           <t>9.8%</t>
-        </is>
-      </c>
-      <c r="F224" s="2" t="inlineStr">
-        <is>
-          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Luisangel Acuna</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
           <t>+920</t>
         </is>
       </c>
-      <c r="C226" s="2" t="inlineStr">
+      <c r="E226" s="2" t="inlineStr">
         <is>
           <t>9.8%</t>
         </is>
       </c>
-      <c r="D226" s="2" t="inlineStr">
-        <is>
-          <t>+980</t>
-        </is>
-      </c>
-      <c r="E226" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Rodolfo Duran</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -7818,27 +7818,27 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>A.J. Ewing</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
           <t>+980</t>
         </is>
       </c>
-      <c r="C231" s="2" t="inlineStr">
+      <c r="E231" s="2" t="inlineStr">
         <is>
           <t>9.3%</t>
-        </is>
-      </c>
-      <c r="D231" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E231" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
         </is>
       </c>
       <c r="F231" s="2" t="inlineStr">
@@ -7850,27 +7850,27 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>A.J. Ewing</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C232" s="2" t="inlineStr">
+      <c r="E232" s="2" t="inlineStr">
         <is>
           <t>nan%</t>
-        </is>
-      </c>
-      <c r="D232" s="2" t="inlineStr">
-        <is>
-          <t>+980</t>
-        </is>
-      </c>
-      <c r="E232" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
         </is>
       </c>
       <c r="F232" s="2" t="inlineStr">
@@ -7882,7 +7882,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Ildemaro Vargas</t>
+          <t>Andruw Monasterio</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -7914,7 +7914,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Andruw Monasterio</t>
+          <t>Ildemaro Vargas</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -7946,7 +7946,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Bryan Torres</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -7978,7 +7978,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Bryan Torres</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -8010,7 +8010,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Alejandro Osuna</t>
+          <t>Ryan Waldschmidt</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -8042,7 +8042,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Ryan Waldschmidt</t>
+          <t>Alejandro Osuna</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -8938,7 +8938,7 @@
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Luis Torrens</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -8970,7 +8970,7 @@
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>Luis Torrens</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
@@ -9002,27 +9002,27 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>Luis Rengifo</t>
+          <t>Alex Call</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
+          <t>+1260</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>7.4%</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
           <t>+1300</t>
         </is>
       </c>
-      <c r="C268" s="2" t="inlineStr">
+      <c r="E268" s="2" t="inlineStr">
         <is>
           <t>7.1%</t>
-        </is>
-      </c>
-      <c r="D268" s="2" t="inlineStr">
-        <is>
-          <t>+1260</t>
-        </is>
-      </c>
-      <c r="E268" s="2" t="inlineStr">
-        <is>
-          <t>7.4%</t>
         </is>
       </c>
       <c r="F268" s="2" t="inlineStr">
@@ -9034,27 +9034,27 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>Alex Call</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
+          <t>+1300</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>7.1%</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
           <t>+1260</t>
         </is>
       </c>
-      <c r="C269" s="2" t="inlineStr">
+      <c r="E269" s="2" t="inlineStr">
         <is>
           <t>7.4%</t>
-        </is>
-      </c>
-      <c r="D269" s="2" t="inlineStr">
-        <is>
-          <t>+1300</t>
-        </is>
-      </c>
-      <c r="E269" s="2" t="inlineStr">
-        <is>
-          <t>7.1%</t>
         </is>
       </c>
       <c r="F269" s="2" t="inlineStr">
@@ -9066,7 +9066,7 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Luis Rengifo</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
@@ -9290,7 +9290,7 @@
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>Victor Scott II</t>
+          <t>Nico Hoerner</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -9322,7 +9322,7 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>Victor Scott II</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update odds files - Mon Jun  1 01:38:35 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -527,12 +527,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+351</t>
+          <t>+311</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -547,34 +547,34 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>24.4%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+326</t>
+          <t>+343</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -586,103 +586,103 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Eugenio Suarez</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+318</t>
+          <t>+342</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>+370</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+343</t>
+          <t>+355</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+350</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Sal Stewart</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>+343</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>22.6%</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>+360</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>21.7%</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>22.2%</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>+353</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>22.1%</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -697,81 +697,81 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Kody Clemens</t>
+          <t>Jac Caglianone</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>+353</t>
+          <t>+359</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Vinnie Pasquantino</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>+328</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>23.4%</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>+410</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>19.6%</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>21.5%</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>+374</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>21.1%</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>21.7%</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
@@ -808,34 +808,34 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Bobby Witt Jr.</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>+386</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>20.6%</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>+360</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>21.7%</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>21.2%</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Eugenio Suarez</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>+367</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>21.4%</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>+370</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>21.3%</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>21.3%</t>
         </is>
       </c>
     </row>
@@ -872,34 +872,34 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>+406</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>19.8%</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>+360</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>21.7%</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>20.8%</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Vinnie Pasquantino</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>+411</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>19.6%</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>+410</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>19.6%</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
@@ -975,12 +975,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+415</t>
+          <t>+429</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -995,24 +995,24 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>18.7%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Max Muncy</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.7%</t>
         </is>
       </c>
     </row>
@@ -1066,17 +1066,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Max Muncy</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1091,199 +1091,199 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>+437</t>
+          <t>+512</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+390</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Nolan Gorman</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>+509</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>Nolan Gorman</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>+509</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>16.4%</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t>Andrew Benintendi</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>+477</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>17.3%</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>17.3%</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Trevor Larnach</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>+486</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>17.1%</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>17.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Josh Bell</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>+494</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>16.8%</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+494</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
@@ -1514,91 +1514,91 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Will Smith</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+565</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Will Smith (LAD)</t>
+          <t>Will Smith</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+583</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Will Smith (LAD)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+583</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1610,91 +1610,91 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+589</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+589</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>14.2%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+544</t>
+          <t>+595</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1706,32 +1706,32 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Michael Massey</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
           <t>+610</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>+630</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.0%</t>
         </is>
       </c>
     </row>
@@ -1770,64 +1770,64 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Drew Romo</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
           <t>+630</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>13.7%</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Blake Dunn</t>
+          <t>Drew Romo</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+571</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
@@ -1866,32 +1866,32 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Michael Massey</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
@@ -2026,32 +2026,32 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Blake Dunn</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
+          <t>+700</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
           <t>+710</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>12.3%</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.4%</t>
         </is>
       </c>
     </row>
@@ -2090,27 +2090,27 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Danny Jansen</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2122,155 +2122,155 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Danny Jansen</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Rob Refsnyder</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
           <t>+730</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>12.0%</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Adrian Del Castillo</t>
+          <t>Rob Refsnyder</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Adrian Del Castillo</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2282,32 +2282,32 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>TJ Friedl</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
@@ -2442,251 +2442,251 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Ryan Waldschmidt</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+512</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>+1800</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>5.3%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.7%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Ryan Waldschmidt</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>10.7%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Bryan Torres</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
           <t>+920</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>9.8%</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>+790</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>11.2%</t>
-        </is>
-      </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Bryan Torres</t>
+          <t>TJ Friedl</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Austin Martin</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>+482</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>+2700</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Austin Martin</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+482</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+3500</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>2.8%</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2698,39 +2698,39 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>+509</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>+2700</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Santiago Espinal</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2745,34 +2745,34 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Kyle Isbel</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2787,66 +2787,66 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Santiago Espinal</t>
+          <t>A.J. Ewing</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Michael Helman</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+578</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -2858,7 +2858,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2890,17 +2890,17 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>A.J. Ewing</t>
+          <t>Ildemaro Vargas</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2915,56 +2915,56 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Tommy Troy</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
           <t>+980</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>9.3%</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>+980</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Michael Helman</t>
+          <t>Kyle Isbel</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2979,98 +2979,98 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Ildemaro Vargas</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Tommy Troy</t>
+          <t>Luis Torrens</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
           <t>9.1%</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>+980</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3082,155 +3082,155 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Luis Torrens</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+509</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
+          <t>16.4%</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>+7500</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>1.3%</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
           <t>8.9%</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>+980</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Miguel Rojas</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.4%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Miguel Rojas</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -3242,49 +3242,49 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Victor Robles</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Victor Robles</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -3299,39 +3299,39 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+578</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+7500</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>1.3%</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.0%</t>
         </is>
       </c>
     </row>
@@ -3498,71 +3498,71 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Nicky Lopez</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>+1560</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+3000</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.7%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Nicky Lopez</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+1560</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>+3500</t>
+          <t>+1300</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Pedro Pages</t>
+          <t>Nelson Velazquez</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3577,17 +3577,17 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>+2000</t>
+          <t>+2200</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>4.3%</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>4.3%</t>
         </is>
       </c>
     </row>
@@ -3609,17 +3609,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>+2200</t>
+          <t>+2500</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>3.8%</t>
         </is>
       </c>
     </row>
@@ -3641,24 +3641,24 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2700</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.6%</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.6%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Nelson Velazquez</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -3673,24 +3673,24 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+3000</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.2%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3705,24 +3705,24 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>+3000</t>
+          <t>+3300</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>2.9%</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>2.9%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -3737,17 +3737,17 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>+3300</t>
+          <t>+3500</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>2.8%</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>2.8%</t>
         </is>
       </c>
     </row>
@@ -3769,24 +3769,24 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>+4000</t>
+          <t>+3500</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>2.4%</t>
+          <t>2.8%</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2.4%</t>
+          <t>2.8%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Nico Hoerner</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -3801,24 +3801,24 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>+4000</t>
+          <t>+7500</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>2.4%</t>
+          <t>1.3%</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2.4%</t>
+          <t>1.3%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>Pedro Pages</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update odds files - Tue Jun  2 05:17:52 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -1608,32 +1608,32 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Tyler Stephenson</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>+404</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>19.8%</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>+470</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>17.5%</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>18.7%</t>
         </is>
@@ -1736,32 +1736,32 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Randal Grichuk</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>+441</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>18.5%</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>18.5%</t>
         </is>
@@ -2312,32 +2312,32 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>Paul Goldschmidt</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>+496</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>16.8%</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>+490</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>16.9%</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>16.9%</t>
         </is>
@@ -3400,32 +3400,32 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+      <c r="A93" s="3" t="inlineStr">
         <is>
           <t>Andrew Benintendi</t>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
+      <c r="B93" s="3" t="inlineStr">
         <is>
           <t>+568</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C93" s="3" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>

</xml_diff>

<commit_message>
Update odds files - Wed Jun  3 13:31:13 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -714,7 +714,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>C Burns</t>
+          <t>T Bradley</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -746,7 +746,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>P Tolle</t>
+          <t>C Burns</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>T Bradley</t>
+          <t>P Tolle</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -793,17 +793,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>-162</t>
+          <t>-156</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>60.9%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>60.9%</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1231,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+303</t>
+          <t>+296</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>24.8%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>24.8%</t>
+          <t>25.3%</t>
         </is>
       </c>
     </row>
@@ -1386,17 +1386,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Max Muncy (LAD)</t>
+          <t>Brandon Lowe</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+341</t>
+          <t>+338</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>22.7%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1411,24 +1411,24 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>22.7%</t>
+          <t>22.8%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Brandon Lowe</t>
+          <t>Max Muncy (LAD)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+345</t>
+          <t>+341</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.7%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1443,24 +1443,24 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.7%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+346</t>
+          <t>+345</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1475,19 +1475,19 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+347</t>
+          <t>+346</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1514,12 +1514,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+352</t>
+          <t>+353</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1546,17 +1546,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Nick Kurtz</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+353</t>
+          <t>+359</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1571,24 +1571,24 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Ben Rice</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+359</t>
+          <t>+373</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1603,24 +1603,24 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.1%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Jorge Soler</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+373</t>
+          <t>+376</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.0%</t>
         </is>
       </c>
     </row>
@@ -1674,17 +1674,17 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Jorge Soler</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+376</t>
+          <t>+378</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>+394</t>
+          <t>+393</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1795,24 +1795,24 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.3%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Hunter Goodman</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+396</t>
+          <t>+401</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
@@ -2024,34 +2024,34 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>+425</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>19.0%</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>19.0%</t>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Kerry Carpenter</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>+422</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
@@ -2088,51 +2088,51 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Luke Raley</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>+433</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>18.8%</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>18.8%</t>
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>19.0%</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Trent Grisham</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+434</t>
+          <t>+433</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2147,24 +2147,24 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Julio Rodriguez</t>
+          <t>Trent Grisham</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>+437</t>
+          <t>+434</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2179,69 +2179,69 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.7%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t>Julio Rodriguez</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>+437</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
           <t>Vinnie Pasquantino</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>+438</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>18.6%</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>18.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>+439</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>18.6%</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>18.6%</t>
         </is>
@@ -2250,103 +2250,103 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>+439</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
           <t>Salvador Perez</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>+445</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>18.3%</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>18.3%</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Dillon Dingler</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>+451</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>18.1%</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>18.1%</t>
-        </is>
-      </c>
-    </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Kerry Carpenter</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>+453</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>18.1%</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>18.1%</t>
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Nelson Velazquez</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>+459</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>17.9%</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Nelson Velazquez</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2376,78 +2376,78 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Ian Happ</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>+459</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>17.9%</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>+460</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>17.9%</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>17.9%</t>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Yandy Diaz</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>+461</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>+463</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -2474,17 +2474,17 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Matt Olson</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>+463</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2499,14 +2499,14 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Matt Olson</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2538,7 +2538,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2570,12 +2570,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>+471</t>
+          <t>+472</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2602,17 +2602,17 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>+472</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -2627,19 +2627,19 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -2666,17 +2666,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Ketel Marte</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>+476</t>
+          <t>+478</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
@@ -2762,12 +2762,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Will Smith (LAD)</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>+488</t>
+          <t>+489</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -2794,7 +2794,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Nathaniel Lowe</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2826,17 +2826,17 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Nathaniel Lowe</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+489</t>
+          <t>+491</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2851,24 +2851,24 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+495</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2883,37 +2883,37 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Brent Rooker</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>+495</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Henry Davis</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>+496</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>16.8%</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>16.8%</t>
         </is>
@@ -2922,17 +2922,17 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Henry Davis</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+496</t>
+          <t>+510</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2947,24 +2947,24 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Tyler O'Neill</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>+504</t>
+          <t>+511</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2979,24 +2979,24 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Ronald Acuna Jr.</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+504</t>
+          <t>+515</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3011,24 +3011,24 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Jose Ramirez</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+510</t>
+          <t>+516</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3043,24 +3043,24 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Tyler O'Neill</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+511</t>
+          <t>+517</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -3075,56 +3075,56 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>Ronald Acuna Jr.</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>+515</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>16.3%</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>16.3%</t>
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>+519</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Will Smith (LAD)</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+516</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3139,24 +3139,24 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+517</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -3171,56 +3171,56 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Basallo</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>+519</t>
-        </is>
-      </c>
-      <c r="C86" s="3" t="inlineStr">
-        <is>
-          <t>16.2%</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E86" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F86" s="3" t="inlineStr">
-        <is>
-          <t>16.2%</t>
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Torkelson</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>+525</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>16.0%</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+523</t>
+          <t>+525</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3235,19 +3235,19 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+525</t>
+          <t>+526</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -3274,17 +3274,17 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+528</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -3299,24 +3299,24 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -3331,19 +3331,19 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+534</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -3370,17 +3370,17 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+537</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3395,14 +3395,14 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -3434,17 +3434,17 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Andrew Benintendi</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>+538</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -3459,14 +3459,14 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3498,12 +3498,12 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Andrew Benintendi</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+543</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -3530,17 +3530,17 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Christopher Morel</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+546</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -3555,24 +3555,24 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+549</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -3587,24 +3587,24 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Christopher Morel</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>+546</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -3619,51 +3619,51 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>Alex Bregman</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>+552</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>15.3%</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>15.3%</t>
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Jake Bauers</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>+557</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+559</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -3688,32 +3688,32 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="3" t="inlineStr">
-        <is>
-          <t>Jake Bauers</t>
-        </is>
-      </c>
-      <c r="B102" s="3" t="inlineStr">
-        <is>
-          <t>+557</t>
-        </is>
-      </c>
-      <c r="C102" s="3" t="inlineStr">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Dansby Swanson</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>15.2%</t>
         </is>
       </c>
-      <c r="D102" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E102" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F102" s="3" t="inlineStr">
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
         <is>
           <t>15.2%</t>
         </is>
@@ -3722,17 +3722,17 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>+559</t>
+          <t>+565</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -3747,24 +3747,24 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Coby Mayo</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>+560</t>
+          <t>+568</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -3779,24 +3779,24 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>+568</t>
+          <t>+571</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -3811,14 +3811,14 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -4010,7 +4010,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -4042,17 +4042,17 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Tristan Gray</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>+582</t>
+          <t>+583</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -4067,19 +4067,19 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Tristan Gray</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>+583</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -4106,7 +4106,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -4138,7 +4138,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -4170,12 +4170,12 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>CJ Abrams</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+586</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -4234,12 +4234,12 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Kyle Stowers</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+594</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -4330,7 +4330,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Eric Haase</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -4362,7 +4362,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -4394,7 +4394,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Eric Haase</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -4458,7 +4458,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -4522,7 +4522,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -4554,17 +4554,17 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Jake Rogers</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Daulton Varsho</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -4778,17 +4778,17 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Daulton Varsho</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -4803,88 +4803,88 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="inlineStr">
-        <is>
-          <t>Ivan Herrera</t>
-        </is>
-      </c>
-      <c r="B137" s="2" t="inlineStr">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>Willson Contreras</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
         <is>
           <t>+650</t>
         </is>
       </c>
-      <c r="C137" s="2" t="inlineStr">
+      <c r="C137" s="3" t="inlineStr">
         <is>
           <t>13.3%</t>
         </is>
       </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E137" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F137" s="2" t="inlineStr">
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
         <is>
           <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="3" t="inlineStr">
-        <is>
-          <t>Willson Contreras</t>
-        </is>
-      </c>
-      <c r="B138" s="3" t="inlineStr">
-        <is>
-          <t>+650</t>
-        </is>
-      </c>
-      <c r="C138" s="3" t="inlineStr">
-        <is>
-          <t>13.3%</t>
-        </is>
-      </c>
-      <c r="D138" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E138" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F138" s="3" t="inlineStr">
-        <is>
-          <t>13.3%</t>
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Curtis Mead</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -4899,24 +4899,24 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -4931,14 +4931,14 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -4970,7 +4970,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -5034,17 +5034,17 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -5059,14 +5059,14 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Jacob Gonzalez</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -5162,17 +5162,17 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Blake Dunn</t>
+          <t>Jacob Gonzalez</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -5187,14 +5187,14 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Jake Rogers</t>
+          <t>Blake Dunn</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -5226,17 +5226,17 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -5251,24 +5251,24 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Vaughn Grissom</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -5283,14 +5283,14 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -5322,7 +5322,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -5354,17 +5354,17 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -5379,88 +5379,88 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>T.J. Rumfield</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
         <is>
           <t>+710</t>
         </is>
       </c>
-      <c r="C155" s="2" t="inlineStr">
+      <c r="C155" s="3" t="inlineStr">
         <is>
           <t>12.3%</t>
         </is>
       </c>
-      <c r="D155" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E155" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F155" s="2" t="inlineStr">
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
         <is>
           <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B156" s="3" t="inlineStr">
-        <is>
-          <t>+710</t>
-        </is>
-      </c>
-      <c r="C156" s="3" t="inlineStr">
-        <is>
-          <t>12.3%</t>
-        </is>
-      </c>
-      <c r="D156" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E156" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F156" s="3" t="inlineStr">
-        <is>
-          <t>12.3%</t>
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Matt McLain</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -5475,7 +5475,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
@@ -5514,7 +5514,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -5546,17 +5546,17 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Vaughn Grissom</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -5571,24 +5571,24 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -5603,24 +5603,24 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -5635,24 +5635,24 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -5667,24 +5667,24 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -5699,24 +5699,24 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -5731,14 +5731,14 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -5770,17 +5770,17 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -5795,24 +5795,24 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Amed Rosario</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -5827,24 +5827,24 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Jorge Mateo</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -5859,24 +5859,24 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -5891,24 +5891,24 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Ryan Ward</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -5923,24 +5923,24 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Jorge Mateo</t>
+          <t>Drew Romo</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -5955,56 +5955,56 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="3" t="inlineStr">
-        <is>
-          <t>Amed Rosario</t>
-        </is>
-      </c>
-      <c r="B173" s="3" t="inlineStr">
-        <is>
-          <t>+770</t>
-        </is>
-      </c>
-      <c r="C173" s="3" t="inlineStr">
-        <is>
-          <t>11.5%</t>
-        </is>
-      </c>
-      <c r="D173" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F173" s="3" t="inlineStr">
-        <is>
-          <t>11.5%</t>
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>J.T. Realmuto</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -6019,14 +6019,14 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Drew Romo</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -6058,17 +6058,17 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Nico Hoerner</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -6083,24 +6083,24 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -6115,56 +6115,56 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>Nico Hoerner</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>+800</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>11.1%</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E178" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F178" s="2" t="inlineStr">
-        <is>
-          <t>11.1%</t>
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Victor Mesa Jr.</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -6179,56 +6179,56 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="3" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B180" s="3" t="inlineStr">
-        <is>
-          <t>+810</t>
-        </is>
-      </c>
-      <c r="C180" s="3" t="inlineStr">
-        <is>
-          <t>11.0%</t>
-        </is>
-      </c>
-      <c r="D180" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E180" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F180" s="3" t="inlineStr">
-        <is>
-          <t>11.0%</t>
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>Edwin Arroyo</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>+830</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Victor Mesa Jr.</t>
+          <t>Esteury Ruiz</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -6243,24 +6243,24 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Keibert Ruiz</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
@@ -6314,17 +6314,17 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Keibert Ruiz</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -6339,24 +6339,24 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Esteury Ruiz</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
@@ -6410,7 +6410,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -6474,17 +6474,17 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -6499,24 +6499,24 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Drew Gilbert</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.3%</t>
         </is>
       </c>
     </row>
@@ -6570,7 +6570,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Taylor Trammell</t>
+          <t>Danny Jansen</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Drew Gilbert</t>
+          <t>Taylor Trammell</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -6634,17 +6634,17 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Danny Jansen</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -6659,14 +6659,14 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Rikuu Nishida</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -6698,7 +6698,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -6730,17 +6730,17 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Rikuu Nishida</t>
+          <t>Pavin Smith</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -6755,14 +6755,14 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Pavin Smith</t>
+          <t>Ildemaro Vargas</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -6922,7 +6922,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -6986,7 +6986,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -7018,7 +7018,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Colt Keith</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -7050,7 +7050,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -7082,17 +7082,17 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -7107,14 +7107,14 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Matt Vierling</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -7146,7 +7146,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Matt Vierling</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -7178,17 +7178,17 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Connor Norby</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -7203,14 +7203,14 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Miguel Amaya</t>
+          <t>Connor Norby</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -7242,7 +7242,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>J.C. Escarra</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -7274,7 +7274,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>J.C. Escarra</t>
+          <t>Miguel Amaya</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -7306,17 +7306,17 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -7331,24 +7331,24 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -7363,14 +7363,14 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Luis Rengifo</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -7402,7 +7402,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Luis Rengifo</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -7434,7 +7434,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Kyle Isbel</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -7466,7 +7466,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>Sterlin Thompson</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -7498,7 +7498,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Sterlin Thompson</t>
+          <t>Kyle Isbel</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -7530,17 +7530,17 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -7555,24 +7555,24 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -7587,14 +7587,14 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Thomas Saggese</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -7626,7 +7626,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Thomas Saggese</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -7658,7 +7658,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -7690,7 +7690,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -7722,12 +7722,12 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Gleyber Torres</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
@@ -7754,7 +7754,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -7786,7 +7786,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -7818,7 +7818,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Gleyber Torres</t>
+          <t>Jared Triolo</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -7850,17 +7850,17 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -7875,14 +7875,14 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Ha-Seong Kim</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -7914,7 +7914,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Cesar Salazar</t>
+          <t>Ha-Seong Kim</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -7946,7 +7946,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Cesar Salazar</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -7978,7 +7978,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Troy Johnston</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Patrick Bailey</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -8138,7 +8138,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Patrick Bailey</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -8266,17 +8266,17 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Jacob Young</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -8362,7 +8362,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Jhonny Pereda</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -8394,17 +8394,17 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Nick Fortes</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -8419,24 +8419,24 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Jhonny Pereda</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -8451,7 +8451,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
@@ -8490,17 +8490,17 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>Jose Fermin (STL)</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -8515,24 +8515,24 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Nick Fortes</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -8547,24 +8547,24 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>Tyler Freeman</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -8579,24 +8579,24 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>Austin Martin</t>
+          <t>Jose Fermin (STL)</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -8611,14 +8611,14 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Tyler Freeman</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -8682,7 +8682,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>Ildemaro Vargas</t>
+          <t>Sal Frelick</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -8714,7 +8714,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>Sal Frelick</t>
+          <t>Richie Palacios</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
@@ -8746,17 +8746,17 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>Masataka Yoshida</t>
+          <t>David Hamilton</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
@@ -8810,17 +8810,17 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Masataka Yoshida</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -8835,14 +8835,14 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Ryan Waldschmidt</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -8874,7 +8874,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>Ryan Waldschmidt</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -8906,7 +8906,7 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>Richie Palacios</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -9007,12 +9007,12 @@
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
@@ -9130,7 +9130,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Austin Martin</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
@@ -9162,7 +9162,7 @@
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
@@ -9226,17 +9226,17 @@
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>Jacob Young</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1240</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.5%</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -9251,7 +9251,7 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.5%</t>
         </is>
       </c>
     </row>
@@ -9514,17 +9514,17 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>Nasim Nunez</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+1420</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -9539,24 +9539,24 @@
       </c>
       <c r="F284" s="2" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Jake Mangum</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>+1420</t>
+          <t>+1540</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -9571,24 +9571,24 @@
       </c>
       <c r="F285" s="2" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.1%</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>Jake Mangum</t>
+          <t>Nasim Nunez</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>+1560</t>
+          <t>+1540</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -9603,7 +9603,7 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.1%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun  4 02:31:16 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,12 +68,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -435,10 +444,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -481,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>U 5.5</t>
+          <t>S. Suzuki</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -496,24 +505,24 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>-1400</t>
+          <t>-1200</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>93.3%</t>
+          <t>92.3%</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>93.3%</t>
+          <t>92.3%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T. Stephenson</t>
+          <t>U 8.5</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -528,24 +537,24 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>-350</t>
+          <t>-550</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>84.6%</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>84.6%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>D. Lee</t>
+          <t>S Imanaga</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -560,24 +569,24 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>-245</t>
+          <t>-184</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>64.8%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>64.8%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S Imanaga</t>
+          <t>C Rodon</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -592,24 +601,24 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>-184</t>
+          <t>-152</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>60.3%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>60.3%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>W Urena</t>
+          <t>C Crow</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -624,24 +633,24 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>-172</t>
+          <t>-150</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>63.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>63.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>A. Pallante</t>
+          <t>U 11.5</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -656,24 +665,24 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>-162</t>
+          <t>-144</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>59.0%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>59.0%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C Crow</t>
+          <t>Z. Gallen</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -688,24 +697,24 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>-160</t>
+          <t>-140</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>61.5%</t>
+          <t>58.3%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>61.5%</t>
+          <t>58.3%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>C Rodon</t>
+          <t>O 9.5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -720,24 +729,24 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>-154</t>
+          <t>-136</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>57.6%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>57.6%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>O 9.5</t>
+          <t>O 10.5</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -752,24 +761,24 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>-138</t>
+          <t>-130</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>56.5%</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>56.5%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>S. Suzuki</t>
+          <t>C Sale</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -784,24 +793,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>-136</t>
+          <t>-125</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>55.6%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>O 6.5</t>
+          <t>Z Wheeler</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -816,24 +825,24 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>-130</t>
+          <t>-120</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>56.5%</t>
+          <t>54.5%</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>56.5%</t>
+          <t>54.5%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>U 8.5</t>
+          <t>O 7.5</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -848,24 +857,24 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>-128</t>
+          <t>-110</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>56.1%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>56.1%</t>
+          <t>52.4%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C Sale</t>
+          <t>U 7.5</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -880,24 +889,24 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>-125</t>
+          <t>-110</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>52.4%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>U 4.5</t>
+          <t>N. Madrigal</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -912,24 +921,24 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>-122</t>
+          <t>-108</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>51.9%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>U 7.5</t>
+          <t>U 10.5</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -944,24 +953,24 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>-120</t>
+          <t>-102</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>50.5%</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>50.5%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Z Wheeler</t>
+          <t>U 9.5</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -976,24 +985,24 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>-120</t>
+          <t>+102</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>49.5%</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>49.5%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Z Gallen</t>
+          <t>O 11.5</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1008,24 +1017,24 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>-120</t>
+          <t>+108</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>48.1%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>48.1%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>O 10.5</t>
+          <t>R Nelson</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1040,24 +1049,24 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>-118</t>
+          <t>+115</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>54.1%</t>
+          <t>46.5%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>54.1%</t>
+          <t>46.5%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>U 10.5</t>
+          <t>A Morris</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1072,24 +1081,24 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>-112</t>
+          <t>+140</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>41.7%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>O 7.5</t>
+          <t>N. Allen</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1104,24 +1113,24 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>+140</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>41.7%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>O 4.5</t>
+          <t>B Bello</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1136,24 +1145,24 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>-108</t>
+          <t>+146</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>40.7%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>O 8.5</t>
+          <t>K Teng</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1168,56 +1177,56 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>-104</t>
+          <t>+150</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>51.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>51.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>U 6.5</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>-102</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>50.5%</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>50.5%</t>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Schwarber</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>+204</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>32.9%</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>32.9%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>U 9.5</t>
+          <t>O 8.5</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1232,290 +1241,290 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>+104</t>
+          <t>+350</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>R Nelson</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>+116</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>46.3%</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>46.3%</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>+355</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>22.0%</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>22.0%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>G. Mitchell</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+441</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>+130</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Adolis Garcia</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>+140</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>K Teng</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>+150</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>40.0%</t>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>+501</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>16.6%</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>A Morris</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+557</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>R. Watson</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+559</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>+158</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>38.8%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>38.8%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>S. Arrighetti</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+575</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>+158</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>38.8%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>38.8%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>J. Chisholm</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+591</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>+164</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>37.9%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>37.9%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+309</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1530,24 +1539,24 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+318</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1562,24 +1571,24 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Jorge Soler</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+365</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1594,24 +1603,24 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Max Muncy (LAD)</t>
+          <t>Jase Bowen</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+392</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1626,24 +1635,24 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+411</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1658,24 +1667,24 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+436</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1690,24 +1699,24 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Miguel Andujar</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+544</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1722,24 +1731,24 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Will Smith (LAD)</t>
+          <t>Freddy Fermin</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1754,24 +1763,24 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Justin Crawford</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>+564</t>
+          <t>+1260</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1786,935 +1795,39 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>7.4%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>I. Herrera</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+1300</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Logan O'Hoppe</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>+620</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>13.9%</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>13.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>O 5.5</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>+630</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Wade Meckler</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>+630</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Oswald Peraza</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>+630</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Donovan Walton</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>+650</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>13.3%</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>13.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Mookie Betts</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>+660</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>13.2%</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>13.2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Kyle Tucker</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>+670</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>13.0%</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>13.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>T.J. Rumfield</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>+720</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>12.2%</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>12.2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Vaughn Grissom</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>+730</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>12.0%</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>12.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Nolan Arenado</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>+810</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>11.0%</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>11.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Willi Castro</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>+900</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>10.0%</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>10.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Troy Johnston</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>+920</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>9.8%</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>9.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Edouard Julien</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>+930</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>9.7%</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>9.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Pavin Smith</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>+940</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>9.6%</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>9.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Sterlin Thompson</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>+950</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>9.5%</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>9.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Gabriel Moreno</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>+970</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Jake McCarthy</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>+1000</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>9.1%</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>9.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Alex Freeland</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>+1000</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>9.1%</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>9.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>J. Duran</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>+1000</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>9.1%</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>9.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Kyle Karros</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>+1040</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>8.8%</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>8.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Jose Fernandez</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>+1080</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>8.5%</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>8.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Tyler Freeman</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>+1140</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>8.1%</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>8.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Ildemaro Vargas</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>+1220</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>7.6%</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>7.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>Ryan Waldschmidt</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>+1240</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>7.5%</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>7.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Geraldo Perdomo</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>+1260</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>7.4%</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>7.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>Alex Call</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>+1380</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>6.8%</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>6.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Tommy Troy</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>+1400</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>6.7%</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>6.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Nick Madrigal</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>+1480</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>6.3%</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>6.3%</t>
+          <t>7.1%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun  4 04:17:55 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -444,10 +444,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S. Suzuki</t>
+          <t>R. Waldschmidt</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -505,24 +505,24 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>-1200</t>
+          <t>-310</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>75.6%</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>75.6%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>U 8.5</t>
+          <t>S Imanaga</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -537,24 +537,24 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>-550</t>
+          <t>-182</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>64.5%</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>64.5%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S Imanaga</t>
+          <t>C Rodon</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -569,24 +569,24 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>-184</t>
+          <t>-152</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>60.3%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>60.3%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>C Rodon</t>
+          <t>O 7.5</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -601,17 +601,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>-152</t>
+          <t>-144</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>60.3%</t>
+          <t>59.0%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>60.3%</t>
+          <t>59.0%</t>
         </is>
       </c>
     </row>
@@ -633,24 +633,24 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>-150</t>
+          <t>-137</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>57.8%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>57.8%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>U 11.5</t>
+          <t>U 10.5</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -665,24 +665,24 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>-144</t>
+          <t>-130</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>56.5%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>56.5%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Z. Gallen</t>
+          <t>C Sale</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -697,24 +697,24 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>-140</t>
+          <t>-125</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>58.3%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>58.3%</t>
+          <t>55.6%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>O 9.5</t>
+          <t>U 8.5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -729,24 +729,24 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>-136</t>
+          <t>-122</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>55.0%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>O 10.5</t>
+          <t>Z Wheeler</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -761,24 +761,24 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>-130</t>
+          <t>-122</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>56.5%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>56.5%</t>
+          <t>55.0%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>C Sale</t>
+          <t>U 9.5</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -793,24 +793,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>-125</t>
+          <t>-122</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>55.0%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Z Wheeler</t>
+          <t>O 9.5</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>-120</t>
+          <t>+100</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>O 7.5</t>
+          <t>O 8.5</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -857,24 +857,24 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>+100</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>U 7.5</t>
+          <t>O 10.5</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -889,24 +889,24 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>-110</t>
+          <t>+106</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>48.5%</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>48.5%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>N. Madrigal</t>
+          <t>U 7.5</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -921,24 +921,24 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>-108</t>
+          <t>+108</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>48.1%</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>48.1%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>U 10.5</t>
+          <t>R Nelson</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -953,24 +953,24 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>-102</t>
+          <t>+114</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>50.5%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>50.5%</t>
+          <t>46.7%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>U 9.5</t>
+          <t>A Morris</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -985,24 +985,24 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>+102</t>
+          <t>+140</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>49.5%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>49.5%</t>
+          <t>41.7%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>O 11.5</t>
+          <t>B Bello</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1017,24 +1017,24 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>+108</t>
+          <t>+146</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>48.1%</t>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>48.1%</t>
+          <t>40.7%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>R Nelson</t>
+          <t>K Teng</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1049,258 +1049,258 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>+115</t>
+          <t>+146</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>46.5%</t>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>46.5%</t>
+          <t>40.7%</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>A Morris</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>+140</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>41.7%</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>41.7%</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Schwarber</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>+195</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>33.9%</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>33.9%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>N. Allen</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+247</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>28.8%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>+140</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>28.8%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>B Bello</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+255</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>+146</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>28.2%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>K Teng</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+283</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>26.1%</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Kyle Schwarber</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>+204</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>32.9%</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>32.9%</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Brent Rooker</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>+287</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>25.8%</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>O 8.5</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>+350</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>22.2%</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>22.2%</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Willson Contreras</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>+293</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>25.4%</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>25.4%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>+355</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>22.0%</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>22.0%</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Matt Olson</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>+308</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>24.5%</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>24.5%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>+441</t>
+          <t>+312</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1315,24 +1315,24 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>24.3%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Adolis Garcia</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+316</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1347,56 +1347,56 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>24.0%</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>+501</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>16.6%</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>16.6%</t>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Byron Buxton</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>+328</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>23.4%</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>23.4%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Trent Grisham</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+557</t>
+          <t>+352</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>22.1%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1411,24 +1411,24 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+559</t>
+          <t>+356</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>21.9%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1443,56 +1443,56 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Gavin Sheets</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>+575</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>14.8%</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>14.8%</t>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>+357</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>21.9%</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+591</t>
+          <t>+362</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1507,24 +1507,24 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>21.6%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+366</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>21.5%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1539,24 +1539,24 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>21.5%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Colby Thomas</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+369</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1571,24 +1571,24 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>21.3%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+376</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1603,24 +1603,24 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>21.0%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Jase Bowen</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+381</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1635,24 +1635,24 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Austin Wells</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+394</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1667,24 +1667,24 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Xander Bogaerts</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+395</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1699,24 +1699,24 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Miguel Andujar</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+403</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1731,103 +1731,2823 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>Cody Bellinger</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>+413</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>+413</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>+413</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Carter Jensen</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>+415</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>+419</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>19.3%</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>19.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Ward</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>+422</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Gavin Sheets</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>+422</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Paul Goldschmidt</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>+440</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Ryan McMahon</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>18.2%</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>18.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Ronald Acuna Jr.</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>+453</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>18.1%</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>18.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Seiya Suzuki</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>+453</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>18.1%</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>18.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Vinnie Pasquantino</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>+457</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Gunnar Henderson</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>+463</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Adley Rutschman</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>+482</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>17.2%</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>17.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Adolis Garcia</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>+491</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Austin Riley</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>+507</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>16.5%</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>16.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Jackson Merrill</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>+511</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>16.4%</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>16.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Michael Harris</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>+512</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Zack Gelof</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>+512</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Andruw Monasterio</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>+531</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Brandon Marsh</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>+532</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Wilyer Abreu</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Narvaez</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>+541</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Josh Bell</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>+547</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Jarren Duran</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>+555</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Henry Bolte</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>+556</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Trea Turner</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Angel Martinez</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>+567</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>+579</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Drake Baldwin</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>+586</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Manny Machado</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Kazuma Okamoto</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Chase DeLauter</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Isaac Collins</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Dansby Swanson</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Alex Bregman</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Coby Mayo</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Brooks Lee</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Moises Ballesteros</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Marcelo Mayer</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>J.T. Realmuto</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Vladimir Guerrero Jr.</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>David Fry</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Anthony Volpe</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Bryson Stott</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Colton Cowser</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>George Springer</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Alec Bohm</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Ozzie Albies</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Jase Bowen</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Mike Yastrzemski</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Ty France</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Jeff McNeil</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Caleb Durbin</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Victor Caratini</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Travis Bazzana</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Michael Massey</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Carson Kelly</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Tristan Gray</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Nico Hoerner</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>+830</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Trevor Larnach</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Isiah Kiner-Falefa</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Ernie Clement</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Jackson Holliday</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Darell Hernaiz</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>+870</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Nick Loftin</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Brayan Rocchio</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Charles McAdoo</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Jose Caballero</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Xander Bogaerts</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Luke Keaschall</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Leody Taveras</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>+970</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Andujar</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>K. Yates</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Jorge Mateo</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
           <t>Freddy Fermin</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>+880</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>10.2%</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>10.2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Austin Hedges</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Isbel</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
         <is>
           <t>Justin Crawford</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>+1260</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>7.4%</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>7.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>I. Herrera</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>+1300</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>7.1%</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>7.1%</t>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Daulton Varsho</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Austin Martin</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Sandy Leon</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Myles Straw</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>+1360</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>6.8%</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>6.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Yohendrick Pinango</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>6.7%</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>6.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Tyler Heineman</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>+1660</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>5.7%</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>5.7%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun  4 13:40:58 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -586,7 +586,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>U 8.5</t>
+          <t>C Sale</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -601,24 +601,24 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>-122</t>
+          <t>-126</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>55.8%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>55.8%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>C Sale</t>
+          <t>U 8.5</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -650,7 +650,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Z Wheeler</t>
+          <t>U 10.5</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -665,24 +665,24 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>-118</t>
+          <t>-115</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>54.1%</t>
+          <t>53.5%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>54.1%</t>
+          <t>53.5%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>U 10.5</t>
+          <t>Z Wheeler</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -697,17 +697,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>-115</t>
+          <t>-114</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>53.5%</t>
+          <t>53.3%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>53.5%</t>
+          <t>53.3%</t>
         </is>
       </c>
     </row>
@@ -857,17 +857,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>+118</t>
+          <t>+115</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>45.9%</t>
+          <t>46.5%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>45.9%</t>
+          <t>46.5%</t>
         </is>
       </c>
     </row>
@@ -953,17 +953,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+152</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>39.7%</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>39.7%</t>
         </is>
       </c>
     </row>
@@ -975,12 +975,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+218</t>
+          <t>+225</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>31.4%</t>
+          <t>30.8%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>31.4%</t>
+          <t>30.8%</t>
         </is>
       </c>
     </row>
@@ -1071,12 +1071,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+277</t>
+          <t>+271</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>27.0%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>27.0%</t>
         </is>
       </c>
     </row>
@@ -1103,12 +1103,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>+286</t>
+          <t>+275</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>26.7%</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1231,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+320</t>
+          <t>+315</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>24.1%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1251,56 +1251,56 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>24.1%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>+339</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>22.8%</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>22.8%</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Colby Thomas</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>+347</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>22.4%</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Colby Thomas</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>+347</t>
+          <t>+349</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>22.3%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1315,39 +1315,39 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>22.3%</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Jazz Chisholm</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>+349</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>22.3%</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>22.3%</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>+352</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>22.1%</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
@@ -1448,34 +1448,34 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Cody Bellinger</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>+390</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>20.4%</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>20.4%</t>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>+382</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>20.7%</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1546,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Jose Ramirez</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+395</t>
+          <t>+390</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1571,19 +1571,19 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+396</t>
+          <t>+395</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1608,83 +1608,83 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Bobby Witt Jr.</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>+397</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>20.1%</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>20.1%</t>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Gavin Sheets</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>+395</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>20.2%</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Gavin Sheets</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>+397</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>20.1%</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>20.1%</t>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>+395</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>20.2%</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+399</t>
+          <t>+396</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1699,19 +1699,19 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+399</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1738,17 +1738,17 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Matt Olson</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+402</t>
+          <t>+400</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1763,88 +1763,88 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Matt Olson</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>+403</t>
+          <t>+400</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
+          <t>20.0%</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>20.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Christian Walker</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>+402</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
           <t>19.9%</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>19.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Basallo</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>+411</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>19.6%</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Brandon Lowe</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+413</t>
+          <t>+407</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1859,56 +1859,56 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>19.7%</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Seiya Suzuki</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>+414</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>19.5%</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>19.5%</t>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>+411</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>19.6%</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>+415</t>
+          <t>+413</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1923,56 +1923,56 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>+419</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>19.3%</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>19.3%</t>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Carter Jensen</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>+414</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Brandon Lowe</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+414</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1987,24 +1987,24 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Ryan McMahon</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+415</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.4%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2019,24 +2019,24 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.4%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Ketel Marte</t>
+          <t>Ryan McMahon</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+426</t>
+          <t>+420</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2051,24 +2051,24 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Oneil Cruz</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+426</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2083,24 +2083,24 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Oneil Cruz</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+433</t>
+          <t>+428</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
@@ -2216,51 +2216,51 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Will Smith (LAD)</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>+449</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>18.2%</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>18.2%</t>
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>+444</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>18.4%</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Ronald Acuna Jr.</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>+445</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2275,24 +2275,24 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Ronald Acuna Jr.</t>
+          <t>Will Smith (LAD)</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>+467</t>
+          <t>+449</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2307,24 +2307,24 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Vinnie Pasquantino</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>+468</t>
+          <t>+457</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2339,88 +2339,88 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>Jake Bauers</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>+469</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>17.6%</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>17.6%</t>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Gunnar Henderson</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>+461</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>+471</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>17.5%</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>17.5%</t>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Josh Bell</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>+464</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>17.7%</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>+481</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2435,56 +2435,56 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Vinnie Pasquantino</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>+484</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>17.1%</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>17.1%</t>
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Jake Bauers</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>+469</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>17.6%</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>+488</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2499,24 +2499,24 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+481</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2531,19 +2531,19 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.2%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Adolis Garcia</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -2570,17 +2570,17 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>Adolis Garcia</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>+496</t>
+          <t>+491</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -2595,24 +2595,24 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+493</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -2627,24 +2627,24 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Coby Mayo</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>+509</t>
+          <t>+496</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2659,24 +2659,24 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Austin Riley</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>+509</t>
+          <t>+502</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2691,24 +2691,24 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Tristan Gray</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>+512</t>
+          <t>+504</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
@@ -2735,12 +2735,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>+512</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2755,24 +2755,24 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>+513</t>
+          <t>+509</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2787,24 +2787,24 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+517</t>
+          <t>+509</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -2819,24 +2819,24 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+519</t>
+          <t>+510</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2851,24 +2851,24 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+521</t>
+          <t>+512</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2883,24 +2883,24 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>+525</t>
+          <t>+515</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2915,24 +2915,24 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Austin Riley</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+517</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2947,24 +2947,24 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+519</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2979,19 +2979,19 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+525</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3018,17 +3018,17 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Tristan Gray</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+536</t>
+          <t>+525</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3043,24 +3043,24 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+542</t>
+          <t>+526</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -3075,24 +3075,24 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+530</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -3107,24 +3107,24 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+545</t>
+          <t>+531</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3139,24 +3139,24 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+561</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
@@ -3210,17 +3210,17 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+569</t>
+          <t>+574</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3235,24 +3235,24 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+569</t>
+          <t>+577</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -3267,24 +3267,24 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+574</t>
+          <t>+581</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -3299,24 +3299,24 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+577</t>
+          <t>+582</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -3331,24 +3331,24 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Angel Martinez</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>+588</t>
+          <t>+583</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -3363,24 +3363,24 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Angel Martinez</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>+594</t>
+          <t>+588</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3395,24 +3395,24 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+594</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -3427,14 +3427,14 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3466,62 +3466,62 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
+          <t>Matt Chapman</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="B95" s="2" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>+600</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B96" s="3" t="inlineStr">
-        <is>
-          <t>+600</t>
-        </is>
-      </c>
-      <c r="C96" s="3" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F96" s="3" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
@@ -3560,32 +3560,32 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>Matt Chapman</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
         <is>
           <t>+600</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C98" s="3" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
@@ -3594,7 +3594,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -3626,17 +3626,17 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Andruw Monasterio</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -3651,24 +3651,24 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Carlos Narvaez</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -3683,46 +3683,46 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="3" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B102" s="3" t="inlineStr">
-        <is>
-          <t>+610</t>
-        </is>
-      </c>
-      <c r="C102" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
-        </is>
-      </c>
-      <c r="D102" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E102" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F102" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>George Springer</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Eric Haase</t>
+          <t>Andruw Monasterio</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -3752,32 +3752,32 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>J.T. Realmuto</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
         <is>
           <t>+610</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr">
+      <c r="C104" s="3" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr">
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
@@ -3786,7 +3786,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Eric Haase</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -3818,17 +3818,17 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Carlos Narvaez</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -3843,24 +3843,24 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -3875,24 +3875,24 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -3907,14 +3907,14 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>David Fry</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -3978,7 +3978,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>David Fry</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -4010,7 +4010,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -4042,7 +4042,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -4074,17 +4074,17 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Anthony Volpe</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -4099,24 +4099,24 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Anthony Volpe</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -4131,24 +4131,24 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -4163,24 +4163,24 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -4195,24 +4195,24 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -4227,14 +4227,14 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Jorge Mateo</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -4266,7 +4266,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Jase Bowen</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -4298,7 +4298,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Jase Bowen</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -4362,17 +4362,17 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Jorge Mateo</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
@@ -4586,7 +4586,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Brice Matthews</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -4682,17 +4682,17 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Brice Matthews</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -4707,24 +4707,24 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -4739,24 +4739,24 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -4771,14 +4771,14 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Charles McAdoo</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -4810,17 +4810,17 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Sal Frelick</t>
+          <t>Charles McAdoo</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -4835,14 +4835,14 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Taylor Trammell</t>
+          <t>Sal Frelick</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -4874,17 +4874,17 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Taylor Trammell</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
@@ -5386,17 +5386,17 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Kyle Isbel</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -5411,14 +5411,14 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Austin Hedges</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -5450,17 +5450,17 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Miguel Andujar</t>
+          <t>Austin Hedges</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -5475,14 +5475,14 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Isiah Kiner-Falefa</t>
+          <t>Miguel Andujar</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -5546,17 +5546,17 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Isiah Kiner-Falefa</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5610,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Kyle Isbel</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -5738,17 +5738,17 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -5763,24 +5763,24 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -5795,24 +5795,24 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Tommy Troy</t>
+          <t>Austin Martin</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -5827,24 +5827,24 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -5859,24 +5859,24 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Myles Straw</t>
+          <t>Tommy Troy</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -5891,24 +5891,24 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Daulton Varsho</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -5923,24 +5923,24 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Daulton Varsho</t>
+          <t>Myles Straw</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>+1220</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -5955,24 +5955,24 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>Austin Martin</t>
+          <t>Cesar Salazar</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -5987,24 +5987,24 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Cesar Salazar</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -6019,24 +6019,24 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Tyler Heineman</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1260</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -6051,24 +6051,24 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.4%</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Tyler Heineman</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1280</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
@@ -6095,12 +6095,12 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>+1540</t>
+          <t>+1420</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Sat Jun  6 03:12:42 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,12 +68,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -435,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -481,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>J. Beeks</t>
+          <t>L. Nootbaar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -496,24 +505,24 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>-245</t>
+          <t>-450</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>81.8%</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>81.8%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>B Brown</t>
+          <t>M Liberatore</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -528,17 +537,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>-188</t>
+          <t>-192</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>65.3%</t>
+          <t>65.8%</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>65.3%</t>
+          <t>65.8%</t>
         </is>
       </c>
     </row>
@@ -560,24 +569,24 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>-188</t>
+          <t>-192</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>65.3%</t>
+          <t>65.8%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>65.3%</t>
+          <t>65.8%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>A Painter</t>
+          <t>B Brown</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -592,24 +601,24 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>-176</t>
+          <t>-184</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>63.8%</t>
+          <t>64.8%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>63.8%</t>
+          <t>64.8%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>J Ryan</t>
+          <t>A Painter</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -624,24 +633,24 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>-170</t>
+          <t>-172</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>63.0%</t>
+          <t>63.2%</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>63.0%</t>
+          <t>63.2%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>E Rodriguez</t>
+          <t>J Ryan</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -656,24 +665,24 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>-156</t>
+          <t>-166</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>60.9%</t>
+          <t>62.4%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>60.9%</t>
+          <t>62.4%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>J. Crooks</t>
+          <t>U 9.5</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -688,24 +697,24 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>-144</t>
+          <t>-158</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>61.2%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>61.2%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>O 6.5</t>
+          <t>E Rodriguez</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -720,24 +729,24 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>-140</t>
+          <t>-156</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>58.3%</t>
+          <t>60.9%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>58.3%</t>
+          <t>60.9%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>O 9.5</t>
+          <t>P. Abner</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -752,24 +761,24 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>-138</t>
+          <t>-154</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>60.6%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>G. Perdomo</t>
+          <t>U 13.5</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -784,24 +793,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>-136</t>
+          <t>-154</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>60.6%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>R. Sasaki</t>
+          <t>T. France</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -816,24 +825,24 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>-136</t>
+          <t>-146</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>59.3%</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>59.3%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>U 8.5</t>
+          <t>U 16.5</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -848,24 +857,24 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>-132</t>
+          <t>-144</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>59.0%</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>59.0%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>U 7.5</t>
+          <t>U 5.5</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -880,24 +889,24 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>-132</t>
+          <t>-138</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>58.0%</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>58.0%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>T. Johnston</t>
+          <t>U 8.5</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -912,24 +921,24 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>-132</t>
+          <t>-120</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>54.5%</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>54.5%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>T. Gray</t>
+          <t>O 6.5</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -944,24 +953,24 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>-130</t>
+          <t>-118</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>56.5%</t>
+          <t>54.1%</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>56.5%</t>
+          <t>54.1%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>O 8.5</t>
+          <t>M. Betts</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -976,17 +985,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>+100</t>
+          <t>-118</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>54.1%</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>54.1%</t>
         </is>
       </c>
     </row>
@@ -1008,24 +1017,24 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>+100</t>
+          <t>-115</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>53.5%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>53.5%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>U 9.5</t>
+          <t>U 6.5</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1040,24 +1049,24 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>+104</t>
+          <t>-112</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>52.8%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>52.8%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>U 6.5</t>
+          <t>O 8.5</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1072,24 +1081,24 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>+106</t>
+          <t>-110</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>48.5%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>48.5%</t>
+          <t>52.4%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Z. Matthews</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1104,24 +1113,24 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>+118</t>
+          <t>-106</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>45.9%</t>
+          <t>51.5%</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>45.9%</t>
+          <t>51.5%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Y Yamamoto</t>
+          <t>U 7.5</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1136,24 +1145,24 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>+126</t>
+          <t>-105</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>44.2%</t>
+          <t>51.2%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>44.2%</t>
+          <t>51.2%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>M. King</t>
+          <t>O 5.5</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1168,24 +1177,24 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>+128</t>
+          <t>+104</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>43.9%</t>
+          <t>49.0%</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>43.9%</t>
+          <t>49.0%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>K Montero</t>
+          <t>O 16.5</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1200,24 +1209,24 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>+128</t>
+          <t>+108</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>43.9%</t>
+          <t>48.1%</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>43.9%</t>
+          <t>48.1%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>G Canning</t>
+          <t>A. Senzatela</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1232,24 +1241,24 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>+134</t>
+          <t>+110</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>42.7%</t>
+          <t>47.6%</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>42.7%</t>
+          <t>47.6%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>T Imai</t>
+          <t>L Bachar</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1264,24 +1273,24 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>+146</t>
+          <t>+115</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>46.5%</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>46.5%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>O 13.5</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1296,24 +1305,24 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>+155</t>
+          <t>+116</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>39.2%</t>
+          <t>46.3%</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>39.2%</t>
+          <t>46.3%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>S Strider</t>
+          <t>O 9.5</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1328,24 +1337,24 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>+160</t>
+          <t>+118</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>38.5%</t>
+          <t>45.9%</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>38.5%</t>
+          <t>45.9%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>M Liberatore</t>
+          <t>Y Yamamoto</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1360,24 +1369,24 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>+164</t>
+          <t>+126</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>37.9%</t>
+          <t>44.2%</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>37.9%</t>
+          <t>44.2%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>J Leiter</t>
+          <t>K Montero</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1392,24 +1401,24 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>+168</t>
+          <t>+128</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>37.3%</t>
+          <t>43.9%</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>37.3%</t>
+          <t>43.9%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>N. Allen</t>
+          <t>G Canning</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1424,162 +1433,162 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>+168</t>
+          <t>+134</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>37.3%</t>
+          <t>42.7%</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>37.3%</t>
+          <t>42.7%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>T Imai</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+448</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+146</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>40.7%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+465</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+155</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>39.2%</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>39.2%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>S Strider</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+158</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>38.8%</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>38.8%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>J Leiter</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+478</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>nan%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+168</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>nan%</t>
+          <t>37.3%</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>37.3%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Oneil Cruz</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+481</t>
+          <t>+285</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1594,24 +1603,24 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>26.0%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Matt Olson</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+486</t>
+          <t>+288</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1626,24 +1635,24 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Brandon Lowe</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+303</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>24.8%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1658,24 +1667,24 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>24.8%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+330</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1690,24 +1699,24 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>23.3%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+342</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1722,24 +1731,24 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>22.6%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+342</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1754,24 +1763,24 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>22.6%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+361</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1786,24 +1795,24 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>21.7%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Vinnie Pasquantino</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+368</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1818,24 +1827,24 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+381</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1850,120 +1859,120 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Moises Ballesteros</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>+950</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>9.5%</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>9.5%</t>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>+391</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>20.4%</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Drew Gilbert</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>+980</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>9.3%</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>20.0%</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Carson Kelly</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>+1140</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>8.1%</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>8.1%</t>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>+414</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+427</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1978,39 +1987,2471 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
+          <t>Kerry Carpenter</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>+437</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Bryce Eldridge</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>+442</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Wilyer Abreu</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>+449</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>18.2%</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>18.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Paul Goldschmidt</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>18.2%</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>18.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Willson Contreras</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>+461</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Julio Rodriguez</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>+462</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Bryan Reynolds</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>+463</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Ian Happ</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>+469</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>17.6%</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>17.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Willy Adames</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>+476</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>17.4%</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>17.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Pete Crow-Armstrong</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>+478</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>17.3%</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>17.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Casey Schmitt</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>+478</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>17.3%</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>17.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Dillon Dingler</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>+492</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Ronald Acuna Jr.</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>+498</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Torkelson</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>+502</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>16.6%</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>16.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Jarren Duran</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>+507</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>16.5%</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>16.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Trent Grisham</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>+523</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>16.1%</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>16.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Cody Bellinger</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>+523</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>16.1%</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>16.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Riley Greene</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>+526</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>16.0%</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>16.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Josh Bell</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>+539</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Trevor Larnach</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>+563</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Austin Riley</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Brooks Lee</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>+574</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Seiya Suzuki</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>+576</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Amed Rosario</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>+582</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Ryan O'Hearn</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>+584</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Jazz Chisholm</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>+595</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>14.4%</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>14.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>+596</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>14.4%</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>14.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Michael Busch</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Michael Massey</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Austin Wells</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Randy Arozarena</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Horwitz</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Josh Naylor</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>James Outman</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Endy Rodriguez</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Orlando Arcia</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Dominic Smith</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Ozzie Albies</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Alex Bregman</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Colt Emerson</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Nick Gonzales</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Kevin McGonigle</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>J.P. Crawford</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Matt Chapman</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Moises Ballesteros</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Victor Caratini</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Mike Yastrzemski</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Ceddanne Rafaela</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Isaac Collins</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Tristan Gray</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Isbel</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Marcelo Mayer</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Susac</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Dansby Swanson</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Nick Loftin</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>+830</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Colt Keith</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>+830</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Masataka Yoshida</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Luke Keaschall</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Jose Caballero</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Jhonny Pereda</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Gleyber Torres</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>+910</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Michael Gasper</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>+910</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Cole Young</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Drew Gilbert</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Anthony Volpe</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Jared Triolo</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Sandy Leon</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Wenceel Perez</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Carson Kelly</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Matt Vierling</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Caleb Durbin</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Jung Hoo Lee</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Jake Mangum</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>+1160</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Mauricio Dubon</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>+1220</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Luis Arraez</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>+1220</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
           <t>Nico Hoerner</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B124" s="2" t="inlineStr">
         <is>
           <t>+1300</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C124" s="2" t="inlineStr">
         <is>
           <t>7.1%</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
         <is>
           <t>7.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Isiah Kiner-Falefa</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Sat Jun  6 11:34:58 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -650,7 +650,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>B Brown</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>B Brown</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>-154</t>
+          <t>-160</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>61.5%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>61.5%</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>B Fisher</t>
+          <t>T Imai</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1145,24 +1145,24 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+146</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>40.7%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>T Imai</t>
+          <t>B Fisher</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1177,17 +1177,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>+155</t>
+          <t>+150</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>39.2%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>39.2%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1418,17 +1418,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+288</t>
+          <t>+291</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>25.6%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1443,24 +1443,24 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>25.6%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Max Muncy (LAD)</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+291</t>
+          <t>+295</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1475,24 +1475,24 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.3%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Max Muncy (LAD)</t>
+          <t>Oneil Cruz</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+295</t>
+          <t>+298</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>25.3%</t>
+          <t>25.1%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>25.3%</t>
+          <t>25.1%</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1546,17 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Oneil Cruz</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+298</t>
+          <t>+301</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>24.9%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>24.9%</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+310</t>
+          <t>+311</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
     </row>
@@ -1736,83 +1736,83 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Christian Walker</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>+340</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>22.7%</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>22.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>Jake Bauers</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>+341</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>22.7%</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>22.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Juan Soto</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>+343</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>22.6%</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>22.6%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+345</t>
+          <t>+343</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1827,24 +1827,24 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.6%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Dominic Canzone</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+348</t>
+          <t>+345</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1859,24 +1859,24 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+354</t>
+          <t>+348</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>22.3%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>22.3%</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Eugenio Suarez</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -1962,7 +1962,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Eugenio Suarez</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -2378,7 +2378,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2410,7 +2410,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Jose Ramirez</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2442,94 +2442,94 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>Andy Pages</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>+407</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>19.7%</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>19.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
           <t>Casey Schmitt</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>+407</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>19.7%</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>19.7%</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
         <is>
           <t>Bobby Witt Jr.</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>+407</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>19.7%</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>19.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Pete Alonso</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>+408</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>19.7%</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>19.7%</t>
         </is>
@@ -2538,17 +2538,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Vinnie Pasquantino</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>+415</t>
+          <t>+408</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2563,14 +2563,14 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.7%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Vinnie Pasquantino</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2922,7 +2922,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Dillon Dingler</t>
+          <t>Andrew Benintendi</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Andrew Benintendi</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3018,7 +3018,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3050,7 +3050,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3082,7 +3082,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -3114,17 +3114,17 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+455</t>
+          <t>+459</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3139,19 +3139,19 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Will Smith (LAD)</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+459</t>
+          <t>+460</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -3178,17 +3178,17 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Will Smith (LAD)</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>+460</t>
+          <t>+464</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -3203,24 +3203,24 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+464</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3235,24 +3235,24 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+468</t>
+          <t>+472</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -3267,19 +3267,19 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+472</t>
+          <t>+473</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -3306,17 +3306,17 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+473</t>
+          <t>+477</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -3331,19 +3331,19 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -3368,83 +3368,83 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>Zach Neto</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>+479</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>17.3%</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>17.3%</t>
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>+486</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>17.1%</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>+486</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="inlineStr">
-        <is>
-          <t>17.1%</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F93" s="3" t="inlineStr">
-        <is>
-          <t>17.1%</t>
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Manzardo</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>+488</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>17.0%</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>17.0%</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>+488</t>
+          <t>+491</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -3459,24 +3459,24 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+495</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -3491,24 +3491,24 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Ronald Acuna Jr.</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>+495</t>
+          <t>+498</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -3523,19 +3523,19 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Ronald Acuna Jr.</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+500</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -3562,17 +3562,17 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+501</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -3587,24 +3587,24 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>+501</t>
+          <t>+506</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -3619,19 +3619,19 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>+506</t>
+          <t>+507</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -3658,17 +3658,17 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>+507</t>
+          <t>+509</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Trent Grisham</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -3818,7 +3818,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Trent Grisham</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3914,17 +3914,17 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>+536</t>
+          <t>+534</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -3939,101 +3939,101 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
+          <t>Wyatt Langford</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>+536</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>15.7%</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>15.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
           <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
-      <c r="B110" s="2" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>+537</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>15.7%</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>15.7%</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="3" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
         <is>
           <t>+544</t>
         </is>
       </c>
-      <c r="C111" s="3" t="inlineStr">
+      <c r="C112" s="3" t="inlineStr">
         <is>
           <t>15.5%</t>
         </is>
       </c>
-      <c r="D111" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E111" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F111" s="3" t="inlineStr">
-        <is>
-          <t>15.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>Bryce Eldridge</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>+545</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>15.5%</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F112" s="2" t="inlineStr">
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
         <is>
           <t>15.5%</t>
         </is>
@@ -4042,12 +4042,12 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>+546</t>
+          <t>+545</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -4074,17 +4074,17 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>+549</t>
+          <t>+546</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
@@ -4138,17 +4138,17 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Angel Martinez</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+559</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -4163,24 +4163,24 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Angel Martinez</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>+559</t>
+          <t>+562</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -4195,14 +4195,14 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -4232,66 +4232,66 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>Carlos Cortes</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="inlineStr">
-        <is>
-          <t>+562</t>
-        </is>
-      </c>
-      <c r="C119" s="2" t="inlineStr">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>+564</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
         <is>
           <t>15.1%</t>
         </is>
       </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="inlineStr">
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
         <is>
           <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Basallo</t>
-        </is>
-      </c>
-      <c r="B120" s="3" t="inlineStr">
-        <is>
-          <t>+564</t>
-        </is>
-      </c>
-      <c r="C120" s="3" t="inlineStr">
-        <is>
-          <t>15.1%</t>
-        </is>
-      </c>
-      <c r="D120" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E120" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F120" s="3" t="inlineStr">
-        <is>
-          <t>15.1%</t>
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Coby Mayo</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Eric Haase</t>
+          <t>Dane Myers</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -4458,7 +4458,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Dane Myers</t>
+          <t>Eric Haase</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -4650,7 +4650,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Curtis Mead</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -4714,7 +4714,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -4746,7 +4746,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -4842,7 +4842,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Heriberto Hernandez</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Heriberto Hernandez</t>
+          <t>Yandy Diaz</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -4904,32 +4904,32 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="3" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B140" s="3" t="inlineStr">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Randy Arozarena</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>+610</t>
         </is>
       </c>
-      <c r="C140" s="3" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
       </c>
-      <c r="D140" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E140" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F140" s="3" t="inlineStr">
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
@@ -4938,7 +4938,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Randy Arozarena</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -4970,7 +4970,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Christopher Morel</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -5000,32 +5000,32 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="inlineStr">
-        <is>
-          <t>Gavin Sheets</t>
-        </is>
-      </c>
-      <c r="B143" s="2" t="inlineStr">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
         <is>
           <t>+610</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr">
+      <c r="C143" s="3" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
       </c>
-      <c r="D143" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E143" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F143" s="2" t="inlineStr">
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
@@ -5034,7 +5034,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Christopher Morel</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Amed Rosario</t>
+          <t>Austin Wells</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -5130,7 +5130,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Austin Wells</t>
+          <t>Amed Rosario</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -5162,7 +5162,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -5194,17 +5194,17 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Michael Massey</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -5219,14 +5219,14 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Michael Massey</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -5258,17 +5258,17 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -5283,14 +5283,14 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -5322,7 +5322,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -5386,7 +5386,7 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -5418,17 +5418,17 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Andres Chaparro</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -5443,14 +5443,14 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Andres Chaparro</t>
+          <t>Drew Romo</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -5514,7 +5514,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Drew Romo</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -5610,7 +5610,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -5642,7 +5642,7 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -5674,7 +5674,7 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -5834,7 +5834,7 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
@@ -5898,7 +5898,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -5930,7 +5930,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -5994,7 +5994,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -6026,7 +6026,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Evan Carter</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -6058,7 +6058,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Evan Carter</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -6154,7 +6154,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -6186,17 +6186,17 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -6211,24 +6211,24 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -6243,14 +6243,14 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -6282,17 +6282,17 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -6307,14 +6307,14 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>CJ Abrams</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -6346,7 +6346,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -6378,7 +6378,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -6474,7 +6474,7 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Lars Nootbaar</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -6506,7 +6506,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -6538,17 +6538,17 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Lars Nootbaar</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -6563,14 +6563,14 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Rikuu Nishida</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -6634,17 +6634,17 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Rikuu Nishida</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -6659,14 +6659,14 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Victor Mesa Jr.</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -6730,7 +6730,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Victor Mesa Jr.</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -6762,17 +6762,17 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
@@ -6826,17 +6826,17 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Patrick Bailey</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -6851,24 +6851,24 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Patrick Bailey</t>
+          <t>Jesus Sanchez</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
@@ -6922,17 +6922,17 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Jesus Sanchez</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -6947,14 +6947,14 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Danny Jansen</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -6986,7 +6986,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Danny Jansen</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -7018,17 +7018,17 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -7043,14 +7043,14 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Sterlin Thompson</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -7114,7 +7114,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Sterlin Thompson</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -7178,17 +7178,17 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Jhonny Pereda</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -7203,14 +7203,14 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Jhonny Pereda</t>
+          <t>Colt Keith</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -7274,17 +7274,17 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>Connor Norby</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -7299,7 +7299,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7338,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Connor Norby</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -7370,17 +7370,17 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -7395,14 +7395,14 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -7434,7 +7434,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Masataka Yoshida</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -7466,7 +7466,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Masataka Yoshida</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -7498,7 +7498,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -7530,7 +7530,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -7626,7 +7626,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -7658,7 +7658,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -7690,7 +7690,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -7722,7 +7722,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Gleyber Torres</t>
+          <t>Tommy Troy</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -7754,17 +7754,17 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Gleyber Torres</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -7779,14 +7779,14 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Richie Palacios</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -7818,7 +7818,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Tommy Troy</t>
+          <t>Richie Palacios</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -7914,17 +7914,17 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Sandy Leon</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -7939,14 +7939,14 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>David Hamilton</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -8010,17 +8010,17 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -8035,7 +8035,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
@@ -8074,7 +8074,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Hayden Senger</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Miguel Andujar</t>
+          <t>Hayden Senger</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -8138,17 +8138,17 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Miguel Andujar</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -8163,7 +8163,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
@@ -8202,7 +8202,7 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Keibert Ruiz</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -8234,7 +8234,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Keibert Ruiz</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -8394,12 +8394,12 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Kyle Isbel</t>
+          <t>Matt Vierling</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
@@ -8426,7 +8426,7 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Justin Crawford</t>
+          <t>Kyle Isbel</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -8458,7 +8458,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>Matt Vierling</t>
+          <t>Justin Crawford</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -8554,7 +8554,7 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Drew Gilbert</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -8586,7 +8586,7 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>Drew Gilbert</t>
+          <t>Esteury Ruiz</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -8618,7 +8618,7 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>Esteury Ruiz</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -8655,12 +8655,12 @@
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>Sandy Leon</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
@@ -8874,17 +8874,17 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -8899,7 +8899,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
@@ -8938,17 +8938,17 @@
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Jared Triolo</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -8963,24 +8963,24 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>Christian Vazquez</t>
+          <t>Jorge Barrosa</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
@@ -8995,14 +8995,14 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>Jorge Barrosa</t>
+          <t>Christian Vazquez</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
@@ -9194,7 +9194,7 @@
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Hunter Feduccia</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -9258,7 +9258,7 @@
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>Hunter Feduccia</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
@@ -9290,7 +9290,7 @@
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>Jake Mangum</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -9354,17 +9354,17 @@
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Xavier Edwards</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1240</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.5%</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -9379,7 +9379,7 @@
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.5%</t>
         </is>
       </c>
     </row>
@@ -9418,17 +9418,17 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>Xavier Edwards</t>
+          <t>Darell Hernaiz</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1280</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -9443,14 +9443,14 @@
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
@@ -9482,7 +9482,7 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>Darell Hernaiz</t>
+          <t>Nick Allen</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
@@ -9514,7 +9514,7 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>Nick Allen</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
@@ -9546,7 +9546,7 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
@@ -9578,17 +9578,17 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Victor Scott II</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1300</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
@@ -9603,24 +9603,24 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.1%</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>Victor Scott II</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -9635,14 +9635,14 @@
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.0%</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
@@ -9706,17 +9706,17 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Nico Hoerner</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1340</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -9731,24 +9731,24 @@
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>6.9%</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>Jake Mangum</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1360</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -9763,7 +9763,7 @@
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Sat Jun  6 11:49:41 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -1130,7 +1130,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T Imai</t>
+          <t>B Fisher</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1145,24 +1145,24 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>+146</t>
+          <t>+150</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>B Fisher</t>
+          <t>T Imai</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1177,17 +1177,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+152</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>39.7%</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>39.7%</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1231,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+195</t>
+          <t>+202</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>33.9%</t>
+          <t>33.1%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1251,88 +1251,88 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>33.9%</t>
+          <t>33.1%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Nick Kurtz</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>+241</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>29.3%</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>29.3%</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Schwarber</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>+246</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>28.9%</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>28.9%</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Kyle Schwarber</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>+246</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>28.9%</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>28.9%</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>+255</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>28.2%</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>28.2%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>+255</t>
+          <t>+282</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>26.2%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1347,24 +1347,24 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>26.2%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Ketel Marte</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+282</t>
+          <t>+288</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1379,24 +1379,24 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+288</t>
+          <t>+291</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>25.6%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1411,24 +1411,24 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>25.6%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+291</t>
+          <t>+294</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.4%</t>
         </is>
       </c>
     </row>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+301</t>
+          <t>+303</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>24.9%</t>
+          <t>24.8%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>24.9%</t>
+          <t>24.8%</t>
         </is>
       </c>
     </row>
@@ -1704,66 +1704,66 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Christian Walker</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>+336</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>22.9%</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>22.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Joc Pederson</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>+339</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>22.8%</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>22.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Christian Walker</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>+340</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>22.7%</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>22.7%</t>
         </is>
       </c>
     </row>
@@ -2026,12 +2026,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Kerry Carpenter</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+373</t>
+          <t>+374</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2058,17 +2058,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+374</t>
+          <t>+383</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2083,19 +2083,19 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Miguel Vargas</t>
+          <t>Kerry Carpenter</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+383</t>
+          <t>+384</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2186,17 +2186,17 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Ben Rice</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>+393</t>
+          <t>+390</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2211,88 +2211,88 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>Ben Rice</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>+393</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>20.3%</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>20.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
           <t>Garrett Mitchell</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>+393</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>20.3%</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>20.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>Nelson Velazquez</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>+396</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>20.2%</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Bryce Harper</t>
+          <t>Nelson Velazquez</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+396</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2307,24 +2307,24 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Adrian Del Castillo</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>+402</t>
+          <t>+399</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2339,56 +2339,56 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Carter Jensen</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>+405</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>19.8%</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>19.8%</t>
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>20.0%</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Jose Ramirez</t>
+          <t>Adrian Del Castillo</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>+406</t>
+          <t>+402</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2403,19 +2403,19 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>+406</t>
+          <t>+405</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2442,17 +2442,17 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+407</t>
+          <t>+406</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
@@ -2538,12 +2538,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Pete Alonso</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>+408</t>
+          <t>+407</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -2570,17 +2570,17 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Vinnie Pasquantino</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>+415</t>
+          <t>+408</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -2595,110 +2595,110 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.7%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
+          <t>Vinnie Pasquantino</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>+415</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
           <t>Julio Rodriguez</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>+418</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>19.3%</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>19.3%</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>Willson Contreras</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>+428</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
         <is>
           <t>18.9%</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
         <is>
           <t>18.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Wilyer Abreu</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>+433</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>18.8%</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -2730,17 +2730,17 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>+438</t>
+          <t>+433</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2755,24 +2755,24 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>+442</t>
+          <t>+438</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2787,69 +2787,69 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>+443</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>18.4%</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>18.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>Paul Goldschmidt</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>+443</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>18.4%</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>18.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="inlineStr">
-        <is>
-          <t>Salvador Perez</t>
-        </is>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>+443</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>18.4%</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F75" s="3" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>18.4%</t>
         </is>
@@ -2858,17 +2858,17 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Andrew Benintendi</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+446</t>
+          <t>+449</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2883,24 +2883,24 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>+447</t>
+          <t>+449</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2915,24 +2915,24 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Andrew Benintendi</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+449</t>
+          <t>+452</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2947,24 +2947,24 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>+449</t>
+          <t>+452</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2979,24 +2979,24 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+449</t>
+          <t>+459</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3011,24 +3011,24 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Dillon Dingler</t>
+          <t>Will Smith (LAD)</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+449</t>
+          <t>+460</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3043,24 +3043,24 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+452</t>
+          <t>+464</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -3075,24 +3075,24 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>+452</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -3107,24 +3107,24 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+459</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3139,24 +3139,24 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Will Smith (LAD)</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+460</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -3171,24 +3171,24 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>+464</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -3203,24 +3203,24 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+468</t>
+          <t>+472</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3235,19 +3235,19 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+472</t>
+          <t>+473</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -3274,17 +3274,17 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+473</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -3299,24 +3299,24 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+484</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -3331,88 +3331,88 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>Zach Neto</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>+479</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>17.3%</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>17.3%</t>
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>+486</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>17.1%</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B92" s="3" t="inlineStr">
-        <is>
-          <t>+486</t>
-        </is>
-      </c>
-      <c r="C92" s="3" t="inlineStr">
-        <is>
-          <t>17.1%</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F92" s="3" t="inlineStr">
-        <is>
-          <t>17.1%</t>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Manzardo</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>+488</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>17.0%</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>17.0%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>+488</t>
+          <t>+491</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -3427,24 +3427,24 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+495</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -3459,14 +3459,14 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Trent Grisham</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -3818,7 +3818,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Trent Grisham</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3914,17 +3914,17 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+536</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -3939,19 +3939,19 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>+536</t>
+          <t>+537</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -3976,64 +3976,64 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>Vladimir Guerrero Jr.</t>
-        </is>
-      </c>
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>+537</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>15.7%</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>15.7%</t>
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>+544</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="3" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="inlineStr">
-        <is>
-          <t>+544</t>
-        </is>
-      </c>
-      <c r="C112" s="3" t="inlineStr">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Cortes</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>+545</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>15.5%</t>
         </is>
       </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr">
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
         <is>
           <t>15.5%</t>
         </is>
@@ -4200,83 +4200,83 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>Carlos Cortes</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="inlineStr">
-        <is>
-          <t>+562</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>+564</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
         <is>
           <t>15.1%</t>
         </is>
       </c>
-      <c r="D118" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="inlineStr">
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
         <is>
           <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Basallo</t>
-        </is>
-      </c>
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t>+564</t>
-        </is>
-      </c>
-      <c r="C119" s="3" t="inlineStr">
-        <is>
-          <t>15.1%</t>
-        </is>
-      </c>
-      <c r="D119" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E119" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F119" s="3" t="inlineStr">
-        <is>
-          <t>15.1%</t>
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Coby Mayo</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>+568</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -4291,19 +4291,19 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+571</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -4746,7 +4746,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -4778,7 +4778,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -4810,7 +4810,7 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -4842,7 +4842,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Heriberto Hernandez</t>
+          <t>Christopher Morel</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Randy Arozarena</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -4906,7 +4906,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Randy Arozarena</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -4938,7 +4938,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Yandy Diaz</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -4970,7 +4970,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -5000,64 +5000,64 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="3" t="inlineStr">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Heriberto Hernandez</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
         <is>
           <t>Jac Caglianone</t>
         </is>
       </c>
-      <c r="B143" s="3" t="inlineStr">
+      <c r="B144" s="3" t="inlineStr">
         <is>
           <t>+610</t>
         </is>
       </c>
-      <c r="C143" s="3" t="inlineStr">
+      <c r="C144" s="3" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
       </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E143" s="3" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F143" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="inlineStr">
-        <is>
-          <t>Christopher Morel</t>
-        </is>
-      </c>
-      <c r="B144" s="2" t="inlineStr">
-        <is>
-          <t>+610</t>
-        </is>
-      </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t>14.1%</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E144" s="2" t="inlineStr">
-        <is>
-          <t>nan%</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="inlineStr">
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>nan%</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
@@ -5098,7 +5098,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Austin Wells</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -5130,7 +5130,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Amed Rosario</t>
+          <t>Austin Wells</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -5194,17 +5194,17 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Michael Massey</t>
+          <t>Amed Rosario</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
@@ -5258,17 +5258,17 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Michael Massey</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
@@ -5386,17 +5386,17 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
@@ -5450,7 +5450,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Drew Romo</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -5482,7 +5482,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -5514,7 +5514,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Drew Romo</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -5546,17 +5546,17 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -5571,24 +5571,24 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
@@ -5674,17 +5674,17 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -5699,14 +5699,14 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -5738,7 +5738,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -5802,17 +5802,17 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
@@ -5898,7 +5898,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -5930,7 +5930,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -5994,7 +5994,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -6026,7 +6026,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Evan Carter</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -6058,7 +6058,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -6122,7 +6122,7 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Xander Bogaerts</t>
+          <t>Evan Carter</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -6154,17 +6154,17 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -6179,24 +6179,24 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -6211,14 +6211,14 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -6282,17 +6282,17 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -6307,14 +6307,14 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -6346,7 +6346,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Lars Nootbaar</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -6378,7 +6378,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -6474,7 +6474,7 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>Lars Nootbaar</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -6506,7 +6506,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>CJ Abrams</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -6538,7 +6538,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Rikuu Nishida</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -6570,7 +6570,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Rikuu Nishida</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -6634,7 +6634,7 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -6666,7 +6666,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Victor Mesa Jr.</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -6698,7 +6698,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Luis Rengifo</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -6730,7 +6730,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Victor Mesa Jr.</t>
+          <t>Luis Rengifo</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -6762,7 +6762,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -6794,7 +6794,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -7050,7 +7050,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Sterlin Thompson</t>
+          <t>Ryan Kreidler</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -7082,7 +7082,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Ryan Kreidler</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -7114,7 +7114,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Sterlin Thompson</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -7274,7 +7274,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Connor Norby</t>
+          <t>Ryan Vilade</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -7306,7 +7306,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vilade</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -7338,7 +7338,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Connor Norby</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -7402,7 +7402,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -7434,7 +7434,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -7626,7 +7626,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -7658,7 +7658,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -7690,7 +7690,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -7727,12 +7727,12 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -7747,24 +7747,24 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Gleyber Torres</t>
+          <t>Richie Palacios</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
@@ -7818,17 +7818,17 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Richie Palacios</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -7843,14 +7843,14 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Sandy Leon</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -7914,17 +7914,17 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Sandy Leon</t>
+          <t>David Hamilton</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -7939,14 +7939,14 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Gleyber Torres</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -8042,7 +8042,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Brandon Valenzuela</t>
+          <t>Hayden Senger</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Miguel Andujar</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Hayden Senger</t>
+          <t>Brandon Valenzuela</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -8138,7 +8138,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Miguel Andujar</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -8298,7 +8298,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -8330,17 +8330,17 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
@@ -8394,7 +8394,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Matt Vierling</t>
+          <t>Justin Crawford</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -8458,17 +8458,17 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>Justin Crawford</t>
+          <t>Wade Meckler</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -8483,14 +8483,14 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>Wade Meckler</t>
+          <t>Troy Johnston</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -8522,7 +8522,7 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Esteury Ruiz</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -8586,7 +8586,7 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>Esteury Ruiz</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -8618,17 +8618,17 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
@@ -8682,7 +8682,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>Wenceel Perez</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -8714,17 +8714,17 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Wenceel Perez</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -8739,7 +8739,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Matt Vierling</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -8874,7 +8874,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -8906,7 +8906,7 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B265" s="2" t="inlineStr">
@@ -9002,17 +9002,17 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>Christian Vazquez</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -9027,14 +9027,14 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Tyler Freeman</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
@@ -9066,17 +9066,17 @@
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>Tyler Freeman</t>
+          <t>Bryce Johnson</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -9091,14 +9091,14 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>Bryce Johnson</t>
+          <t>Christian Vazquez</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
@@ -9194,7 +9194,7 @@
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>Hunter Feduccia</t>
+          <t>Adam Frazier</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -9226,7 +9226,7 @@
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>Adam Frazier</t>
+          <t>Hunter Feduccia</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
@@ -9290,7 +9290,7 @@
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Austin Martin</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
@@ -9322,7 +9322,7 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>Austin Martin</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
@@ -9354,17 +9354,17 @@
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>Xavier Edwards</t>
+          <t>Darell Hernaiz</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -9379,14 +9379,14 @@
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Xavier Edwards</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
@@ -9418,17 +9418,17 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>Darell Hernaiz</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1240</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.5%</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -9443,7 +9443,7 @@
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.5%</t>
         </is>
       </c>
     </row>
@@ -9482,7 +9482,7 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>Nick Allen</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
@@ -9514,7 +9514,7 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
@@ -9546,7 +9546,7 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Nick Allen</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
@@ -9610,7 +9610,7 @@
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Jacob Young</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
@@ -9642,7 +9642,7 @@
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
@@ -9674,7 +9674,7 @@
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>Jacob Young</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update odds files - Mon Jun  8 15:37:45 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -523,12 +523,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+240</t>
+          <t>+244</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>29.1%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -539,52 +539,52 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>29.1%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Kyle Schwarber</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>+262</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>27.6%</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>27.6%</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Nick Kurtz</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>+261</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>27.7%</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>27.7%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Brent Rooker</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+278</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.5%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+277</t>
+          <t>+286</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>25.9%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -623,35 +623,35 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>25.9%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Nick Kurtz</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>+285</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>26.0%</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>26.0%</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Schwarber</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>+287</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>25.8%</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
@@ -663,12 +663,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+309</t>
+          <t>+320</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -679,24 +679,24 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>23.8%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Junior Caminero</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>+327</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -707,7 +707,7 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.4%</t>
         </is>
       </c>
     </row>
@@ -740,75 +740,75 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Andrew Vaughn</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>+335</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>23.0%</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>23.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Willson Contreras</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>+333</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>23.1%</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>23.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Junior Caminero</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>+348</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>22.3%</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>22.3%</t>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>+337</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>22.9%</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>22.9%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Trent Grisham</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+364</t>
+          <t>+367</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -819,52 +819,52 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Colby Thomas</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>+393</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>20.3%</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>20.3%</t>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>+380</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>20.8%</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>+393</t>
+          <t>+394</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -875,24 +875,24 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Yandy Diaz</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+406</t>
+          <t>+401</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Pete Alonso</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+412</t>
+          <t>+401</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,52 +931,52 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>William Contreras</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>+413</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>19.5%</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>19.5%</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Patrick Wisdom</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>+409</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>19.6%</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Trent Grisham</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+416</t>
+          <t>+410</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+416</t>
+          <t>+411</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1015,7 +1015,7 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
@@ -1050,17 +1050,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>+424</t>
+          <t>+421</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1071,42 +1071,42 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Jose Ramirez</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>+424</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>19.1%</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>19.1%</t>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>+428</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>18.9%</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Luke Raley</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1134,17 +1134,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+448</t>
+          <t>+440</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1155,52 +1155,52 @@
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Basallo</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>+457</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>18.0%</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>18.0%</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Julio Rodriguez</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>+441</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Julio Rodriguez</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>+457</t>
+          <t>+441</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1211,24 +1211,24 @@
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>+471</t>
+          <t>+458</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1239,24 +1239,24 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+472</t>
+          <t>+461</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1267,24 +1267,24 @@
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+462</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1295,24 +1295,24 @@
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1323,52 +1323,52 @@
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>+480</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>17.2%</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>17.2%</t>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Zack Gelof</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>+471</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>17.5%</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+472</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1379,24 +1379,24 @@
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Adolis Garcia</t>
+          <t>Coby Mayo</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+473</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1407,24 +1407,24 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Patrick Wisdom</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+485</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+485</t>
+          <t>+480</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.2%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+488</t>
+          <t>+492</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1491,24 +1491,24 @@
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>+494</t>
+          <t>+499</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1519,24 +1519,24 @@
       <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Eugenio Suarez</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+495</t>
+          <t>+506</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1547,24 +1547,24 @@
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+497</t>
+          <t>+510</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1575,24 +1575,24 @@
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Dominic Canzone</t>
+          <t>Eugenio Suarez</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+502</t>
+          <t>+517</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1603,24 +1603,24 @@
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Bryce Harper</t>
+          <t>Isaac Paredes</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>+508</t>
+          <t>+525</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1631,24 +1631,24 @@
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+514</t>
+          <t>+528</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1659,52 +1659,52 @@
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>+525</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>16.0%</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>16.0%</t>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Jonah Heim</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>+533</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+535</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1715,24 +1715,24 @@
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Adolis Garcia</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1743,24 +1743,24 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Jonah Heim</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+538</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,19 +1771,19 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+552</t>
+          <t>+555</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+553</t>
+          <t>+562</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1827,24 +1827,24 @@
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+564</t>
+          <t>+569</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1855,24 +1855,24 @@
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+564</t>
+          <t>+574</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1883,24 +1883,24 @@
       <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+573</t>
+          <t>+575</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1911,24 +1911,24 @@
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Ryan McMahon</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+573</t>
+          <t>+582</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1939,24 +1939,24 @@
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>+582</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1967,24 +1967,24 @@
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Ryan McMahon</t>
+          <t>Luis Rengifo</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>+586</t>
+          <t>+593</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1995,24 +1995,24 @@
       <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Luis Rengifo</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>+594</t>
+          <t>+599</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2023,24 +2023,24 @@
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>+594</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2051,19 +2051,19 @@
       <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>+598</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2086,17 +2086,17 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2107,52 +2107,52 @@
       <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Trea Turner</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>+600</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>14.3%</t>
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2163,14 +2163,14 @@
       <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Randy Arozarena</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2198,17 +2198,17 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Jase Bowen</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2219,24 +2219,24 @@
       <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Randy Arozarena</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2247,14 +2247,14 @@
       <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2282,17 +2282,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Blake Perkins</t>
+          <t>Angel Martinez</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2303,14 +2303,14 @@
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2338,7 +2338,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Angel Martinez</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2366,17 +2366,17 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>LaMonte Wade Jr.</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2387,14 +2387,14 @@
       <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2422,17 +2422,17 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Blake Perkins</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2443,24 +2443,24 @@
       <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2471,24 +2471,24 @@
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2499,24 +2499,24 @@
       <c r="E73" s="2" t="inlineStr"/>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -2527,24 +2527,24 @@
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2555,24 +2555,24 @@
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2583,24 +2583,24 @@
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>LaMonte Wade Jr.</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2611,24 +2611,24 @@
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Jase Bowen</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2639,24 +2639,24 @@
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2667,24 +2667,24 @@
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -2695,24 +2695,24 @@
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -2723,24 +2723,24 @@
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2751,24 +2751,24 @@
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Joey Ortiz</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -2779,24 +2779,24 @@
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -2807,24 +2807,24 @@
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Spencer Jones</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -2835,24 +2835,24 @@
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>CJ Abrams</t>
+          <t>Joey Ortiz</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -2863,24 +2863,24 @@
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Xander Bogaerts</t>
+          <t>Miguel Andujar</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -2891,7 +2891,7 @@
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
@@ -2903,12 +2903,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -2919,24 +2919,24 @@
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Miguel Andujar</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -2947,24 +2947,24 @@
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>J.C. Escarra</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -2975,7 +2975,7 @@
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
@@ -2987,12 +2987,12 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -3003,24 +3003,24 @@
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3031,14 +3031,14 @@
       <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>J.C. Escarra</t>
+          <t>Nathaniel Lowe</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -3066,17 +3066,17 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -3087,24 +3087,24 @@
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Carlos Narvaez</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -3115,24 +3115,24 @@
       <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Darell Hernaiz</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -3143,24 +3143,24 @@
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Nathaniel Lowe</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -3171,24 +3171,24 @@
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Patrick Bailey</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -3199,14 +3199,14 @@
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Andruw Monasterio</t>
+          <t>Carlos Narvaez</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -3234,7 +3234,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Andruw Monasterio</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3262,17 +3262,17 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Rodolfo Duran</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
       <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3318,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Rodolfo Duran</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -3346,17 +3346,17 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -3367,24 +3367,24 @@
       <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Wade Meckler</t>
+          <t>Patrick Bailey</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -3395,24 +3395,24 @@
       <c r="E105" s="2" t="inlineStr"/>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -3423,24 +3423,24 @@
       <c r="E106" s="2" t="inlineStr"/>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Daulton Varsho</t>
+          <t>Steward Berroa</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -3451,24 +3451,24 @@
       <c r="E107" s="2" t="inlineStr"/>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Masataka Yoshida</t>
+          <t>Curtis Mead</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -3479,24 +3479,24 @@
       <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Darell Hernaiz</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -3507,24 +3507,24 @@
       <c r="E109" s="2" t="inlineStr"/>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -3535,24 +3535,24 @@
       <c r="E110" s="2" t="inlineStr"/>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Daulton Varsho</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -3563,24 +3563,24 @@
       <c r="E111" s="2" t="inlineStr"/>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Jhonny Pereda</t>
+          <t>Wade Meckler</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -3591,24 +3591,24 @@
       <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Nick Fortes</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -3619,14 +3619,14 @@
       <c r="E113" s="2" t="inlineStr"/>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -3654,17 +3654,17 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Masataka Yoshida</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -3675,14 +3675,14 @@
       <c r="E115" s="2" t="inlineStr"/>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Nolan Schanuel</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -3710,7 +3710,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Jhonny Pereda</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -3738,12 +3738,12 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Nolan Schanuel</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Daniel Susac</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -3794,17 +3794,17 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Nick Fortes</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -3815,24 +3815,24 @@
       <c r="E120" s="2" t="inlineStr"/>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -3843,24 +3843,24 @@
       <c r="E121" s="2" t="inlineStr"/>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -3871,7 +3871,7 @@
       <c r="E122" s="2" t="inlineStr"/>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
@@ -3883,12 +3883,12 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -3899,14 +3899,14 @@
       <c r="E123" s="2" t="inlineStr"/>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Charles McAdoo</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -3934,17 +3934,17 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Steward Berroa</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -3955,7 +3955,7 @@
       <c r="E125" s="2" t="inlineStr"/>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
@@ -3967,12 +3967,12 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -3983,24 +3983,24 @@
       <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Ben Williamson</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -4011,24 +4011,24 @@
       <c r="E127" s="2" t="inlineStr"/>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Drew Gilbert</t>
+          <t>Charles McAdoo</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -4039,24 +4039,24 @@
       <c r="E128" s="2" t="inlineStr"/>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -4067,24 +4067,24 @@
       <c r="E129" s="2" t="inlineStr"/>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -4095,24 +4095,24 @@
       <c r="E130" s="2" t="inlineStr"/>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1240</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.5%</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -4123,14 +4123,14 @@
       <c r="E131" s="2" t="inlineStr"/>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.5%</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Ben Williamson</t>
+          <t>Drew Gilbert</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -4158,17 +4158,17 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1300</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -4179,24 +4179,24 @@
       <c r="E133" s="2" t="inlineStr"/>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.1%</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -4207,24 +4207,24 @@
       <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.0%</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1360</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="E135" s="2" t="inlineStr"/>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1360</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -4263,24 +4263,24 @@
       <c r="E136" s="2" t="inlineStr"/>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1380</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -4291,24 +4291,24 @@
       <c r="E137" s="2" t="inlineStr"/>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1440</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -4319,24 +4319,24 @@
       <c r="E138" s="2" t="inlineStr"/>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.5%</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Myles Straw</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>+1440</t>
+          <t>+1500</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -4347,24 +4347,24 @@
       <c r="E139" s="2" t="inlineStr"/>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>6.2%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Myles Straw</t>
+          <t>Tyler Heineman</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>+1460</t>
+          <t>+1560</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -4375,24 +4375,24 @@
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.0%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Jacob Young</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>+1600</t>
+          <t>+1640</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.7%</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -4403,24 +4403,24 @@
       <c r="E141" s="2" t="inlineStr"/>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.7%</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Tyler Heineman</t>
+          <t>Chandler Simpson</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>+1600</t>
+          <t>+1660</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.7%</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -4431,24 +4431,24 @@
       <c r="E142" s="2" t="inlineStr"/>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.7%</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Drew Millas</t>
+          <t>Jacob Young</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>+1640</t>
+          <t>+1720</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>5.5%</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -4459,24 +4459,24 @@
       <c r="E143" s="2" t="inlineStr"/>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>5.5%</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Chandler Simpson</t>
+          <t>Drew Millas</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>+1660</t>
+          <t>+1760</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>5.4%</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -4487,7 +4487,7 @@
       <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>5.4%</t>
         </is>
       </c>
     </row>
@@ -4499,12 +4499,12 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>+1900</t>
+          <t>+2100</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -4515,7 +4515,7 @@
       <c r="E145" s="2" t="inlineStr"/>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Mon Jun  8 19:43:26 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+230</t>
+          <t>+213</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>30.3%</t>
+          <t>31.9%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>30.3%</t>
+          <t>31.9%</t>
         </is>
       </c>
     </row>
@@ -523,12 +523,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+244</t>
+          <t>+235</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>29.1%</t>
+          <t>29.9%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -539,7 +539,7 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>29.1%</t>
+          <t>29.9%</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+261</t>
+          <t>+259</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -567,14 +567,14 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>27.9%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Brent Rooker</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -600,58 +600,58 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Brent Rooker</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>+286</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>25.9%</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>25.9%</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Schwarber</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>+281</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>26.2%</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>26.2%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Kyle Schwarber</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>+287</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>25.8%</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>25.8%</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>+289</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>25.7%</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>25.7%</t>
         </is>
       </c>
     </row>
@@ -663,12 +663,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+320</t>
+          <t>+302</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>24.9%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -679,24 +679,24 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>24.9%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Junior Caminero</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+327</t>
+          <t>+318</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.9%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -707,24 +707,24 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Andrew Vaughn</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>+331</t>
+          <t>+323</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -735,24 +735,24 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>23.6%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Junior Caminero</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>+335</t>
+          <t>+326</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.5%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -763,7 +763,7 @@
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
@@ -775,12 +775,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>+337</t>
+          <t>+332</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>22.9%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -791,24 +791,24 @@
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>22.9%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+367</t>
+          <t>+335</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -819,80 +819,80 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>23.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Christian Walker</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>+356</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>21.9%</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>21.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Colby Thomas</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>+368</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
           <t>21.4%</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Colby Thomas</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>+380</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>20.8%</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>20.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Pete Alonso</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>+394</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>20.2%</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>20.2%</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+401</t>
+          <t>+380</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+401</t>
+          <t>+381</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,52 +931,52 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Patrick Wisdom</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>+409</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>19.6%</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>19.6%</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Casey Schmitt</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>+382</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>20.7%</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Trent Grisham</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+410</t>
+          <t>+395</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+411</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1015,7 +1015,7 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+405</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1043,80 +1043,80 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Rafael Devers</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>+421</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>19.2%</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>19.2%</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Patrick Wisdom</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>+406</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Basallo</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>+428</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>18.9%</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>18.9%</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Yandy Diaz</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>+410</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>19.6%</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Trent Grisham</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1127,24 +1127,24 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Luke Raley</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+438</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1155,24 +1155,24 @@
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Julio Rodriguez</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>+441</t>
+          <t>+439</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1183,7 +1183,7 @@
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
@@ -1218,17 +1218,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>+458</t>
+          <t>+453</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1239,24 +1239,24 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>+455</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1267,24 +1267,24 @@
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+462</t>
+          <t>+457</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1295,24 +1295,24 @@
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Julio Rodriguez</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+468</t>
+          <t>+458</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1323,19 +1323,19 @@
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+471</t>
+          <t>+472</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1358,12 +1358,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+472</t>
+          <t>+473</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1391,12 +1391,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+473</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1407,24 +1407,24 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Dominic Canzone</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+479</t>
+          <t>+484</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+486</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+492</t>
+          <t>+497</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
@@ -1526,17 +1526,17 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+506</t>
+          <t>+500</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1547,33 +1547,33 @@
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Garrett Mitchell</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>+510</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>+509</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>16.4%</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>16.4%</t>
         </is>
@@ -1587,12 +1587,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+517</t>
+          <t>+512</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1603,52 +1603,52 @@
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>+525</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>16.0%</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>16.0%</t>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Josh Naylor</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>+513</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1659,24 +1659,24 @@
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Jonah Heim</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>Jonah Heim</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+535</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1715,52 +1715,52 @@
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Adolis Garcia</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>+540</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>15.6%</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>15.6%</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>+544</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+546</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,24 +1771,24 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+555</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+562</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1827,24 +1827,24 @@
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+569</t>
+          <t>+574</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1855,19 +1855,19 @@
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Adolis Garcia</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+574</t>
+          <t>+576</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -1890,17 +1890,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+578</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1911,24 +1911,24 @@
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Ryan McMahon</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+582</t>
+          <t>+584</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1939,24 +1939,24 @@
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Ryan McMahon</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>+592</t>
+          <t>+584</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1967,24 +1967,24 @@
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Luis Rengifo</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>+593</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1995,24 +1995,24 @@
       <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Chase DeLauter</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+593</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2023,24 +2023,24 @@
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Luis Rengifo</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+594</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2051,19 +2051,19 @@
       <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Chase DeLauter</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+599</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2086,17 +2086,17 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2107,33 +2107,33 @@
       <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr">
         <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Jeremy Pena</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
           <t>14.1%</t>
         </is>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>+610</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr"/>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>14.1%</t>
         </is>
@@ -2142,7 +2142,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Spencer Jones</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2170,17 +2170,17 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Jase Bowen</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2191,24 +2191,24 @@
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Jase Bowen</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2219,14 +2219,14 @@
       <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Randy Arozarena</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2254,17 +2254,17 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2275,7 +2275,7 @@
       <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
@@ -2310,17 +2310,17 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -2331,24 +2331,24 @@
       <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
@@ -2394,17 +2394,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Blake Perkins</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2415,24 +2415,24 @@
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Blake Perkins</t>
+          <t>Edmundo Sosa</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2443,24 +2443,24 @@
       <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2471,24 +2471,24 @@
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2499,24 +2499,24 @@
       <c r="E73" s="2" t="inlineStr"/>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -2527,7 +2527,7 @@
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
@@ -2539,12 +2539,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2555,24 +2555,24 @@
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Austin Slater</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2583,24 +2583,24 @@
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>LaMonte Wade Jr.</t>
+          <t>Randy Arozarena</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2611,24 +2611,24 @@
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Joey Ortiz</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2639,24 +2639,24 @@
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>LaMonte Wade Jr.</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2667,24 +2667,24 @@
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -2695,24 +2695,24 @@
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Sam Huff</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -2723,24 +2723,24 @@
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2751,24 +2751,24 @@
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -2779,14 +2779,14 @@
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2814,17 +2814,17 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -2835,24 +2835,24 @@
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Joey Ortiz</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -2863,24 +2863,24 @@
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Miguel Andujar</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -2891,24 +2891,24 @@
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -2919,24 +2919,24 @@
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>CJ Abrams</t>
+          <t>Ryan Vilade</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -2947,24 +2947,24 @@
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>J.C. Escarra</t>
+          <t>Miguel Andujar</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -2975,24 +2975,24 @@
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Ryan Vilade</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -3003,24 +3003,24 @@
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Xander Bogaerts</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3031,24 +3031,24 @@
       <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Nathaniel Lowe</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -3059,24 +3059,24 @@
       <c r="E93" s="2" t="inlineStr"/>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -3087,24 +3087,24 @@
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Nathaniel Lowe</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -3115,24 +3115,24 @@
       <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Darell Hernaiz</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -3143,24 +3143,24 @@
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -3171,24 +3171,24 @@
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -3199,24 +3199,24 @@
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Carlos Narvaez</t>
+          <t>Darell Hernaiz</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -3227,14 +3227,14 @@
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Andruw Monasterio</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3262,17 +3262,17 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -3283,14 +3283,14 @@
       <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Carlos Narvaez</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3346,17 +3346,17 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Daniel Susac</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -3367,24 +3367,24 @@
       <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Patrick Bailey</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -3395,24 +3395,24 @@
       <c r="E105" s="2" t="inlineStr"/>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Wade Meckler</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -3423,24 +3423,24 @@
       <c r="E106" s="2" t="inlineStr"/>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Steward Berroa</t>
+          <t>Patrick Bailey</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -3451,24 +3451,24 @@
       <c r="E107" s="2" t="inlineStr"/>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -3479,24 +3479,24 @@
       <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Blaze Alexander</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -3507,24 +3507,24 @@
       <c r="E109" s="2" t="inlineStr"/>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Nolan Schanuel</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -3535,24 +3535,24 @@
       <c r="E110" s="2" t="inlineStr"/>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Daulton Varsho</t>
+          <t>J.C. Escarra</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -3563,24 +3563,24 @@
       <c r="E111" s="2" t="inlineStr"/>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Wade Meckler</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -3591,24 +3591,24 @@
       <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Nick Fortes</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -3619,24 +3619,24 @@
       <c r="E113" s="2" t="inlineStr"/>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -3647,24 +3647,24 @@
       <c r="E114" s="2" t="inlineStr"/>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Masataka Yoshida</t>
+          <t>Jhonny Pereda</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -3675,24 +3675,24 @@
       <c r="E115" s="2" t="inlineStr"/>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Nolan Schanuel</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -3703,24 +3703,24 @@
       <c r="E116" s="2" t="inlineStr"/>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Jhonny Pereda</t>
+          <t>Curtis Mead</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -3731,24 +3731,24 @@
       <c r="E117" s="2" t="inlineStr"/>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -3759,24 +3759,24 @@
       <c r="E118" s="2" t="inlineStr"/>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Nick Fortes</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -3787,14 +3787,14 @@
       <c r="E119" s="2" t="inlineStr"/>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Christian Vazquez</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -3822,17 +3822,17 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -3843,14 +3843,14 @@
       <c r="E121" s="2" t="inlineStr"/>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -3878,17 +3878,17 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Blake Dunn</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -3899,14 +3899,14 @@
       <c r="E123" s="2" t="inlineStr"/>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Blake Dunn</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -3934,7 +3934,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -3962,17 +3962,17 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Christian Vazquez</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -3983,24 +3983,24 @@
       <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Ben Williamson</t>
+          <t>Drew Gilbert</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -4011,24 +4011,24 @@
       <c r="E127" s="2" t="inlineStr"/>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Charles McAdoo</t>
+          <t>Ben Williamson</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -4039,24 +4039,24 @@
       <c r="E128" s="2" t="inlineStr"/>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Isiah Kiner-Falefa</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -4067,24 +4067,24 @@
       <c r="E129" s="2" t="inlineStr"/>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -4095,24 +4095,24 @@
       <c r="E130" s="2" t="inlineStr"/>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -4123,24 +4123,24 @@
       <c r="E131" s="2" t="inlineStr"/>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Drew Gilbert</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -4151,24 +4151,24 @@
       <c r="E132" s="2" t="inlineStr"/>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1280</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -4179,14 +4179,14 @@
       <c r="E133" s="2" t="inlineStr"/>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -4214,17 +4214,17 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>+1360</t>
+          <t>+1400</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.7%</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="E135" s="2" t="inlineStr"/>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.7%</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Tyler Heineman</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>+1360</t>
+          <t>+1420</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -4263,7 +4263,7 @@
       <c r="E136" s="2" t="inlineStr"/>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
@@ -4275,12 +4275,12 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1420</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -4291,7 +4291,7 @@
       <c r="E137" s="2" t="inlineStr"/>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
@@ -4331,12 +4331,12 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>+1500</t>
+          <t>+1440</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -4347,24 +4347,24 @@
       <c r="E139" s="2" t="inlineStr"/>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.5%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Tyler Heineman</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>+1560</t>
+          <t>+1460</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -4375,7 +4375,7 @@
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.4%</t>
         </is>
       </c>
     </row>
@@ -4387,12 +4387,12 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>+1640</t>
+          <t>+1620</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -4403,19 +4403,19 @@
       <c r="E141" s="2" t="inlineStr"/>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>5.8%</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Chandler Simpson</t>
+          <t>Drew Millas</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>+1660</t>
+          <t>+1640</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -4438,17 +4438,17 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Jacob Young</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>+1720</t>
+          <t>+1700</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -4459,24 +4459,24 @@
       <c r="E143" s="2" t="inlineStr"/>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>5.6%</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Drew Millas</t>
+          <t>Jacob Young</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>+1760</t>
+          <t>+1720</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>5.5%</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -4487,7 +4487,7 @@
       <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>5.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Wed Jun 10 02:20:21 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,10 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -58,9 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -428,10 +435,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -471,6 +478,510 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>+322</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>23.7%</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>23.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Max Muncy (LAD)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>+455</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Freddie Freeman</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>+518</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Tucker</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>+537</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>15.7%</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>15.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Oneil Cruz</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>+551</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Brandon Lowe</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>+566</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Andy Pages</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>+587</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Will Smith (LAD)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Ward</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Ryan O'Hearn</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Endy Rodriguez</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Alex Freeland</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Bryan Reynolds</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Nick Gonzales</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Horwitz</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>6.7%</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>6.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Jared Triolo</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>+1760</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Jake Mangum</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update odds files - Wed Jun 10 03:30:15 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,12 +68,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -435,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -509,17 +518,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Max Muncy (LAD)</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+455</t>
+          <t>+427</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -530,24 +539,24 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Eugenio Suarez</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+518</t>
+          <t>+443</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -558,24 +567,24 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+537</t>
+          <t>+450</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -586,24 +595,24 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Oneil Cruz</t>
+          <t>Max Muncy (LAD)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+455</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -614,52 +623,52 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Brandon Lowe</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>+566</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>15.0%</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>15.0%</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>+458</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>17.9%</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -670,24 +679,24 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Will Smith (LAD)</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+518</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -698,24 +707,24 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+537</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -726,24 +735,24 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Nathaniel Lowe</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+542</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -754,24 +763,24 @@
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Oneil Cruz</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+551</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -782,24 +791,24 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Brandon Lowe</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+566</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -810,24 +819,24 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+577</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -838,24 +847,24 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+587</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -866,24 +875,24 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -894,24 +903,24 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Tyler O'Neill</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -922,24 +931,24 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+1760</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -950,24 +959,24 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Jake Mangum</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+2000</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -977,6 +986,510 @@
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Will Smith (LAD)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Matt McLain</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Adley Rutschman</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Blake Dunn</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Ward</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Ward</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Ryan O'Hearn</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Jackson Holliday</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Edwin Arroyo</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Endy Rodriguez</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Alex Freeland</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Blaze Alexander</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Bryan Reynolds</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Nick Gonzales</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Horwitz</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>6.7%</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>6.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Jared Triolo</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>+1760</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Jake Mangum</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>4.8%</t>
         </is>

</xml_diff>

<commit_message>
Update odds files - Thu Jun 11 00:18:20 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+138</t>
+          <t>+133</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>42.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>42.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
     </row>
@@ -523,12 +523,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+191</t>
+          <t>+183</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>34.4%</t>
+          <t>35.3%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -539,7 +539,7 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>34.4%</t>
+          <t>35.3%</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+247</t>
+          <t>+246</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>28.9%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>28.9%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+248</t>
+          <t>+247</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>28.8%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>28.8%</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+262</t>
+          <t>+261</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>27.7%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -707,7 +707,7 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>27.7%</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>+269</t>
+          <t>+268</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>27.2%</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -735,7 +735,7 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>27.2%</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+322</t>
+          <t>+314</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>23.7%</t>
+          <t>24.2%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>23.7%</t>
+          <t>24.2%</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1055,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>+355</t>
+          <t>+350</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun 11 00:24:31 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+133</t>
+          <t>+134</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>42.7%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>42.7%</t>
         </is>
       </c>
     </row>
@@ -523,12 +523,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+183</t>
+          <t>+174</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>36.5%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -539,7 +539,7 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>36.5%</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+246</t>
+          <t>+247</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>28.9%</t>
+          <t>28.8%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>28.9%</t>
+          <t>28.8%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+247</t>
+          <t>+248</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>28.7%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -623,24 +623,24 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>28.7%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Gary Sanchez</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+255</t>
+          <t>+252</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>28.4%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -651,24 +651,24 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>28.4%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Gary Sanchez</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+260</t>
+          <t>+255</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>27.8%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -679,7 +679,7 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>27.8%</t>
+          <t>28.2%</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+261</t>
+          <t>+256</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>28.1%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -707,7 +707,7 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>28.1%</t>
         </is>
       </c>
     </row>
@@ -770,17 +770,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>+287</t>
+          <t>+285</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -791,14 +791,14 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.0%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -826,17 +826,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Andrew Vaughn</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>+289</t>
+          <t>+288</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -847,7 +847,7 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+309</t>
+          <t>+312</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+314</t>
+          <t>+323</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>23.6%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+323</t>
+          <t>+326</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.5%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -959,24 +959,24 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Michael Conforto</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+326</t>
+          <t>+330</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.3%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Michael Conforto</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>+343</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1015,24 +1015,24 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>22.6%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>+343</t>
+          <t>+353</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.1%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1043,24 +1043,24 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+362</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1071,24 +1071,24 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>21.6%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>+362</t>
+          <t>+403</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1099,24 +1099,24 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>+403</t>
+          <t>+405</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1127,7 +1127,7 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
@@ -1246,12 +1246,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Alika Williams</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+475</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1274,17 +1274,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+477</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1295,19 +1295,19 @@
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Alika Williams</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+478</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1610,7 +1610,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Shay Whitcomb</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1666,17 +1666,17 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Shay Whitcomb</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1687,7 +1687,7 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1727,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1743,24 +1743,24 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Sal Frelick</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,14 +1771,14 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1806,17 +1806,17 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Sal Frelick</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1827,7 +1827,7 @@
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun 11 00:36:38 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+134</t>
+          <t>+130</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>42.7%</t>
+          <t>43.5%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>42.7%</t>
+          <t>43.5%</t>
         </is>
       </c>
     </row>
@@ -523,12 +523,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+174</t>
+          <t>+170</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>36.5%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -539,7 +539,7 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>36.5%</t>
+          <t>37.0%</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+247</t>
+          <t>+240</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>29.4%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+248</t>
+          <t>+247</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>28.8%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>28.8%</t>
         </is>
       </c>
     </row>
@@ -635,12 +635,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+252</t>
+          <t>+253</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>28.4%</t>
+          <t>28.3%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -651,7 +651,7 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>28.4%</t>
+          <t>28.3%</t>
         </is>
       </c>
     </row>
@@ -775,12 +775,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>+285</t>
+          <t>+279</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -791,24 +791,24 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>26.4%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Andrew Vaughn</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+287</t>
+          <t>+280</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.3%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -819,19 +819,19 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.3%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>+288</t>
+          <t>+287</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>+290</t>
+          <t>+288</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -875,24 +875,24 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+312</t>
+          <t>+323</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>23.6%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+323</t>
+          <t>+326</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.5%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Michael Conforto</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+326</t>
+          <t>+330</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -959,24 +959,24 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.3%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Michael Conforto</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>+334</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.0%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+343</t>
+          <t>+347</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1015,24 +1015,24 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>+353</t>
+          <t>+361</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.7%</t>
         </is>
       </c>
     </row>
@@ -1078,17 +1078,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>+403</t>
+          <t>+363</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1099,24 +1099,24 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>21.6%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>+405</t>
+          <t>+386</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.6%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1127,7 +1127,7 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.6%</t>
         </is>
       </c>
     </row>
@@ -1162,12 +1162,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>+431</t>
+          <t>+432</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1190,17 +1190,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Alika Williams</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>+432</t>
+          <t>+442</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
@@ -1223,12 +1223,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+460</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1239,24 +1239,24 @@
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+463</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1267,24 +1267,24 @@
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+475</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1295,19 +1295,19 @@
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Alika Williams</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+478</t>
+          <t>+477</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1470,17 +1470,17 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Brice Matthews</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+562</t>
+          <t>+560</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1491,24 +1491,24 @@
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Brice Matthews</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+562</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1519,19 +1519,19 @@
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Cole Carrigg</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>+580</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1554,17 +1554,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Trey Mancini</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+588</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1575,24 +1575,24 @@
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+598</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1603,24 +1603,24 @@
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Trey Mancini</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1631,7 +1631,7 @@
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
@@ -1699,12 +1699,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1727,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1743,24 +1743,24 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Sal Frelick</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,24 +1771,24 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Sal Frelick</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Troy Johnston</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1827,24 +1827,24 @@
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1855,7 +1855,7 @@
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
@@ -1923,12 +1923,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1939,7 +1939,7 @@
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun 11 12:18:01 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -490,17 +490,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nick Kurtz</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+130</t>
+          <t>+245</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>29.0%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,24 +511,24 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>29.0%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+170</t>
+          <t>+257</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>37.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -539,24 +539,24 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>37.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+238</t>
+          <t>+296</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>29.6%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -567,24 +567,24 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>29.6%</t>
+          <t>25.3%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Hunter Goodman</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+240</t>
+          <t>+311</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+247</t>
+          <t>+323</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -623,24 +623,24 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>23.6%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+253</t>
+          <t>+326</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>28.3%</t>
+          <t>23.5%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -651,24 +651,24 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>28.3%</t>
+          <t>23.5%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Gary Sanchez</t>
+          <t>Kerry Carpenter</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+255</t>
+          <t>+330</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -679,80 +679,80 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>23.3%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Jackson Chourio</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>+256</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>28.1%</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>28.1%</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>+331</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>23.2%</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>23.2%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Jake Bauers</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>+268</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>27.2%</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>27.2%</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Matt Olson</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>+333</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>23.1%</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Yordan Alvarez</t>
+          <t>Max Muncy (LAD)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>+272</t>
+          <t>+341</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>22.7%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -763,24 +763,24 @@
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>22.7%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>+279</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -791,24 +791,24 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>21.7%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+280</t>
+          <t>+366</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>26.3%</t>
+          <t>21.5%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -819,24 +819,24 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>26.3%</t>
+          <t>21.5%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>+287</t>
+          <t>+374</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -847,24 +847,24 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>21.1%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>+288</t>
+          <t>+383</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -875,24 +875,24 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+323</t>
+          <t>+389</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+326</t>
+          <t>+392</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>20.3%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Michael Conforto</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>+395</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -959,24 +959,24 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+334</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+347</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1015,24 +1015,24 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>+361</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1043,24 +1043,24 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>+362</t>
+          <t>+405</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1071,24 +1071,24 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Brandon Lowe</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>+363</t>
+          <t>+409</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1099,24 +1099,24 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>+386</t>
+          <t>+409</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1127,24 +1127,24 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+406</t>
+          <t>+415</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.4%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1155,24 +1155,24 @@
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.4%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>+432</t>
+          <t>+417</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1183,80 +1183,80 @@
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Alika Williams</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>+442</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>18.5%</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>18.5%</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>+418</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>19.3%</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>+460</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>17.9%</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>17.9%</t>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Randal Grichuk</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>+419</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>19.3%</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+463</t>
+          <t>+429</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1267,52 +1267,52 @@
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Dansby Swanson</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>+475</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>17.4%</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>17.4%</t>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>+430</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>18.9%</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Austin Riley</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+433</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1323,24 +1323,24 @@
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1351,24 +1351,24 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+488</t>
+          <t>+442</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1379,24 +1379,24 @@
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Julio Rodriguez</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+444</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1407,24 +1407,24 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Braxton Fulford</t>
+          <t>Patrick Wisdom</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+504</t>
+          <t>+446</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+447</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Tyler O'Neill</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+560</t>
+          <t>+448</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1491,24 +1491,24 @@
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Brice Matthews</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+562</t>
+          <t>+449</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1519,24 +1519,24 @@
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+450</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1547,24 +1547,24 @@
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+588</t>
+          <t>+452</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1575,24 +1575,24 @@
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+598</t>
+          <t>+454</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1603,24 +1603,24 @@
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Trey Mancini</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1631,24 +1631,24 @@
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+471</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1659,24 +1659,24 @@
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Shay Whitcomb</t>
+          <t>Vinnie Pasquantino</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+473</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Lars Nootbaar</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+491</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1715,24 +1715,24 @@
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Joey Ortiz</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+492</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1743,24 +1743,24 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,24 +1771,24 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Sal Frelick</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+515</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1827,24 +1827,24 @@
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+519</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1855,24 +1855,24 @@
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Chad Stevens</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+521</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1883,24 +1883,24 @@
       <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Christian Vazquez</t>
+          <t>Coby Mayo</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1911,24 +1911,24 @@
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Wade Meckler</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+528</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1939,24 +1939,24 @@
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>Randy Arozarena</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+532</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1967,24 +1967,24 @@
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+542</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1995,7 +1995,2527 @@
       <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Jackson Holliday</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>+549</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>JJ Wetherholt</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>+549</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Tucker</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>+549</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Tristan Gray</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>+552</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Nolan Gorman</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>+555</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>15.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Trevor Larnach</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>+561</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Ward</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>+562</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Ozzie Albies</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Marcell Ozuna</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>+574</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Andrew Benintendi</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>+576</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Herrera</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>+577</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Moises Ballesteros</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>+581</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>+582</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr"/>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Josh Bell</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>+588</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>14.5%</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>14.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Willi Castro</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Victor Caratini</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Ward</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>MJ Melendez</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Michael Massey</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Josh Jung</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>+610</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>14.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Ezequiel Tovar</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Mike Yastrzemski</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Colt Emerson</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>13.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Elias Diaz</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Cole Young</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Carson Kelly</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Brooks Lee</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Jake McCarthy</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Matt Vierling</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Bryan Reynolds</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Evan Carter</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Cole Carrigg</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Jimmy Crooks</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Ryan O'Hearn</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>T.J. Rumfield</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Leody Taveras</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Owen Caissie</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Ezequiel Duran</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Carson Benge</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Kameron Misner</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Joe Mack</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Edouard Julien</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>+780</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Dominic Smith</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>+780</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Troy Johnston</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Nathan Church</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Jorge Mateo</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Connor Norby</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Zach McKinstry</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Karros</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Liam Hicks</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Derek Hill</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Colt Keith</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>+830</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Nolan Arenado</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Isaac Collins</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>10.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Alex Freeland</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Jacob Gonzalez</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>+870</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Mauricio Dubon</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>+870</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Billy Cook</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Brett Baty</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr"/>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Nico Hoerner</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Gleyber Torres</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr"/>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>AJ Ewing</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Masyn Winn</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Jakob Marsee</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Bo Bichette</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr"/>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Edgar Quero</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr"/>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Maikel Garcia</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr"/>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Otto Lopez</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr"/>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Nick Gonzales</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr"/>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Jhonny Pereda</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr"/>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Sandy Leon</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr"/>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Sam Huff</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr"/>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Pavin Smith</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr"/>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Jared Triolo</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr"/>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Ildemaro Vargas</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr"/>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Chase Meidroth</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel Moreno</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr"/>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Javier Sanoja</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Luke Keaschall</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr"/>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>8.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Geraldo Perdomo</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>8.2%</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr"/>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>8.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Tommy Troy</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr"/>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Xavier Edwards</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr"/>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Ryan Waldschmidt</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>+1180</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>7.8%</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr"/>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>7.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Flores</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
           <t>7.7%</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr"/>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>7.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Austin Martin</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>+1240</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>7.5%</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr"/>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>7.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Luisangel Acuna</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>+1240</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>7.5%</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>7.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Jake Mangum</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>+1340</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>6.9%</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>6.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Nicky Lopez</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>+1360</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>6.8%</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>6.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Sam Antonacci</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>+1360</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>6.8%</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr"/>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>6.8%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Sat Jun 13 12:55:01 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -600,75 +600,75 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Shohei Ohtani</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>+263</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Schwarber</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>+264</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>27.5%</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>27.5%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Kyle Schwarber</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>+264</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>27.5%</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>27.5%</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Colby Thomas</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>+268</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>27.2%</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>27.2%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Colby Thomas</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+268</t>
+          <t>+272</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>26.9%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -679,7 +679,7 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>26.9%</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+332</t>
+          <t>+335</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>23.0%</t>
         </is>
       </c>
     </row>
@@ -971,12 +971,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+358</t>
+          <t>+341</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>22.7%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>22.7%</t>
         </is>
       </c>
     </row>
@@ -1048,56 +1048,56 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Max Muncy (LAD)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>+362</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>21.6%</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>21.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Bobby Witt Jr.</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>+362</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>21.6%</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>21.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Max Muncy (LAD)</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>+362</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>21.6%</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>21.6%</t>
         </is>
@@ -1636,56 +1636,56 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Nathaniel Lowe</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>+415</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>+415</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>19.4%</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>19.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Nathaniel Lowe</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>+415</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>19.4%</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr"/>
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>19.4%</t>
         </is>
@@ -1722,17 +1722,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>+429</t>
+          <t>+422</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1743,24 +1743,24 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>Coby Mayo</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+429</t>
+          <t>+425</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,24 +1771,24 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Miguel Vargas</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+431</t>
+          <t>+429</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Vinnie Pasquantino</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+431</t>
+          <t>+429</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1827,24 +1827,24 @@
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Dalton Rushing</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+437</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1855,24 +1855,24 @@
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Vinnie Pasquantino</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+438</t>
+          <t>+431</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1883,24 +1883,24 @@
       <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Coby Mayo</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+439</t>
+          <t>+431</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1911,24 +1911,24 @@
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+436</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1939,24 +1939,24 @@
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.7%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Braxton Fulford</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1967,14 +1967,14 @@
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Braxton Fulford</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2000,93 +2000,93 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>T.J. Rumfield</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>+440</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Willson Contreras</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>+441</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>18.5%</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr"/>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>18.5%</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Zach Neto</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>+442</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>18.5%</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr"/>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>18.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>+444</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>18.4%</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr"/>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2112,28 +2112,28 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Riley Greene</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>+444</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>18.4%</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>18.4%</t>
         </is>
@@ -2142,17 +2142,17 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>+445</t>
+          <t>+444</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2163,19 +2163,19 @@
       <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>+447</t>
+          <t>+445</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2198,17 +2198,17 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+448</t>
+          <t>+447</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2219,7 +2219,7 @@
       <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
@@ -2254,17 +2254,17 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>+451</t>
+          <t>+448</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2275,24 +2275,24 @@
       <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Jose Ramirez</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>+452</t>
+          <t>+455</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2303,19 +2303,19 @@
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>+455</t>
+          <t>+456</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2336,56 +2336,56 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Wilyer Abreu</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>+456</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>Jake Bauers</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>+456</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C69" s="3" t="inlineStr">
         <is>
           <t>18.0%</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr"/>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>18.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>Kazuma Okamoto</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>+456</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>18.0%</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr"/>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>18.0%</t>
         </is>
@@ -2450,7 +2450,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2478,7 +2478,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Ryan Ward</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2618,7 +2618,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2758,7 +2758,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Dillon Dingler</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3150,7 +3150,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -3178,17 +3178,17 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+509</t>
+          <t>+513</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -3199,24 +3199,24 @@
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>+513</t>
+          <t>+517</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -3227,14 +3227,14 @@
       <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3346,12 +3346,12 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+527</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -3374,12 +3374,12 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>+530</t>
+          <t>+528</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -3402,17 +3402,17 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Angel Martinez</t>
+          <t>Curtis Mead</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+530</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -3423,19 +3423,19 @@
       <c r="E106" s="2" t="inlineStr"/>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Michael Massey</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+532</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Michael Massey</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -3486,12 +3486,12 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -3514,12 +3514,12 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Pavin Smith</t>
+          <t>Angel Martinez</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -3542,17 +3542,17 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Pavin Smith</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>+536</t>
+          <t>+534</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -3563,24 +3563,24 @@
       <c r="E111" s="2" t="inlineStr"/>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>+539</t>
+          <t>+536</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -3591,19 +3591,19 @@
       <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+539</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -3626,17 +3626,17 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>+545</t>
+          <t>+543</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -3647,14 +3647,14 @@
       <c r="E114" s="2" t="inlineStr"/>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Jacob Wilson</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -3682,17 +3682,17 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Jacob Wilson</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+545</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -3703,7 +3703,7 @@
       <c r="E116" s="2" t="inlineStr"/>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
@@ -3850,12 +3850,12 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Jahmai Jones</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+559</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -3878,12 +3878,12 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Kyle Higashioka</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>+559</t>
+          <t>+560</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -3906,17 +3906,17 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Kyle Higashioka</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>+560</t>
+          <t>+563</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -3927,24 +3927,24 @@
       <c r="E124" s="2" t="inlineStr"/>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>+563</t>
+          <t>+567</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -3955,24 +3955,24 @@
       <c r="E125" s="2" t="inlineStr"/>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Ryan McMahon</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>+567</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -3983,7 +3983,7 @@
       <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
@@ -4018,12 +4018,12 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Ryan McMahon</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+573</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -4046,17 +4046,17 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Jahmai Jones</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>+573</t>
+          <t>+576</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -4067,7 +4067,7 @@
       <c r="E129" s="2" t="inlineStr"/>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>+580</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -4191,12 +4191,12 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+593</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -4207,7 +4207,7 @@
       <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -4326,7 +4326,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Brice Matthews</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -4354,7 +4354,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Brice Matthews</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -4382,7 +4382,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -4578,7 +4578,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Justin Foscue</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -4606,7 +4606,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -4634,7 +4634,7 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -4662,7 +4662,7 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -4690,17 +4690,17 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Justin Foscue</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -4711,14 +4711,14 @@
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Keibert Ruiz</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -4746,17 +4746,17 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Keibert Ruiz</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -4767,14 +4767,14 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -4830,7 +4830,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -4858,7 +4858,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Owen Caissie</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -4886,7 +4886,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Owen Caissie</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -4914,7 +4914,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Ryan Waldschmidt</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -4942,7 +4942,7 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -4970,17 +4970,17 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -4991,14 +4991,14 @@
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Ryan Waldschmidt</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -5054,7 +5054,7 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Wenceel Perez</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -5082,17 +5082,17 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -5103,24 +5103,24 @@
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>David Fry</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -5131,24 +5131,24 @@
       <c r="E167" s="2" t="inlineStr"/>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Tyler Callihan</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -5159,24 +5159,24 @@
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -5187,24 +5187,24 @@
       <c r="E169" s="2" t="inlineStr"/>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Tyler Callihan</t>
+          <t>David Fry</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -5215,24 +5215,24 @@
       <c r="E170" s="2" t="inlineStr"/>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Alex Jackson</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -5243,24 +5243,24 @@
       <c r="E171" s="2" t="inlineStr"/>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Alex Jackson</t>
+          <t>Wenceel Perez</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -5271,7 +5271,7 @@
       <c r="E172" s="2" t="inlineStr"/>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
@@ -5334,17 +5334,17 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Matt Vierling</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -5355,14 +5355,14 @@
       <c r="E175" s="2" t="inlineStr"/>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Jorge Mateo</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -5390,17 +5390,17 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>Jorge Mateo</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -5411,7 +5411,7 @@
       <c r="E177" s="2" t="inlineStr"/>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
@@ -5446,7 +5446,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -5474,7 +5474,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Jordan Lawlar</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -5502,7 +5502,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Zach McKinstry</t>
+          <t>Jordan Lawlar</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -5530,17 +5530,17 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Matt Vierling</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -5551,24 +5551,24 @@
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Zach McKinstry</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -5579,14 +5579,14 @@
       <c r="E183" s="2" t="inlineStr"/>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Victor Mesa Jr.</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -5614,7 +5614,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Ha-Seong Kim</t>
+          <t>Blake Dunn</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -5642,7 +5642,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Blake Dunn</t>
+          <t>Ha-Seong Kim</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -5670,17 +5670,17 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Victor Mesa Jr.</t>
+          <t>Ildemaro Vargas</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -5691,14 +5691,14 @@
       <c r="E187" s="2" t="inlineStr"/>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -5726,7 +5726,7 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -5754,7 +5754,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Ildemaro Vargas</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -5782,7 +5782,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Kameron Misner</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -5810,7 +5810,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Kameron Misner</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -5894,7 +5894,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Michael Helman</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -5922,17 +5922,17 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -5943,24 +5943,24 @@
       <c r="E196" s="2" t="inlineStr"/>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Sandy Leon</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -5971,7 +5971,7 @@
       <c r="E197" s="2" t="inlineStr"/>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
@@ -6006,7 +6006,7 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>Braden Montgomery</t>
+          <t>Sandy Leon</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -6034,17 +6034,17 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Michael Helman</t>
+          <t>Braden Montgomery</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -6055,7 +6055,7 @@
       <c r="E200" s="2" t="inlineStr"/>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Pedro Pages</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -6146,7 +6146,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Pedro Pages</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -6174,7 +6174,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Jacob Gonzalez</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -6202,7 +6202,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Jacob Gonzalez</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -6314,7 +6314,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Max Schuemann</t>
+          <t>Hunter Feduccia</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -6342,7 +6342,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Hunter Feduccia</t>
+          <t>Max Schuemann</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -6370,7 +6370,7 @@
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -6426,7 +6426,7 @@
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -6454,17 +6454,17 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -6475,7 +6475,7 @@
       <c r="E215" s="2" t="inlineStr"/>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
@@ -6538,17 +6538,17 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Masataka Yoshida</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -6559,14 +6559,14 @@
       <c r="E218" s="2" t="inlineStr"/>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -6594,7 +6594,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Stuart Fairchild</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -6622,7 +6622,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Stuart Fairchild</t>
+          <t>Masataka Yoshida</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -6706,7 +6706,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>J.C. Escarra</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -6762,7 +6762,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>J.C. Escarra</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -6846,17 +6846,17 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -6867,14 +6867,14 @@
       <c r="E229" s="2" t="inlineStr"/>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -6902,7 +6902,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -6930,7 +6930,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -6958,7 +6958,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Drew Romo</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -6986,17 +6986,17 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -7007,14 +7007,14 @@
       <c r="E234" s="2" t="inlineStr"/>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Wade Meckler</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -7042,17 +7042,17 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Austin Hedges</t>
+          <t>Wade Meckler</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -7063,14 +7063,14 @@
       <c r="E236" s="2" t="inlineStr"/>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Austin Hedges</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -7098,7 +7098,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Drew Romo</t>
+          <t>Luis Rengifo</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -7126,7 +7126,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Luis Rengifo</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -7266,7 +7266,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -7322,7 +7322,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -7350,7 +7350,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Victor Robles</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -7378,7 +7378,7 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Victor Robles</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -7602,7 +7602,7 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>Justin Crawford</t>
+          <t>Sal Frelick</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -7630,7 +7630,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>Sal Frelick</t>
+          <t>Justin Crawford</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -7658,7 +7658,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
@@ -7686,7 +7686,7 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update odds files - Sun Jun 14 15:26:34 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F258"/>
+  <dimension ref="A1:F260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -663,7 +663,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+254</t>
+          <t>+255</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -686,7 +686,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -714,7 +714,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Juan Soto</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1132,47 +1132,47 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>+342</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>22.6%</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>22.6%</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Vargas</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>+344</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>22.5%</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Miguel Vargas</t>
+          <t>Julio Rodriguez</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>+344</t>
+          <t>+347</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1183,33 +1183,33 @@
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Julio Rodriguez</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>+347</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>22.4%</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>22.4%</t>
         </is>
@@ -1386,17 +1386,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+377</t>
+          <t>+375</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1407,24 +1407,24 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>21.1%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Dominic Canzone</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+378</t>
+          <t>+377</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1435,7 +1435,7 @@
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.0%</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1526,7 +1526,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1636,37 +1636,37 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Brandon Lowe</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>+401</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>20.0%</t>
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>+402</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>19.9%</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Bobby Witt Jr.</t>
+          <t>Willson Contreras</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1692,37 +1692,37 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>Willson Contreras</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>+402</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>19.9%</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>19.9%</t>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Brandon Lowe</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>+404</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Ben Rice</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1750,17 +1750,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+406</t>
+          <t>+412</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,24 +1771,24 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+409</t>
+          <t>+419</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1799,14 +1799,14 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Braxton Fulford</t>
+          <t>Cole Carrigg</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -1834,12 +1834,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+421</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1860,28 +1860,28 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>Willi Castro</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Christian Walker</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>+421</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>19.2%</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>19.2%</t>
         </is>
@@ -1890,17 +1890,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Braxton Fulford</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+421</t>
+          <t>+423</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1911,7 +1911,7 @@
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
@@ -1944,30 +1944,30 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Jarren Duran</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>+425</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>19.0%</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>19.0%</t>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Matt McLain</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>+430</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>18.9%</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
@@ -2002,17 +2002,17 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>+439</t>
+          <t>+440</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2023,24 +2023,24 @@
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>+440</t>
+          <t>+443</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2051,24 +2051,24 @@
       <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>+443</t>
+          <t>+446</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2079,24 +2079,24 @@
       <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>MJ Melendez</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>+446</t>
+          <t>+450</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2107,24 +2107,24 @@
       <c r="E59" s="2" t="inlineStr"/>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>MJ Melendez</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+455</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2135,7 +2135,7 @@
       <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2366,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -2394,7 +2394,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Yandy Diaz</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2450,7 +2450,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Keibert Ruiz</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2478,7 +2478,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Keibert Ruiz</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2674,12 +2674,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+497</t>
+          <t>+496</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -2702,17 +2702,17 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+497</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -2723,24 +2723,24 @@
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+502</t>
+          <t>+498</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2751,14 +2751,14 @@
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Rhys Hoskins</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Victor Mesa Jr.</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2812,75 +2812,75 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="3" t="inlineStr">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Victor Mesa Jr.</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>+502</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>16.6%</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>16.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
         <is>
           <t>Jac Caglianone</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>+503</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t>16.6%</t>
         </is>
       </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E85" s="3" t="inlineStr"/>
-      <c r="F85" s="3" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr"/>
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>16.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>Kyle Higashioka</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>+506</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>16.5%</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr"/>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Kyle Higashioka</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+512</t>
+          <t>+506</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -2891,7 +2891,7 @@
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
@@ -2924,28 +2924,28 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="inlineStr">
+      <c r="A89" s="3" t="inlineStr">
         <is>
           <t>Jacob Wilson</t>
         </is>
       </c>
-      <c r="B89" s="2" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>+519</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
+      <c r="C89" s="3" t="inlineStr">
         <is>
           <t>16.2%</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr"/>
-      <c r="F89" s="2" t="inlineStr">
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr"/>
+      <c r="F89" s="3" t="inlineStr">
         <is>
           <t>16.2%</t>
         </is>
@@ -2954,12 +2954,12 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Royce Lewis</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -2982,7 +2982,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Royce Lewis</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -3094,7 +3094,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3122,7 +3122,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3290,7 +3290,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3318,7 +3318,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -3570,17 +3570,17 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+547</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -3591,24 +3591,24 @@
       <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>+553</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -3619,19 +3619,19 @@
       <c r="E113" s="2" t="inlineStr"/>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Lars Nootbaar</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>+554</t>
+          <t>+553</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -3654,17 +3654,17 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Jordan Lawlar</t>
+          <t>Lars Nootbaar</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+554</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -3675,24 +3675,24 @@
       <c r="E115" s="2" t="inlineStr"/>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Jordan Lawlar</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>+565</t>
+          <t>+556</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -3703,24 +3703,24 @@
       <c r="E116" s="2" t="inlineStr"/>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Dalton Rushing</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>+565</t>
+          <t>+563</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -3731,19 +3731,19 @@
       <c r="E117" s="2" t="inlineStr"/>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Sterlin Thompson</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>+568</t>
+          <t>+565</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Sterlin Thompson</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -3794,17 +3794,17 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>+571</t>
+          <t>+568</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -3815,24 +3815,24 @@
       <c r="E120" s="2" t="inlineStr"/>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Kerry Carpenter</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>+576</t>
+          <t>+571</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -3843,24 +3843,24 @@
       <c r="E121" s="2" t="inlineStr"/>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Justin Foscue</t>
+          <t>Kerry Carpenter</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+576</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -3871,24 +3871,24 @@
       <c r="E122" s="2" t="inlineStr"/>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Blake Dunn</t>
+          <t>Nick Solak</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>+597</t>
+          <t>+589</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -3899,24 +3899,24 @@
       <c r="E123" s="2" t="inlineStr"/>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Justin Foscue</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>+597</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -3927,24 +3927,24 @@
       <c r="E124" s="2" t="inlineStr"/>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Jase Bowen</t>
+          <t>Blake Dunn</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>+598</t>
+          <t>+596</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -3955,19 +3955,19 @@
       <c r="E125" s="2" t="inlineStr"/>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Jasson Dominguez</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>+598</t>
+          <t>+597</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -3990,12 +3990,12 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Nick Solak</t>
+          <t>Jase Bowen</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+598</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -4018,7 +4018,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Alejandro Kirk</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -4046,7 +4046,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Alejandro Kirk</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -4074,7 +4074,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Jasson Dominguez</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -4102,7 +4102,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Jesus Sanchez</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -4158,7 +4158,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -4186,17 +4186,17 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Jesus Sanchez</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -4207,14 +4207,14 @@
       <c r="E134" s="2" t="inlineStr"/>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -4270,17 +4270,17 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -4291,24 +4291,24 @@
       <c r="E137" s="2" t="inlineStr"/>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -4319,7 +4319,7 @@
       <c r="E138" s="2" t="inlineStr"/>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
@@ -4354,17 +4354,17 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -4375,24 +4375,24 @@
       <c r="E140" s="2" t="inlineStr"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -4403,24 +4403,24 @@
       <c r="E141" s="2" t="inlineStr"/>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -4431,24 +4431,24 @@
       <c r="E142" s="2" t="inlineStr"/>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -4459,24 +4459,24 @@
       <c r="E143" s="2" t="inlineStr"/>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Ildemaro Vargas</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -4487,24 +4487,24 @@
       <c r="E144" s="2" t="inlineStr"/>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -4515,24 +4515,24 @@
       <c r="E145" s="2" t="inlineStr"/>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Ildemaro Vargas</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -4543,14 +4543,14 @@
       <c r="E146" s="2" t="inlineStr"/>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Amed Rosario</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -4578,7 +4578,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Jeremiah Jackson</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -4606,17 +4606,17 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -4627,24 +4627,24 @@
       <c r="E149" s="2" t="inlineStr"/>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -4655,24 +4655,24 @@
       <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Tyler Callihan</t>
+          <t>Amed Rosario</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -4683,24 +4683,24 @@
       <c r="E151" s="2" t="inlineStr"/>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Arias</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -4711,24 +4711,24 @@
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Tyler Callihan</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -4739,24 +4739,24 @@
       <c r="E153" s="2" t="inlineStr"/>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -4767,14 +4767,14 @@
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Heriberto Hernandez</t>
+          <t>Jimmy Crooks</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -4802,7 +4802,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Crooks</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -4830,17 +4830,17 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Drew Romo</t>
+          <t>Heriberto Hernandez</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -4851,14 +4851,14 @@
       <c r="E157" s="2" t="inlineStr"/>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Drew Romo</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -4886,7 +4886,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Gary Sanchez</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -4914,7 +4914,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Gary Sanchez</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -4942,17 +4942,17 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Tommy Troy</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -4963,24 +4963,24 @@
       <c r="E161" s="2" t="inlineStr"/>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Tommy Troy</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -4991,7 +4991,7 @@
       <c r="E162" s="2" t="inlineStr"/>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
@@ -5026,7 +5026,7 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>David Fry</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -5054,17 +5054,17 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>David Fry</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -5075,24 +5075,24 @@
       <c r="E165" s="2" t="inlineStr"/>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Sandy Leon</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -5103,7 +5103,7 @@
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
@@ -5138,17 +5138,17 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Sandy Leon</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -5159,14 +5159,14 @@
       <c r="E168" s="2" t="inlineStr"/>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
@@ -5194,7 +5194,7 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -5222,17 +5222,17 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>LuJames Groover</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -5243,7 +5243,7 @@
       <c r="E171" s="2" t="inlineStr"/>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
@@ -5278,17 +5278,17 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>Michael Conforto</t>
+          <t>Blaze Alexander</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -5299,24 +5299,24 @@
       <c r="E173" s="2" t="inlineStr"/>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Max Schuemann</t>
+          <t>LuJames Groover</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -5327,14 +5327,14 @@
       <c r="E174" s="2" t="inlineStr"/>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Michael Conforto</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -5362,17 +5362,17 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Jose Trevino</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -5383,24 +5383,24 @@
       <c r="E176" s="2" t="inlineStr"/>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Victor Robles</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -5411,14 +5411,14 @@
       <c r="E177" s="2" t="inlineStr"/>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -5446,7 +5446,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -5474,17 +5474,17 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -5495,24 +5495,24 @@
       <c r="E180" s="2" t="inlineStr"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Jose Trevino</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -5523,24 +5523,24 @@
       <c r="E181" s="2" t="inlineStr"/>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>Anthony Volpe</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -5551,24 +5551,24 @@
       <c r="E182" s="2" t="inlineStr"/>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Victor Robles</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -5579,7 +5579,7 @@
       <c r="E183" s="2" t="inlineStr"/>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
@@ -5642,7 +5642,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Owen Caissie</t>
+          <t>Max Schuemann</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -5670,7 +5670,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Tristan Gray</t>
+          <t>Owen Caissie</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -5698,17 +5698,17 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Tristan Gray</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -5719,14 +5719,14 @@
       <c r="E188" s="2" t="inlineStr"/>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -5782,17 +5782,17 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -5803,14 +5803,14 @@
       <c r="E191" s="2" t="inlineStr"/>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Kameron Misner</t>
+          <t>Jacob Gonzalez</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -5838,7 +5838,7 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Jacob Gonzalez</t>
+          <t>Michael Helman</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -5866,7 +5866,7 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Kameron Misner</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -5894,7 +5894,7 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -5922,7 +5922,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Michael Helman</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -5950,17 +5950,17 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Trey Mancini</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
@@ -5971,24 +5971,24 @@
       <c r="E197" s="2" t="inlineStr"/>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Trey Mancini</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -5999,7 +5999,7 @@
       <c r="E198" s="2" t="inlineStr"/>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Ali Sanchez</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -6062,7 +6062,7 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Richie Palacios</t>
+          <t>Anthony Volpe</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -6090,17 +6090,17 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Richie Palacios</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -6111,24 +6111,24 @@
       <c r="E202" s="2" t="inlineStr"/>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Jake Rogers</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -6139,24 +6139,24 @@
       <c r="E203" s="2" t="inlineStr"/>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Luis Torrens</t>
+          <t>Jake Rogers</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -6167,14 +6167,14 @@
       <c r="E204" s="2" t="inlineStr"/>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Samad Taylor</t>
+          <t>Jhonny Pereda</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -6202,17 +6202,17 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Samad Taylor</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -6223,24 +6223,24 @@
       <c r="E206" s="2" t="inlineStr"/>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Luis Torrens</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -6251,24 +6251,24 @@
       <c r="E207" s="2" t="inlineStr"/>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Ali Sanchez</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -6279,14 +6279,14 @@
       <c r="E208" s="2" t="inlineStr"/>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -6314,7 +6314,7 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -6342,17 +6342,17 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Nick Fortes</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -6363,24 +6363,24 @@
       <c r="E211" s="2" t="inlineStr"/>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -6391,24 +6391,24 @@
       <c r="E212" s="2" t="inlineStr"/>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -6419,14 +6419,14 @@
       <c r="E213" s="2" t="inlineStr"/>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Nick Fortes</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -6454,17 +6454,17 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Joe Mack</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -6475,19 +6475,19 @@
       <c r="E215" s="2" t="inlineStr"/>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Jhonny Pereda</t>
+          <t>Joe Mack</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
@@ -6510,17 +6510,17 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Andrew Vaughn</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -6531,24 +6531,24 @@
       <c r="E217" s="2" t="inlineStr"/>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Charles McAdoo</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -6559,14 +6559,14 @@
       <c r="E218" s="2" t="inlineStr"/>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Tristan Peters</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -6594,7 +6594,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Gleyber Torres</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -6622,17 +6622,17 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Tristan Peters</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -6643,24 +6643,24 @@
       <c r="E221" s="2" t="inlineStr"/>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Masataka Yoshida</t>
+          <t>Gleyber Torres</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -6671,14 +6671,14 @@
       <c r="E222" s="2" t="inlineStr"/>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Charles McAdoo</t>
+          <t>Masataka Yoshida</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -6734,17 +6734,17 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -6755,24 +6755,24 @@
       <c r="E225" s="2" t="inlineStr"/>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -6783,24 +6783,24 @@
       <c r="E226" s="2" t="inlineStr"/>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Miles Mastrobuoni</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -6811,24 +6811,24 @@
       <c r="E227" s="2" t="inlineStr"/>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Miles Mastrobuoni</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -6839,24 +6839,24 @@
       <c r="E228" s="2" t="inlineStr"/>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Colt Keith</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -6867,24 +6867,24 @@
       <c r="E229" s="2" t="inlineStr"/>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -6895,24 +6895,24 @@
       <c r="E230" s="2" t="inlineStr"/>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Patrick Bailey</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -6923,24 +6923,24 @@
       <c r="E231" s="2" t="inlineStr"/>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -6951,7 +6951,7 @@
       <c r="E232" s="2" t="inlineStr"/>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
@@ -6986,17 +6986,17 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Patrick Bailey</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -7007,24 +7007,24 @@
       <c r="E234" s="2" t="inlineStr"/>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Connor Norby</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -7035,14 +7035,14 @@
       <c r="E235" s="2" t="inlineStr"/>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Joey Loperfido</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -7070,17 +7070,17 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Joey Loperfido</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -7091,24 +7091,24 @@
       <c r="E237" s="2" t="inlineStr"/>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Connor Norby</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -7119,24 +7119,24 @@
       <c r="E238" s="2" t="inlineStr"/>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -7147,24 +7147,24 @@
       <c r="E239" s="2" t="inlineStr"/>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -7175,24 +7175,24 @@
       <c r="E240" s="2" t="inlineStr"/>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Daniel Susac</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -7203,24 +7203,24 @@
       <c r="E241" s="2" t="inlineStr"/>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Nasim Nunez</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -7231,24 +7231,24 @@
       <c r="E242" s="2" t="inlineStr"/>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Nasim Nunez</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1200</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.7%</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -7259,24 +7259,24 @@
       <c r="E243" s="2" t="inlineStr"/>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.7%</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Blake Perkins</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1200</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.7%</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -7287,24 +7287,24 @@
       <c r="E244" s="2" t="inlineStr"/>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.7%</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Luis Rengifo</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1260</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -7315,7 +7315,7 @@
       <c r="E245" s="2" t="inlineStr"/>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.4%</t>
         </is>
       </c>
     </row>
@@ -7350,7 +7350,7 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Luis Rengifo</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -7378,17 +7378,17 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Drew Gilbert</t>
+          <t>Jared Triolo</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1300</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -7399,14 +7399,14 @@
       <c r="E248" s="2" t="inlineStr"/>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>7.1%</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Blake Perkins</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -7434,17 +7434,17 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Drew Gilbert</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -7455,24 +7455,24 @@
       <c r="E250" s="2" t="inlineStr"/>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.0%</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>Isiah Kiner-Falefa</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>+1420</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -7483,24 +7483,24 @@
       <c r="E251" s="2" t="inlineStr"/>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>7.0%</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>Joey Ortiz</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>+1440</t>
+          <t>+1340</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -7511,24 +7511,24 @@
       <c r="E252" s="2" t="inlineStr"/>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>6.9%</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Isiah Kiner-Falefa</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>+1500</t>
+          <t>+1420</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -7539,24 +7539,24 @@
       <c r="E253" s="2" t="inlineStr"/>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>Jake Mangum</t>
+          <t>Joey Ortiz</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>+1600</t>
+          <t>+1440</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -7567,24 +7567,24 @@
       <c r="E254" s="2" t="inlineStr"/>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>6.5%</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>+1640</t>
+          <t>+1500</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -7595,24 +7595,24 @@
       <c r="E255" s="2" t="inlineStr"/>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>6.2%</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Jake Mangum</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>+1880</t>
+          <t>+1600</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -7623,24 +7623,24 @@
       <c r="E256" s="2" t="inlineStr"/>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>5.9%</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>Chandler Simpson</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>+1900</t>
+          <t>+1640</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>5.7%</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -7651,24 +7651,24 @@
       <c r="E257" s="2" t="inlineStr"/>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>5.7%</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>David Hamilton</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+1880</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -7678,6 +7678,62 @@
       </c>
       <c r="E258" s="2" t="inlineStr"/>
       <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>5.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>Chandler Simpson</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>+1900</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>5.0%</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr"/>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>Nico Hoerner</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>3.8%</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr"/>
+      <c r="F260" s="2" t="inlineStr">
         <is>
           <t>3.8%</t>
         </is>

</xml_diff>

<commit_message>
Update odds files - Mon Jun 15 13:36:34 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -523,12 +523,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>+235</t>
+          <t>+217</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>29.9%</t>
+          <t>31.5%</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -539,7 +539,7 @@
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>29.9%</t>
+          <t>31.5%</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>+248</t>
+          <t>+240</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -567,7 +567,7 @@
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>29.4%</t>
         </is>
       </c>
     </row>
@@ -602,17 +602,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Hunter Goodman</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>+268</t>
+          <t>+274</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -623,24 +623,24 @@
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>26.7%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+278</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -651,7 +651,7 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.5%</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>+295</t>
+          <t>+305</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>25.3%</t>
+          <t>24.7%</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -735,7 +735,7 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>25.3%</t>
+          <t>24.7%</t>
         </is>
       </c>
     </row>
@@ -798,17 +798,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Juan Soto</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>+324</t>
+          <t>+318</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.9%</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -819,24 +819,24 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Brandon Lowe</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>+327</t>
+          <t>+324</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -847,7 +847,7 @@
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.6%</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Brandon Lowe</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>+344</t>
+          <t>+334</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>23.0%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+352</t>
+          <t>+344</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -931,7 +931,7 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
@@ -943,12 +943,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+358</t>
+          <t>+350</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -959,24 +959,24 @@
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>+361</t>
+          <t>+352</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>22.1%</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -987,7 +987,7 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
@@ -1246,17 +1246,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>+395</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1267,7 +1267,7 @@
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
@@ -1302,17 +1302,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Kyle Stowers</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+418</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1323,24 +1323,24 @@
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Ketel Marte</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>+423</t>
+          <t>+420</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1351,80 +1351,80 @@
       <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="3" t="inlineStr">
         <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Ketel Marte</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>+423</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
           <t>19.1%</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>19.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Bobby Witt Jr.</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>+423</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>19.1%</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>19.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>Freddie Freeman</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>+427</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>19.0%</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>19.0%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>+439</t>
+          <t>+427</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1435,7 +1435,7 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>+455</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1547,7 +1547,7 @@
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
@@ -1610,12 +1610,12 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Joc Pederson</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>+476</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1638,17 +1638,17 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Joc Pederson</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>+479</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1659,24 +1659,24 @@
       <c r="E43" s="3" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>+486</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Max Muncy (ATH)</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+486</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1715,61 +1715,61 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
+          <t>17.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Max Muncy (ATH)</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>+487</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
           <t>17.0%</t>
         </is>
       </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>17.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Isaac Paredes</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>+490</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>16.9%</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>16.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Spencer Torkelson</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>+492</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>16.9%</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>16.9%</t>
         </is>
@@ -1778,12 +1778,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>+493</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1806,17 +1806,17 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Lars Nootbaar</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>+496</t>
+          <t>+492</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1827,80 +1827,80 @@
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr">
         <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Lars Nootbaar</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>+496</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
           <t>16.8%</t>
         </is>
       </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>16.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Salvador Perez</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>+496</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>16.8%</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>16.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>Jonathan Aranda</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>+498</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>16.7%</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>+502</t>
+          <t>+498</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -1911,14 +1911,14 @@
       <c r="E52" s="3" t="inlineStr"/>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Tyler Callihan</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1946,17 +1946,17 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>+507</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1967,24 +1967,24 @@
       <c r="E54" s="3" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>+508</t>
+          <t>+515</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1995,24 +1995,24 @@
       <c r="E55" s="3" t="inlineStr"/>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Francisco Alvarez</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>+515</t>
+          <t>+519</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2023,24 +2023,24 @@
       <c r="E56" s="3" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>+519</t>
+          <t>+524</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2051,24 +2051,24 @@
       <c r="E57" s="3" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Tyler Callihan</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>+523</t>
+          <t>+525</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2079,24 +2079,24 @@
       <c r="E58" s="3" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>+524</t>
+          <t>+528</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2107,14 +2107,14 @@
       <c r="E59" s="3" t="inlineStr"/>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>MJ Melendez</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -2142,7 +2142,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>MJ Melendez</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -2198,12 +2198,12 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+534</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2224,75 +2224,75 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>Wyatt Langford</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>+534</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>15.8%</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr"/>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>15.8%</t>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>+535</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>15.7%</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>+535</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>15.7%</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr"/>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>15.7%</t>
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Dansby Swanson</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>15.6%</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>+538</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2303,24 +2303,24 @@
       <c r="E66" s="3" t="inlineStr"/>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+551</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2331,24 +2331,24 @@
       <c r="E67" s="3" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2359,24 +2359,24 @@
       <c r="E68" s="3" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Ryan Ward</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2387,24 +2387,24 @@
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2415,19 +2415,19 @@
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>+552</t>
+          <t>+554</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -2450,17 +2450,17 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>+552</t>
+          <t>+556</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2471,7 +2471,7 @@
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
@@ -2730,17 +2730,17 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>+594</t>
+          <t>+598</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -2751,19 +2751,19 @@
       <c r="E82" s="3" t="inlineStr"/>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>+598</t>
+          <t>+599</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -2814,12 +2814,12 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -2842,17 +2842,17 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2863,14 +2863,14 @@
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -2926,7 +2926,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2954,17 +2954,17 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Noelvi Marte</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -2975,14 +2975,14 @@
       <c r="E90" s="3" t="inlineStr"/>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -3010,7 +3010,7 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Curtis Mead</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -3036,65 +3036,65 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Brandon Marsh</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr"/>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>Jac Caglianone</t>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>+630</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>13.7%</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr"/>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
         <is>
           <t>13.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="3" t="inlineStr">
-        <is>
-          <t>Bo Bichette</t>
-        </is>
-      </c>
-      <c r="B94" s="3" t="inlineStr">
-        <is>
-          <t>+640</t>
-        </is>
-      </c>
-      <c r="C94" s="3" t="inlineStr">
-        <is>
-          <t>13.5%</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E94" s="3" t="inlineStr"/>
-      <c r="F94" s="3" t="inlineStr">
-        <is>
-          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Noelvi Marte</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -3178,7 +3178,7 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -3234,7 +3234,7 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Ryan Vilade</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -3262,17 +3262,17 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -3283,14 +3283,14 @@
       <c r="E101" s="3" t="inlineStr"/>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Austin Slater</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -3318,7 +3318,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Ryan Vilade</t>
+          <t>Austin Slater</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -3374,7 +3374,7 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Braxton Fulford</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -3402,7 +3402,7 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Braxton Fulford</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Kyle Higashioka</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -3458,7 +3458,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Kyle Higashioka</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -3486,17 +3486,17 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       <c r="E109" s="3" t="inlineStr"/>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
@@ -3542,17 +3542,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -3563,7 +3563,7 @@
       <c r="E111" s="3" t="inlineStr"/>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
@@ -3654,7 +3654,7 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -3682,7 +3682,7 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>Matt Vierling</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -3710,7 +3710,7 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Lane Thomas</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -3738,7 +3738,7 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Matt Vierling</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -3766,7 +3766,7 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Lane Thomas</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -3822,7 +3822,7 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Crooks</t>
+          <t>Pavin Smith</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -3850,7 +3850,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Pavin Smith</t>
+          <t>Jimmy Crooks</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -3934,7 +3934,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Nick Fortes</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -3962,7 +3962,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Nick Fortes</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3990,7 +3990,7 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -4102,7 +4102,7 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Blaze Jordan</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -4130,7 +4130,7 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>Blaze Jordan</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -4158,7 +4158,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -4186,7 +4186,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -4270,7 +4270,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Ryan Kreidler</t>
+          <t>Troy Johnston</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -4298,7 +4298,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>Alex Jackson</t>
+          <t>Ryan Kreidler</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -4326,7 +4326,7 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Alex Jackson</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -4380,30 +4380,30 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>Jacob Wilson</t>
-        </is>
-      </c>
-      <c r="B141" s="2" t="inlineStr">
-        <is>
-          <t>+930</t>
-        </is>
-      </c>
-      <c r="C141" s="2" t="inlineStr">
-        <is>
-          <t>9.7%</t>
-        </is>
-      </c>
-      <c r="D141" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E141" s="2" t="inlineStr"/>
-      <c r="F141" s="2" t="inlineStr">
-        <is>
-          <t>9.7%</t>
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>Xander Bogaerts</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr"/>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
@@ -4464,28 +4464,28 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="3" t="inlineStr">
-        <is>
-          <t>Xander Bogaerts</t>
-        </is>
-      </c>
-      <c r="B144" s="3" t="inlineStr">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Jacob Wilson</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
         <is>
           <t>+950</t>
         </is>
       </c>
-      <c r="C144" s="3" t="inlineStr">
+      <c r="C144" s="2" t="inlineStr">
         <is>
           <t>9.5%</t>
         </is>
       </c>
-      <c r="D144" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E144" s="3" t="inlineStr"/>
-      <c r="F144" s="3" t="inlineStr">
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr">
         <is>
           <t>9.5%</t>
         </is>
@@ -4522,7 +4522,7 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>Ryan Waldschmidt</t>
+          <t>Joey Loperfido</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -4578,12 +4578,12 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>Joey Loperfido</t>
+          <t>Ryan Waldschmidt</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -4606,7 +4606,7 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>Joe Mack</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -4634,17 +4634,17 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Joe Mack</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -4655,14 +4655,14 @@
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Jared Triolo</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
@@ -4690,7 +4690,7 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Zach McKinstry</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
@@ -4718,17 +4718,17 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>Zach McKinstry</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4739,14 +4739,14 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Colt Keith</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
@@ -4774,7 +4774,7 @@
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -4830,7 +4830,7 @@
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Rincones Jr.</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
@@ -4858,7 +4858,7 @@
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Gabriel Rincones Jr.</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -4914,17 +4914,17 @@
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -4935,14 +4935,14 @@
       <c r="E160" s="3" t="inlineStr"/>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -4970,17 +4970,17 @@
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Nolan Schanuel</t>
+          <t>Ben Williamson</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4991,24 +4991,24 @@
       <c r="E162" s="3" t="inlineStr"/>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>Ben Williamson</t>
+          <t>Nolan Schanuel</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -5019,7 +5019,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
@@ -5082,17 +5082,17 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Wade Meckler</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -5103,14 +5103,14 @@
       <c r="E166" s="3" t="inlineStr"/>
       <c r="F166" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
@@ -5138,17 +5138,17 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>LuJames Groover</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -5159,14 +5159,14 @@
       <c r="E168" s="3" t="inlineStr"/>
       <c r="F168" s="3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>Wade Meckler</t>
+          <t>LuJames Groover</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update odds files - Mon Jun 15 19:34:56 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F181"/>
+  <dimension ref="A1:F180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -495,12 +495,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+215</t>
+          <t>+214</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>31.7%</t>
+          <t>31.8%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>31.7%</t>
+          <t>31.8%</t>
         </is>
       </c>
     </row>
@@ -523,12 +523,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>+217</t>
+          <t>+215</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>31.5%</t>
+          <t>31.7%</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -539,7 +539,7 @@
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>31.5%</t>
+          <t>31.7%</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>+240</t>
+          <t>+241</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>29.3%</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -567,7 +567,7 @@
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>29.3%</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>+255</t>
+          <t>+245</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>29.0%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -595,7 +595,7 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>29.0%</t>
         </is>
       </c>
     </row>
@@ -607,12 +607,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>+274</t>
+          <t>+253</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>28.3%</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -623,24 +623,24 @@
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>28.3%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Yordan Alvarez</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+278</t>
+          <t>+273</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -651,24 +651,24 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>26.8%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Yordan Alvarez</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>+279</t>
+          <t>+273</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -679,24 +679,24 @@
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>26.8%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>+293</t>
+          <t>+286</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.9%</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -707,24 +707,24 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.9%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Max Muncy (LAD)</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>+305</t>
+          <t>+288</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>24.7%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -735,52 +735,52 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
+          <t>25.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Max Muncy (LAD)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>+305</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
           <t>24.7%</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>+311</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>24.3%</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>24.3%</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>24.7%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>+316</t>
+          <t>+309</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>24.4%</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -791,7 +791,7 @@
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>24.4%</t>
         </is>
       </c>
     </row>
@@ -803,12 +803,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>+318</t>
+          <t>+314</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>24.2%</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -819,24 +819,24 @@
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>24.2%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Juan Soto</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>+324</t>
+          <t>+316</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -847,35 +847,35 @@
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>24.0%</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Michael Busch</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>+332</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>23.1%</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>23.1%</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>+318</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>23.9%</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
@@ -887,12 +887,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>+334</t>
+          <t>+327</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -903,7 +903,7 @@
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.4%</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+344</t>
+          <t>+332</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -931,14 +931,14 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Eugenio Suarez</t>
+          <t>Yandy Diaz</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -966,17 +966,17 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>+352</t>
+          <t>+351</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>+373</t>
+          <t>+354</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1015,24 +1015,24 @@
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>22.0%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>+373</t>
+          <t>+358</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1043,19 +1043,19 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>+374</t>
+          <t>+375</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1078,17 +1078,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Kerry Carpenter</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>+379</t>
+          <t>+377</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1099,24 +1099,24 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.0%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>+381</t>
+          <t>+379</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1127,24 +1127,24 @@
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>+382</t>
+          <t>+385</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>20.6%</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1155,24 +1155,24 @@
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>20.6%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Eugenio Suarez</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>+387</t>
+          <t>+385</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>20.6%</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1183,24 +1183,24 @@
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>20.6%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>+394</t>
+          <t>+389</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1211,19 +1211,19 @@
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Kerry Carpenter</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>+395</t>
+          <t>+394</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1246,7 +1246,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1274,17 +1274,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>+413</t>
+          <t>+400</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1295,24 +1295,24 @@
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>+418</t>
+          <t>+403</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1323,24 +1323,24 @@
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Kyle Stowers</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+404</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1351,80 +1351,80 @@
       <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Ketel Marte</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>+423</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>19.1%</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>19.1%</t>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>+405</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Bobby Witt Jr.</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>+423</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>19.1%</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>19.1%</t>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Alec Burleson</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>+413</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>+427</t>
+          <t>+422</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>+439</t>
+          <t>+423</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>+446</t>
+          <t>+424</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1491,7 +1491,7 @@
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
@@ -1503,12 +1503,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>+447</t>
+          <t>+432</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1519,24 +1519,24 @@
       <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Joc Pederson</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>+469</t>
+          <t>+454</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1547,24 +1547,24 @@
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Dalton Rushing</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+462</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1575,24 +1575,24 @@
       <c r="E40" s="3" t="inlineStr"/>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Max Muncy (ATH)</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+466</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1603,24 +1603,24 @@
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1631,24 +1631,24 @@
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Joc Pederson</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>+476</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1659,24 +1659,24 @@
       <c r="E43" s="3" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>+479</t>
+          <t>+473</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>+486</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1715,24 +1715,24 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Max Muncy (ATH)</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1743,7 +1743,7 @@
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,24 +1771,24 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="3" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>+492</t>
+          <t>+483</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1827,24 +1827,24 @@
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.2%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Lars Nootbaar</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>+496</t>
+          <t>+483</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -1855,52 +1855,52 @@
       <c r="E50" s="3" t="inlineStr"/>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>17.2%</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Salvador Perez</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>+496</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>16.8%</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>16.8%</t>
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Corbin Carroll</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>+487</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>17.0%</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>17.0%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Royce Lewis</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+496</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -1911,19 +1911,19 @@
       <c r="E52" s="3" t="inlineStr"/>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>+502</t>
+          <t>+501</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -1946,17 +1946,17 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Tyler Callihan</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>+508</t>
+          <t>+504</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1967,7 +1967,7 @@
       <c r="E54" s="3" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>+515</t>
+          <t>+507</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1995,24 +1995,24 @@
       <c r="E55" s="3" t="inlineStr"/>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>+519</t>
+          <t>+511</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2023,24 +2023,24 @@
       <c r="E56" s="3" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>+524</t>
+          <t>+514</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2051,80 +2051,80 @@
       <c r="E57" s="3" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>Tyler Callihan</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>+525</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>16.0%</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr"/>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>16.0%</t>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>+514</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>Jared Young</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>+528</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>15.9%</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr"/>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>15.9%</t>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>+518</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>MJ Melendez</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>+529</t>
+          <t>+519</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2135,24 +2135,24 @@
       <c r="E60" s="3" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Lars Nootbaar</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>+529</t>
+          <t>+522</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2163,52 +2163,52 @@
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>+533</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>15.8%</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>15.8%</t>
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Moises Ballesteros</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>+526</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>16.0%</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr"/>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+529</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2219,52 +2219,52 @@
       <c r="E63" s="3" t="inlineStr"/>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>+535</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>15.7%</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>15.7%</t>
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>MJ Melendez</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>+529</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>15.9%</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr"/>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>+540</t>
+          <t>+532</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2275,24 +2275,24 @@
       <c r="E65" s="3" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Ryan Ward</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2303,24 +2303,24 @@
       <c r="E66" s="3" t="inlineStr"/>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2331,24 +2331,24 @@
       <c r="E67" s="3" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>+552</t>
+          <t>+534</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2359,24 +2359,24 @@
       <c r="E68" s="3" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>+552</t>
+          <t>+536</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2387,24 +2387,24 @@
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>+552</t>
+          <t>+542</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2415,24 +2415,24 @@
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>+554</t>
+          <t>+544</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2443,24 +2443,24 @@
       <c r="E71" s="3" t="inlineStr"/>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2471,24 +2471,24 @@
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Keibert Ruiz</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>+562</t>
+          <t>+551</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2499,52 +2499,52 @@
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>Matt McLain</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>+564</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>15.1%</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>15.1%</t>
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Manny Machado</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>+559</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr"/>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>+566</t>
+          <t>+559</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2555,42 +2555,42 @@
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>Dylan Crews</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>+567</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>15.0%</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr"/>
-      <c r="F76" s="3" t="inlineStr">
-        <is>
-          <t>15.0%</t>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>+562</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>CJ Abrams</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -2618,7 +2618,7 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -2646,12 +2646,12 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Royce Lewis</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>+573</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -2674,12 +2674,12 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>+574</t>
+          <t>+576</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -2700,47 +2700,47 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="3" t="inlineStr">
-        <is>
-          <t>Kevin McGonigle</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>+589</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="inlineStr">
-        <is>
-          <t>14.5%</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr"/>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>14.5%</t>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>+578</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>+598</t>
+          <t>+583</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -2751,24 +2751,24 @@
       <c r="E82" s="3" t="inlineStr"/>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2779,7 +2779,7 @@
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
@@ -2791,12 +2791,12 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+593</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2807,24 +2807,24 @@
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+593</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2835,24 +2835,24 @@
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Austin Slater</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2863,24 +2863,24 @@
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Curtis Mead</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -2891,24 +2891,24 @@
       <c r="E87" s="3" t="inlineStr"/>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2919,35 +2919,35 @@
       <c r="E88" s="3" t="inlineStr"/>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>Zack Gelof</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>+610</t>
-        </is>
-      </c>
-      <c r="C89" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E89" s="3" t="inlineStr"/>
-      <c r="F89" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Matt McLain</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
@@ -2982,17 +2982,17 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -3003,24 +3003,24 @@
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -3031,24 +3031,24 @@
       <c r="E92" s="3" t="inlineStr"/>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -3059,52 +3059,52 @@
       <c r="E93" s="3" t="inlineStr"/>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>+630</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr"/>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Bo Bichette</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr"/>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Keibert Ruiz</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -3115,14 +3115,14 @@
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>Dane Myers</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -3150,7 +3150,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -3178,17 +3178,17 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Braxton Fulford</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -3199,14 +3199,14 @@
       <c r="E98" s="3" t="inlineStr"/>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -3234,7 +3234,7 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Ryan Vilade</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -3262,7 +3262,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -3290,17 +3290,17 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
@@ -3311,14 +3311,14 @@
       <c r="E102" s="3" t="inlineStr"/>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Austin Slater</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -3374,17 +3374,17 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -3395,14 +3395,14 @@
       <c r="E105" s="3" t="inlineStr"/>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Braxton Fulford</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -3430,17 +3430,17 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Kyle Higashioka</t>
+          <t>Blake Dunn</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -3451,24 +3451,24 @@
       <c r="E107" s="3" t="inlineStr"/>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -3479,14 +3479,14 @@
       <c r="E108" s="3" t="inlineStr"/>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -3514,7 +3514,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Heriberto Hernandez</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -3542,17 +3542,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Ryan Vilade</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -3563,24 +3563,24 @@
       <c r="E111" s="3" t="inlineStr"/>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Kyle Higashioka</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -3591,24 +3591,24 @@
       <c r="E112" s="3" t="inlineStr"/>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Heriberto Hernandez</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -3619,24 +3619,24 @@
       <c r="E113" s="3" t="inlineStr"/>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -3647,24 +3647,24 @@
       <c r="E114" s="3" t="inlineStr"/>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Edmundo Sosa</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -3675,24 +3675,24 @@
       <c r="E115" s="3" t="inlineStr"/>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Tyler Freeman</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -3703,7 +3703,7 @@
       <c r="E116" s="3" t="inlineStr"/>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
@@ -3715,12 +3715,12 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -3731,24 +3731,24 @@
       <c r="E117" s="3" t="inlineStr"/>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Matt Vierling</t>
+          <t>Starling Marte</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -3759,24 +3759,24 @@
       <c r="E118" s="3" t="inlineStr"/>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Matt Vierling</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+740</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -3787,24 +3787,24 @@
       <c r="E119" s="3" t="inlineStr"/>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>Starling Marte</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -3815,24 +3815,24 @@
       <c r="E120" s="3" t="inlineStr"/>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Pavin Smith</t>
+          <t>Cole Carrigg</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3843,24 +3843,24 @@
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Crooks</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
@@ -3871,24 +3871,24 @@
       <c r="E122" s="3" t="inlineStr"/>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -3899,24 +3899,24 @@
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>Owen Caissie</t>
+          <t>Pavin Smith</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -3927,24 +3927,24 @@
       <c r="E124" s="3" t="inlineStr"/>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -3955,24 +3955,24 @@
       <c r="E125" s="3" t="inlineStr"/>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Nick Fortes</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -3983,24 +3983,24 @@
       <c r="E126" s="3" t="inlineStr"/>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Gleyber Torres</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -4011,24 +4011,24 @@
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Alex Jackson</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
@@ -4039,24 +4039,24 @@
       <c r="E128" s="3" t="inlineStr"/>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>Tyler Freeman</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
@@ -4067,14 +4067,14 @@
       <c r="E129" s="3" t="inlineStr"/>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -4102,17 +4102,17 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>Blaze Jordan</t>
+          <t>Nick Fortes</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -4123,24 +4123,24 @@
       <c r="E131" s="3" t="inlineStr"/>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Owen Caissie</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
@@ -4151,14 +4151,14 @@
       <c r="E132" s="3" t="inlineStr"/>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.3%</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Joe Mack</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -4186,17 +4186,17 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Rodolfo Duran</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
@@ -4207,24 +4207,24 @@
       <c r="E134" s="3" t="inlineStr"/>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Jimmy Crooks</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="E135" s="3" t="inlineStr"/>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>Gleyber Torres</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
@@ -4263,24 +4263,24 @@
       <c r="E136" s="3" t="inlineStr"/>
       <c r="F136" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -4291,52 +4291,52 @@
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="3" t="inlineStr">
-        <is>
-          <t>Ryan Kreidler</t>
-        </is>
-      </c>
-      <c r="B138" s="3" t="inlineStr">
-        <is>
-          <t>+900</t>
-        </is>
-      </c>
-      <c r="C138" s="3" t="inlineStr">
-        <is>
-          <t>10.0%</t>
-        </is>
-      </c>
-      <c r="D138" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E138" s="3" t="inlineStr"/>
-      <c r="F138" s="3" t="inlineStr">
-        <is>
-          <t>10.0%</t>
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Jacob Wilson</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr"/>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Alex Jackson</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -4347,24 +4347,24 @@
       <c r="E139" s="3" t="inlineStr"/>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -4375,14 +4375,14 @@
       <c r="E140" s="3" t="inlineStr"/>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>Xander Bogaerts</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -4410,7 +4410,7 @@
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>Rodolfo Duran</t>
+          <t>Zach McKinstry</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -4438,17 +4438,17 @@
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Ryan Kreidler</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
@@ -4459,42 +4459,42 @@
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="inlineStr">
-        <is>
-          <t>Jacob Wilson</t>
-        </is>
-      </c>
-      <c r="B144" s="2" t="inlineStr">
-        <is>
-          <t>+950</t>
-        </is>
-      </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t>9.5%</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E144" s="2" t="inlineStr"/>
-      <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t>9.5%</t>
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>Colt Keith</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr"/>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>Justin Crawford</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -4522,17 +4522,17 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>Joey Loperfido</t>
+          <t>Gabriel Rincones Jr.</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
@@ -4543,19 +4543,19 @@
       <c r="E146" s="3" t="inlineStr"/>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Jase Bowen</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
@@ -4583,12 +4583,12 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
@@ -4599,24 +4599,24 @@
       <c r="E148" s="3" t="inlineStr"/>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Justin Crawford</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -4627,24 +4627,24 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>Joe Mack</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -4655,14 +4655,14 @@
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Blaze Jordan</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
@@ -4690,7 +4690,7 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>Zach McKinstry</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
@@ -4718,17 +4718,17 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4739,24 +4739,24 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -4767,24 +4767,24 @@
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Jared Triolo</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
@@ -4795,24 +4795,24 @@
       <c r="E155" s="3" t="inlineStr"/>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>Tommy Troy</t>
+          <t>Joey Loperfido</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -4823,24 +4823,24 @@
       <c r="E156" s="3" t="inlineStr"/>
       <c r="F156" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -4851,14 +4851,14 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Rincones Jr.</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -4886,17 +4886,17 @@
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>Jase Bowen</t>
+          <t>Tommy Troy</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -4907,7 +4907,7 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
@@ -4919,12 +4919,12 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -4935,14 +4935,14 @@
       <c r="E160" s="3" t="inlineStr"/>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -4970,17 +4970,17 @@
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Ben Williamson</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4991,24 +4991,24 @@
       <c r="E162" s="3" t="inlineStr"/>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>Nolan Schanuel</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -5019,14 +5019,14 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>Austin Martin</t>
+          <t>Christian Vazquez</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -5054,17 +5054,17 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>Christian Vazquez</t>
+          <t>Ben Williamson</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -5075,24 +5075,24 @@
       <c r="E165" s="3" t="inlineStr"/>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>Wade Meckler</t>
+          <t>LuJames Groover</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -5103,24 +5103,24 @@
       <c r="E166" s="3" t="inlineStr"/>
       <c r="F166" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -5131,24 +5131,24 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Nolan Schanuel</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1200</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>7.7%</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -5159,24 +5159,24 @@
       <c r="E168" s="3" t="inlineStr"/>
       <c r="F168" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>7.7%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>LuJames Groover</t>
+          <t>Wade Meckler</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -5187,24 +5187,24 @@
       <c r="E169" s="3" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Will Wagner</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -5215,24 +5215,24 @@
       <c r="E170" s="3" t="inlineStr"/>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Xavier Edwards</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -5243,7 +5243,7 @@
       <c r="E171" s="3" t="inlineStr"/>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
@@ -5255,12 +5255,12 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1280</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -5271,24 +5271,24 @@
       <c r="E172" s="3" t="inlineStr"/>
       <c r="F172" s="3" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>Jacob Young</t>
+          <t>Austin Martin</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1280</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -5299,7 +5299,7 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5334,7 @@
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>Will Wagner</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -5362,7 +5362,7 @@
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Samad Taylor</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -5390,17 +5390,17 @@
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>Samad Taylor</t>
+          <t>Jacob Young</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+1380</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -5411,24 +5411,24 @@
       <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>Nasim Nunez</t>
+          <t>Jake Mangum</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>+1440</t>
+          <t>+1640</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>5.7%</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -5439,24 +5439,24 @@
       <c r="E178" s="3" t="inlineStr"/>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>5.7%</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>Jake Mangum</t>
+          <t>Nasim Nunez</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>+1560</t>
+          <t>+1680</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -5467,24 +5467,24 @@
       <c r="E179" s="3" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>5.6%</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>Xavier Edwards</t>
+          <t>Nicky Lopez</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>+1600</t>
+          <t>+1780</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.3%</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -5494,34 +5494,6 @@
       </c>
       <c r="E180" s="3" t="inlineStr"/>
       <c r="F180" s="3" t="inlineStr">
-        <is>
-          <t>5.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="3" t="inlineStr">
-        <is>
-          <t>Nicky Lopez</t>
-        </is>
-      </c>
-      <c r="B181" s="3" t="inlineStr">
-        <is>
-          <t>+1780</t>
-        </is>
-      </c>
-      <c r="C181" s="3" t="inlineStr">
-        <is>
-          <t>5.3%</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E181" s="3" t="inlineStr"/>
-      <c r="F181" s="3" t="inlineStr">
         <is>
           <t>5.3%</t>
         </is>

</xml_diff>

<commit_message>
Update odds files - Mon Jun 15 21:45:34 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F181"/>
+  <dimension ref="A1:F180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -602,17 +602,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Nick Kurtz</t>
+          <t>Hunter Goodman</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>+245</t>
+          <t>+244</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>29.1%</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -623,24 +623,24 @@
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>29.1%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+249</t>
+          <t>+253</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>28.3%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -651,7 +651,7 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>28.3%</t>
         </is>
       </c>
     </row>
@@ -852,75 +852,75 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>James Wood</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>+316</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>24.0%</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>24.0%</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>+318</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>23.9%</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>+318</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>23.9%</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>23.9%</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Mike Trout</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>+320</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>23.8%</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>23.8%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+325</t>
+          <t>+327</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.4%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+327</t>
+          <t>+333</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -959,7 +959,7 @@
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
@@ -1022,17 +1022,17 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>+356</t>
+          <t>+355</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1043,24 +1043,24 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>22.0%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+356</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>21.9%</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1071,24 +1071,24 @@
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>+370</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1099,7 +1099,7 @@
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>21.7%</t>
         </is>
       </c>
     </row>
@@ -1218,17 +1218,17 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+393</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1239,19 +1239,19 @@
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.3%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>+401</t>
+          <t>+400</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1442,17 +1442,17 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>+445</t>
+          <t>+444</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Ketel Marte</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+445</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1491,7 +1491,7 @@
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
@@ -1554,17 +1554,17 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>+458</t>
+          <t>+456</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1575,24 +1575,24 @@
       <c r="E40" s="3" t="inlineStr"/>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>+469</t>
+          <t>+458</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1603,24 +1603,24 @@
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Dalton Rushing</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1631,14 +1631,14 @@
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1722,17 +1722,17 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>+479</t>
+          <t>+482</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1743,19 +1743,19 @@
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.2%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>+482</t>
+          <t>+483</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1778,7 +1778,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Max Muncy (ATH)</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1804,58 +1804,58 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>Max Muncy (ATH)</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Cortes</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>+483</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>17.2%</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>17.2%</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>Carlos Cortes</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>+483</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>17.2%</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr"/>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>17.2%</t>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>+487</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>17.0%</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>17.0%</t>
         </is>
       </c>
     </row>
@@ -1888,70 +1888,70 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>+487</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Tyler Callihan</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>+489</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>17.0%</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="3" t="inlineStr">
         <is>
           <t>17.0%</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>Tyler Callihan</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>+489</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>17.0%</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr"/>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>17.0%</t>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Tyler Stephenson</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>+492</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>+492</t>
+          <t>+493</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -1974,17 +1974,17 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>+492</t>
+          <t>+494</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1995,24 +1995,24 @@
       <c r="E55" s="3" t="inlineStr"/>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Lars Nootbaar</t>
+          <t>Royce Lewis</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>+492</t>
+          <t>+495</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2023,52 +2023,52 @@
       <c r="E56" s="3" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>Spencer Torkelson</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>+493</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>16.9%</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>16.9%</t>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Bryson Stott</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>+498</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>+494</t>
+          <t>+499</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2079,52 +2079,52 @@
       <c r="E58" s="3" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>Royce Lewis</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>+495</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>16.8%</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr"/>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>16.8%</t>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>+501</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>16.6%</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>+499</t>
+          <t>+507</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2135,52 +2135,52 @@
       <c r="E60" s="3" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>+501</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>16.6%</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr"/>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>16.6%</t>
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Lars Nootbaar</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>+509</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>16.4%</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Francisco Alvarez</t>
+          <t>MJ Melendez</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>+507</t>
+          <t>+511</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2191,35 +2191,35 @@
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>MJ Melendez</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>+511</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>16.4%</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr"/>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>16.4%</t>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>+514</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
@@ -2252,28 +2252,28 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Salvador Perez</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>+514</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Jackson Merrill</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>+515</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>16.3%</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr"/>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>16.3%</t>
         </is>
@@ -2366,17 +2366,17 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>+532</t>
+          <t>+529</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2387,19 +2387,19 @@
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+532</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -2450,12 +2450,12 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Ryan Ward</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -2478,17 +2478,17 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>+536</t>
+          <t>+534</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2499,7 +2499,7 @@
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
@@ -2618,12 +2618,12 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>+569</t>
+          <t>+571</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -2646,12 +2646,12 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Curtis Mead</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>+571</t>
+          <t>+573</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -2674,17 +2674,17 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Curtis Mead</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>+573</t>
+          <t>+574</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -2695,61 +2695,61 @@
       <c r="E80" s="3" t="inlineStr"/>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="3" t="inlineStr">
-        <is>
-          <t>Manny Machado</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>+574</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="inlineStr">
-        <is>
-          <t>14.8%</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr"/>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>14.8%</t>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>+578</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>+578</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Josh Jung</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>+581</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
         <is>
           <t>14.7%</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr"/>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr"/>
+      <c r="F82" s="3" t="inlineStr">
         <is>
           <t>14.7%</t>
         </is>
@@ -2758,17 +2758,17 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>+587</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2779,52 +2779,52 @@
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="3" t="inlineStr">
-        <is>
-          <t>Brandon Marsh</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>+583</t>
-        </is>
-      </c>
-      <c r="C84" s="3" t="inlineStr">
-        <is>
-          <t>14.6%</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr"/>
-      <c r="F84" s="3" t="inlineStr">
-        <is>
-          <t>14.6%</t>
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>+589</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>14.5%</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2835,33 +2835,33 @@
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>+589</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Zack Gelof</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>+591</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t>14.5%</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr"/>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr"/>
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>14.5%</t>
         </is>
@@ -2870,12 +2870,12 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -2898,17 +2898,17 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Endy Rodriguez</t>
+          <t>Brice Matthews</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>+592</t>
+          <t>+594</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2919,24 +2919,24 @@
       <c r="E88" s="3" t="inlineStr"/>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Brice Matthews</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>+594</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2947,14 +2947,14 @@
       <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -2980,28 +2980,28 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>Matt McLain</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Brandon Marsh</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>+600</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr"/>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr"/>
+      <c r="F91" s="3" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
@@ -3010,17 +3010,17 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -3031,14 +3031,14 @@
       <c r="E92" s="3" t="inlineStr"/>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -3066,17 +3066,17 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -3087,7 +3087,7 @@
       <c r="E94" s="3" t="inlineStr"/>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3178,7 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Braxton Fulford</t>
+          <t>Keibert Ruiz</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -3206,7 +3206,7 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Noelvi Marte</t>
+          <t>Braxton Fulford</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -3234,7 +3234,7 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Keibert Ruiz</t>
+          <t>Noelvi Marte</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -3262,7 +3262,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Taylor Trammell</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -3290,7 +3290,7 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Gavin Sheets</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -3318,7 +3318,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Taylor Trammell</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -3514,7 +3514,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>Heriberto Hernandez</t>
+          <t>Starling Marte</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -3542,7 +3542,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Ryan Vilade</t>
+          <t>Heriberto Hernandez</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
@@ -3570,7 +3570,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Ryan Vilade</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
@@ -3598,7 +3598,7 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Starling Marte</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -3654,7 +3654,7 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -3766,17 +3766,17 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -3787,14 +3787,14 @@
       <c r="E119" s="3" t="inlineStr"/>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -3822,17 +3822,17 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Gleyber Torres</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3843,7 +3843,7 @@
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
@@ -3878,17 +3878,17 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Gleyber Torres</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -3899,14 +3899,14 @@
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Alex Jackson</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -3934,17 +3934,17 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Alex Jackson</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -3955,24 +3955,24 @@
       <c r="E125" s="3" t="inlineStr"/>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -3983,24 +3983,24 @@
       <c r="E126" s="3" t="inlineStr"/>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Pavin Smith</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -4011,7 +4011,7 @@
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
@@ -4074,17 +4074,17 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Lourdes Gurriel Jr.</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
@@ -4095,7 +4095,7 @@
       <c r="E130" s="3" t="inlineStr"/>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>Nick Fortes</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -4158,7 +4158,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Nick Fortes</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -4186,7 +4186,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>Matt Shaw</t>
+          <t>Joe Mack</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -4242,7 +4242,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>Joe Mack</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -4270,17 +4270,17 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -4291,14 +4291,14 @@
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Matt Shaw</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -4326,7 +4326,7 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Jimmy Crooks</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -4354,7 +4354,7 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Crooks</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -4382,7 +4382,7 @@
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>Lourdes Gurriel Jr.</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -4410,17 +4410,17 @@
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
@@ -4431,7 +4431,7 @@
       <c r="E142" s="3" t="inlineStr"/>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
@@ -4466,17 +4466,17 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
@@ -4487,14 +4487,14 @@
       <c r="E144" s="3" t="inlineStr"/>
       <c r="F144" s="3" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Jacob Wilson</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -4520,37 +4520,37 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="inlineStr">
-        <is>
-          <t>Jacob Wilson</t>
-        </is>
-      </c>
-      <c r="B146" s="2" t="inlineStr">
-        <is>
-          <t>+940</t>
-        </is>
-      </c>
-      <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>9.6%</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E146" s="2" t="inlineStr"/>
-      <c r="F146" s="2" t="inlineStr">
-        <is>
-          <t>9.6%</t>
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>Nick Gonzales</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr"/>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Rodolfo Duran</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -4578,7 +4578,7 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Pavin Smith</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
@@ -4606,7 +4606,7 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -4634,17 +4634,17 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>Rodolfo Duran</t>
+          <t>Jared Triolo</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -4655,19 +4655,19 @@
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Colt Keith</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
@@ -4690,17 +4690,17 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>Gabriel Rincones Jr.</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -4711,7 +4711,7 @@
       <c r="E152" s="3" t="inlineStr"/>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
@@ -4723,12 +4723,12 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4739,7 +4739,7 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
@@ -4751,12 +4751,12 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -4767,14 +4767,14 @@
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Rincones Jr.</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -4802,7 +4802,7 @@
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Blaze Jordan</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
@@ -4830,17 +4830,17 @@
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>Blaze Jordan</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -4851,14 +4851,14 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -4886,17 +4886,17 @@
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>Zach McKinstry</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -4907,14 +4907,14 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>Austin Martin</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -4942,17 +4942,17 @@
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Zach McKinstry</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -4963,24 +4963,24 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Cody Freeman</t>
+          <t>Austin Martin</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4991,24 +4991,24 @@
       <c r="E162" s="3" t="inlineStr"/>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>Tommy Troy</t>
+          <t>Cody Freeman</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -5019,24 +5019,24 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
@@ -5047,24 +5047,24 @@
       <c r="E164" s="3" t="inlineStr"/>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Tommy Troy</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -5075,7 +5075,7 @@
       <c r="E165" s="3" t="inlineStr"/>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
@@ -5110,17 +5110,17 @@
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>Ben Williamson</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -5131,14 +5131,14 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>Will Wagner</t>
+          <t>Ben Williamson</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -5166,17 +5166,17 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>Christian Vazquez</t>
+          <t>Will Wagner</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
@@ -5187,14 +5187,14 @@
       <c r="E169" s="3" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>Xavier Edwards</t>
+          <t>Christian Vazquez</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -5278,17 +5278,17 @@
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Xavier Edwards</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>+1220</t>
+          <t>+1240</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>7.5%</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -5299,7 +5299,7 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>7.5%</t>
         </is>
       </c>
     </row>
@@ -5339,12 +5339,12 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1360</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -5355,24 +5355,24 @@
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>LuJames Groover</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1360</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -5383,19 +5383,19 @@
       <c r="E176" s="3" t="inlineStr"/>
       <c r="F176" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Jacob Young</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>+1360</t>
+          <t>+1380</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
@@ -5418,17 +5418,17 @@
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>Jacob Young</t>
+          <t>Jake Mangum</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1540</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -5439,24 +5439,24 @@
       <c r="E178" s="3" t="inlineStr"/>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.1%</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>Jake Mangum</t>
+          <t>Nasim Nunez</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>+1540</t>
+          <t>+1560</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -5467,24 +5467,24 @@
       <c r="E179" s="3" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.0%</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>Nasim Nunez</t>
+          <t>Nicky Lopez</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>+1560</t>
+          <t>+1640</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>5.7%</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -5494,34 +5494,6 @@
       </c>
       <c r="E180" s="3" t="inlineStr"/>
       <c r="F180" s="3" t="inlineStr">
-        <is>
-          <t>6.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="3" t="inlineStr">
-        <is>
-          <t>Nicky Lopez</t>
-        </is>
-      </c>
-      <c r="B181" s="3" t="inlineStr">
-        <is>
-          <t>+1640</t>
-        </is>
-      </c>
-      <c r="C181" s="3" t="inlineStr">
-        <is>
-          <t>5.7%</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E181" s="3" t="inlineStr"/>
-      <c r="F181" s="3" t="inlineStr">
         <is>
           <t>5.7%</t>
         </is>

</xml_diff>

<commit_message>
Update odds files - Wed Jun 17 16:03:08 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+232</t>
+          <t>+206</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>30.1%</t>
+          <t>32.7%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>30.1%</t>
+          <t>32.7%</t>
         </is>
       </c>
     </row>
@@ -551,12 +551,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>+260</t>
+          <t>+250</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>27.8%</t>
+          <t>28.6%</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -567,7 +567,7 @@
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>27.8%</t>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -607,12 +607,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>+288</t>
+          <t>+279</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -623,24 +623,24 @@
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.4%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Juan Soto</t>
+          <t>Yordan Alvarez</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+290</t>
+          <t>+288</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -651,24 +651,24 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Yordan Alvarez</t>
+          <t>Cal Raleigh</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>+290</t>
+          <t>+298</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.1%</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -679,19 +679,19 @@
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.1%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cal Raleigh</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>+298</t>
+          <t>+299</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -719,12 +719,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>+305</t>
+          <t>+303</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>24.7%</t>
+          <t>24.8%</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -735,7 +735,7 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>24.7%</t>
+          <t>24.8%</t>
         </is>
       </c>
     </row>
@@ -824,75 +824,75 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Wilyer Abreu</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>+327</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>23.4%</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>23.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Jac Caglianone</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>+328</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>23.4%</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>23.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Kyle Stowers</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>+331</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>23.2%</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>23.2%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Ian Happ</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>+338</t>
+          <t>+332</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Junior Caminero</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+339</t>
+          <t>+334</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.0%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Junior Caminero</t>
+          <t>Ian Happ</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+344</t>
+          <t>+338</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -959,7 +959,7 @@
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.8%</t>
         </is>
       </c>
     </row>
@@ -992,30 +992,30 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Christian Walker</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>+353</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>22.1%</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>22.1%</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>+349</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>22.3%</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>22.3%</t>
         </is>
       </c>
     </row>
@@ -1048,30 +1048,30 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>+353</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>22.1%</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>22.1%</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Jordan Walker</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>+358</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>21.8%</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Mark Vientos</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1162,17 +1162,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>+359</t>
+          <t>+363</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1183,24 +1183,24 @@
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.6%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Pete Alonso</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>+363</t>
+          <t>+365</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.5%</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1211,7 +1211,7 @@
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.5%</t>
         </is>
       </c>
     </row>
@@ -1246,17 +1246,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Francisco Alvarez</t>
+          <t>Mark Vientos</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>+370</t>
+          <t>+368</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1267,24 +1267,24 @@
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>+371</t>
+          <t>+370</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1295,7 +1295,7 @@
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>21.3%</t>
         </is>
       </c>
     </row>
@@ -1330,17 +1330,17 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>+379</t>
+          <t>+375</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1351,24 +1351,24 @@
       <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.1%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>+381</t>
+          <t>+376</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1379,24 +1379,24 @@
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>21.0%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>+383</t>
+          <t>+378</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1407,24 +1407,24 @@
       <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Dillon Dingler</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>+391</t>
+          <t>+379</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>+403</t>
+          <t>+383</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>+404</t>
+          <t>+403</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1491,19 +1491,19 @@
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>+405</t>
+          <t>+404</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1526,7 +1526,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1552,28 +1552,28 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>Miguel Vargas</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Bo Bichette</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>+406</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>19.8%</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>19.8%</t>
         </is>
@@ -1582,7 +1582,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1664,47 +1664,47 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Max Muncy (LAD)</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>+421</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>19.2%</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>19.2%</t>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Endy Rodriguez</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>+413</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Max Muncy (LAD)</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>+429</t>
+          <t>+418</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1715,47 +1715,47 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Endy Rodriguez</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>+430</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>18.9%</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>18.9%</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Riley Greene</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>+421</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Eugenio Suarez</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>+431</t>
+          <t>+432</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1778,17 +1778,17 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Eugenio Suarez</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>+432</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="3" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Kerry Carpenter</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>+435</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1827,19 +1827,19 @@
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>+446</t>
+          <t>+445</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -1860,56 +1860,56 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>George Springer</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>+446</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>18.3%</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>18.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Michael Massey</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>+448</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>18.2%</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>18.2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>Kerry Carpenter</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>+449</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>18.2%</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr"/>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>18.2%</t>
         </is>
@@ -1918,12 +1918,12 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+449</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -1946,17 +1946,17 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>+451</t>
+          <t>+450</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1967,19 +1967,19 @@
       <c r="E54" s="3" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>Spencer Horwitz</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>+452</t>
+          <t>+451</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -2002,12 +2002,12 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>+453</t>
+          <t>+452</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -2030,17 +2030,17 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>+456</t>
+          <t>+453</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2051,24 +2051,24 @@
       <c r="E57" s="3" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Dominic Canzone</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>+458</t>
+          <t>+453</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2079,24 +2079,24 @@
       <c r="E58" s="3" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Tyler Callihan</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>+459</t>
+          <t>+454</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2107,24 +2107,24 @@
       <c r="E59" s="3" t="inlineStr"/>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>+462</t>
+          <t>+456</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2135,24 +2135,24 @@
       <c r="E60" s="3" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>+464</t>
+          <t>+458</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2163,24 +2163,24 @@
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>+464</t>
+          <t>+459</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2191,24 +2191,24 @@
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Manny Machado</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>+468</t>
+          <t>+462</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2219,24 +2219,24 @@
       <c r="E63" s="3" t="inlineStr"/>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Austin Riley</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+464</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2247,24 +2247,24 @@
       <c r="E64" s="3" t="inlineStr"/>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Lars Nootbaar</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2275,19 +2275,19 @@
       <c r="E65" s="3" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>CJ Abrams</t>
+          <t>Austin Riley</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>+476</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -2338,17 +2338,17 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>+479</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2359,24 +2359,24 @@
       <c r="E68" s="3" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Tyler Callihan</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>+481</t>
+          <t>+478</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2387,24 +2387,24 @@
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>+482</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2415,24 +2415,24 @@
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+482</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2443,24 +2443,24 @@
       <c r="E71" s="3" t="inlineStr"/>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.2%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+482</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2471,33 +2471,33 @@
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr">
         <is>
+          <t>17.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Gunnar Henderson</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>+487</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
           <t>17.0%</t>
         </is>
       </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Fernando Tatis Jr.</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>+488</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>17.0%</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr"/>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr"/>
+      <c r="F73" s="3" t="inlineStr">
         <is>
           <t>17.0%</t>
         </is>
@@ -2506,12 +2506,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Isaac Paredes</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+489</t>
+          <t>+488</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -2532,56 +2532,56 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="3" t="inlineStr">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Jake Bauers</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>16.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>Randal Grichuk</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>+490</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>16.9%</t>
         </is>
       </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr"/>
-      <c r="F75" s="3" t="inlineStr">
-        <is>
-          <t>16.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>Jake Bauers</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>+490</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>16.9%</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr"/>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr"/>
+      <c r="F76" s="3" t="inlineStr">
         <is>
           <t>16.9%</t>
         </is>
@@ -2590,17 +2590,17 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Yandy Diaz</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>+496</t>
+          <t>+492</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -2611,24 +2611,24 @@
       <c r="E77" s="3" t="inlineStr"/>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Lane Thomas</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+496</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -2639,19 +2639,19 @@
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Lane Thomas</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>+499</t>
+          <t>+498</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -2672,103 +2672,103 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Jackson Merrill</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>+498</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr"/>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>Samuel Basallo</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B81" s="2" t="inlineStr">
         <is>
           <t>+499</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>16.7%</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr"/>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
         <is>
           <t>16.7%</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
-        <is>
-          <t>Gavin Sheets</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>+504</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="inlineStr">
-        <is>
-          <t>16.6%</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr"/>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>16.6%</t>
-        </is>
-      </c>
-    </row>
     <row r="82">
-      <c r="A82" s="3" t="inlineStr">
-        <is>
-          <t>Sal Stewart</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>+505</t>
-        </is>
-      </c>
-      <c r="C82" s="3" t="inlineStr">
-        <is>
-          <t>16.5%</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E82" s="3" t="inlineStr"/>
-      <c r="F82" s="3" t="inlineStr">
-        <is>
-          <t>16.5%</t>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>+499</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>+508</t>
+          <t>+499</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2779,24 +2779,24 @@
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>+509</t>
+          <t>+504</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2807,24 +2807,24 @@
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>+510</t>
+          <t>+505</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2835,24 +2835,24 @@
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>+511</t>
+          <t>+505</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2863,24 +2863,24 @@
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>+512</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -2891,24 +2891,24 @@
       <c r="E87" s="3" t="inlineStr"/>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Lars Nootbaar</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>+514</t>
+          <t>+510</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2919,24 +2919,24 @@
       <c r="E88" s="3" t="inlineStr"/>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+512</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2947,24 +2947,24 @@
       <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Jonathan Aranda</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>+525</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -2975,24 +2975,24 @@
       <c r="E90" s="3" t="inlineStr"/>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>+529</t>
+          <t>+526</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -3003,24 +3003,24 @@
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Rhys Hoskins</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>+538</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -3031,7 +3031,7 @@
       <c r="E92" s="3" t="inlineStr"/>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -3094,17 +3094,17 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Amed Rosario</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>+544</t>
+          <t>+538</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -3115,14 +3115,14 @@
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>Owen Caissie</t>
+          <t>Amed Rosario</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -3206,7 +3206,7 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -3234,17 +3234,17 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Nathaniel Lowe</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -3255,24 +3255,24 @@
       <c r="E100" s="3" t="inlineStr"/>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+554</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -3283,19 +3283,19 @@
       <c r="E101" s="3" t="inlineStr"/>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>+554</t>
+          <t>+555</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -3318,17 +3318,17 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>+555</t>
+          <t>+556</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -3339,24 +3339,24 @@
       <c r="E103" s="3" t="inlineStr"/>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Nathaniel Lowe</t>
+          <t>Owen Caissie</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>+557</t>
+          <t>+561</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
@@ -3367,7 +3367,7 @@
       <c r="E104" s="3" t="inlineStr"/>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
@@ -3379,12 +3379,12 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>+557</t>
+          <t>+561</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -3395,14 +3395,14 @@
       <c r="E105" s="3" t="inlineStr"/>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Jimmy Crooks</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -3430,12 +3430,12 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Dalton Rushing</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>+567</t>
+          <t>+565</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -3458,7 +3458,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -3486,7 +3486,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Jake Rogers</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -3514,12 +3514,12 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>+578</t>
+          <t>+581</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -3542,17 +3542,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Jake Rogers</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>+584</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -3563,7 +3563,7 @@
       <c r="E111" s="3" t="inlineStr"/>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
@@ -3598,17 +3598,17 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -3619,7 +3619,7 @@
       <c r="E113" s="3" t="inlineStr"/>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
@@ -3682,17 +3682,17 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>Matt Vierling</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+595</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -3703,7 +3703,7 @@
       <c r="E116" s="3" t="inlineStr"/>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
@@ -3738,12 +3738,12 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+599</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -3766,7 +3766,7 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -3822,17 +3822,17 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3843,24 +3843,24 @@
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
@@ -3871,14 +3871,14 @@
       <c r="E122" s="3" t="inlineStr"/>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Kevin McGonigle</t>
+          <t>Cole Carrigg</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -3906,17 +3906,17 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>Jimmy Crooks</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -3927,14 +3927,14 @@
       <c r="E124" s="3" t="inlineStr"/>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -3962,7 +3962,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Alejandro Kirk</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3990,17 +3990,17 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Alejandro Kirk</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -4011,7 +4011,7 @@
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
@@ -4046,7 +4046,7 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>Last Season HR</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -4102,17 +4102,17 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Spencer Steer</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -4123,7 +4123,7 @@
       <c r="E131" s="3" t="inlineStr"/>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4158,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -4214,7 +4214,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -4242,7 +4242,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Arias</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -4270,7 +4270,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Braden Montgomery</t>
+          <t>Matt Vierling</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -4298,7 +4298,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Braden Montgomery</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -4326,7 +4326,7 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Blaze Jordan</t>
+          <t>Last Season HR</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -4382,7 +4382,7 @@
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -4438,17 +4438,17 @@
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Blaze Jordan</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
@@ -4459,14 +4459,14 @@
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>Xander Bogaerts</t>
+          <t>Jose Tena</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -4494,7 +4494,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>Jose Tena</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -4550,7 +4550,7 @@
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -4578,7 +4578,7 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
@@ -4606,17 +4606,17 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Hao-Yu Lee</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -4627,14 +4627,14 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
@@ -4662,17 +4662,17 @@
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Eric Haase</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -4683,24 +4683,24 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -4711,24 +4711,24 @@
       <c r="E152" s="3" t="inlineStr"/>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>Miguel Amaya</t>
+          <t>Eric Haase</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4739,7 +4739,7 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Miguel Amaya</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
@@ -4830,17 +4830,17 @@
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>Anthony Volpe</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -4851,7 +4851,7 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
@@ -4886,7 +4886,7 @@
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Anthony Volpe</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -4914,7 +4914,7 @@
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Samad Taylor</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -4942,7 +4942,7 @@
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -4970,7 +4970,7 @@
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Jordan Lawlar</t>
+          <t>Jared Triolo</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -4998,7 +4998,7 @@
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>Samad Taylor</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -5026,7 +5026,7 @@
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -5054,7 +5054,7 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Marcelo Mayer</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
@@ -5082,7 +5082,7 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
@@ -5110,17 +5110,17 @@
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -5131,14 +5131,14 @@
       <c r="E167" s="3" t="inlineStr"/>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -5166,7 +5166,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -5194,17 +5194,17 @@
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -5215,14 +5215,14 @@
       <c r="E170" s="3" t="inlineStr"/>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Brett Sullivan</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -5250,17 +5250,17 @@
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>Brett Sullivan</t>
+          <t>Edwin Arroyo</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -5271,24 +5271,24 @@
       <c r="E172" s="3" t="inlineStr"/>
       <c r="F172" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Rincones Jr.</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -5299,24 +5299,24 @@
       <c r="E173" s="3" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>Hao-Yu Lee</t>
+          <t>Jordan Lawlar</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -5327,24 +5327,24 @@
       <c r="E174" s="3" t="inlineStr"/>
       <c r="F174" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -5355,24 +5355,24 @@
       <c r="E175" s="3" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>Edwin Arroyo</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -5383,24 +5383,24 @@
       <c r="E176" s="3" t="inlineStr"/>
       <c r="F176" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>Zack Short</t>
+          <t>Gabriel Rincones Jr.</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
@@ -5411,24 +5411,24 @@
       <c r="E177" s="3" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Luis Torrens</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -5439,14 +5439,14 @@
       <c r="E178" s="3" t="inlineStr"/>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>Denzer Guzman</t>
+          <t>Rob Refsnyder</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
@@ -5474,17 +5474,17 @@
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>Rob Refsnyder</t>
+          <t>Eli White</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
@@ -5495,24 +5495,24 @@
       <c r="E180" s="3" t="inlineStr"/>
       <c r="F180" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>Luis Torrens</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -5523,24 +5523,24 @@
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>Victor Mesa Jr.</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
@@ -5551,24 +5551,24 @@
       <c r="E182" s="3" t="inlineStr"/>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>Eli White</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -5579,24 +5579,24 @@
       <c r="E183" s="3" t="inlineStr"/>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Zack Short</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -5607,14 +5607,14 @@
       <c r="E184" s="3" t="inlineStr"/>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>Victor Mesa Jr.</t>
+          <t>Denzer Guzman</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
@@ -5670,17 +5670,17 @@
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Tyler Freeman</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
@@ -5691,24 +5691,24 @@
       <c r="E187" s="3" t="inlineStr"/>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>Tyler Freeman</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
@@ -5719,24 +5719,24 @@
       <c r="E188" s="3" t="inlineStr"/>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Rodolfo Duran</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
@@ -5747,24 +5747,24 @@
       <c r="E189" s="3" t="inlineStr"/>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
@@ -5775,24 +5775,24 @@
       <c r="E190" s="3" t="inlineStr"/>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>Trey Mancini</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
@@ -5803,7 +5803,7 @@
       <c r="E191" s="3" t="inlineStr"/>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
@@ -5838,7 +5838,7 @@
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Troy Johnston</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
@@ -5866,7 +5866,7 @@
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
@@ -5894,17 +5894,17 @@
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>Rodolfo Duran</t>
+          <t>Nico Hoerner</t>
         </is>
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -5915,14 +5915,14 @@
       <c r="E195" s="3" t="inlineStr"/>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.3%</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Joey Loperfido</t>
         </is>
       </c>
       <c r="B196" s="3" t="inlineStr">
@@ -5950,7 +5950,7 @@
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="B197" s="3" t="inlineStr">
@@ -6006,17 +6006,17 @@
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Trey Mancini</t>
         </is>
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
@@ -6027,14 +6027,14 @@
       <c r="E199" s="3" t="inlineStr"/>
       <c r="F199" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B200" s="3" t="inlineStr">
@@ -6062,17 +6062,17 @@
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
         <is>
-          <t>Yainer Diaz</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -6083,24 +6083,24 @@
       <c r="E201" s="3" t="inlineStr"/>
       <c r="F201" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="3" t="inlineStr">
         <is>
-          <t>Joey Loperfido</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D202" s="3" t="inlineStr">
@@ -6111,14 +6111,14 @@
       <c r="E202" s="3" t="inlineStr"/>
       <c r="F202" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
         <is>
-          <t>Alex Call</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B203" s="3" t="inlineStr">
@@ -6146,17 +6146,17 @@
     <row r="204">
       <c r="A204" s="3" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>John Rave</t>
         </is>
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D204" s="3" t="inlineStr">
@@ -6167,14 +6167,14 @@
       <c r="E204" s="3" t="inlineStr"/>
       <c r="F204" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
         <is>
-          <t>John Rave</t>
+          <t>Alex Call</t>
         </is>
       </c>
       <c r="B205" s="3" t="inlineStr">
@@ -6230,7 +6230,7 @@
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
         <is>
-          <t>Sandy Leon</t>
+          <t>Miguel Rojas</t>
         </is>
       </c>
       <c r="B207" s="3" t="inlineStr">
@@ -6258,17 +6258,17 @@
     <row r="208">
       <c r="A208" s="3" t="inlineStr">
         <is>
-          <t>Tommy Troy</t>
+          <t>Sandy Leon</t>
         </is>
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -6279,24 +6279,24 @@
       <c r="E208" s="3" t="inlineStr"/>
       <c r="F208" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
         <is>
-          <t>Petey Halpin</t>
+          <t>Colt Keith</t>
         </is>
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D209" s="3" t="inlineStr">
@@ -6307,7 +6307,7 @@
       <c r="E209" s="3" t="inlineStr"/>
       <c r="F209" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
@@ -6342,17 +6342,17 @@
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
         <is>
-          <t>Miguel Rojas</t>
+          <t>Petey Halpin</t>
         </is>
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D211" s="3" t="inlineStr">
@@ -6363,14 +6363,14 @@
       <c r="E211" s="3" t="inlineStr"/>
       <c r="F211" s="3" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="3" t="inlineStr">
         <is>
-          <t>Patrick Bailey</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="B212" s="3" t="inlineStr">
@@ -6398,17 +6398,17 @@
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Patrick Bailey</t>
         </is>
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D213" s="3" t="inlineStr">
@@ -6419,7 +6419,7 @@
       <c r="E213" s="3" t="inlineStr"/>
       <c r="F213" s="3" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
@@ -6454,12 +6454,12 @@
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
         <is>
-          <t>LuJames Groover</t>
+          <t>Jake Meyers</t>
         </is>
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C215" s="3" t="inlineStr">
@@ -6482,17 +6482,17 @@
     <row r="216">
       <c r="A216" s="3" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Esteury Ruiz</t>
         </is>
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
@@ -6503,24 +6503,24 @@
       <c r="E216" s="3" t="inlineStr"/>
       <c r="F216" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
         <is>
-          <t>Esteury Ruiz</t>
+          <t>Tommy Troy</t>
         </is>
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D217" s="3" t="inlineStr">
@@ -6531,24 +6531,24 @@
       <c r="E217" s="3" t="inlineStr"/>
       <c r="F217" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="3" t="inlineStr">
         <is>
-          <t>Colt Keith</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D218" s="3" t="inlineStr">
@@ -6559,14 +6559,14 @@
       <c r="E218" s="3" t="inlineStr"/>
       <c r="F218" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Cooper Pratt</t>
         </is>
       </c>
       <c r="B219" s="3" t="inlineStr">
@@ -6594,7 +6594,7 @@
     <row r="220">
       <c r="A220" s="3" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>LuJames Groover</t>
         </is>
       </c>
       <c r="B220" s="3" t="inlineStr">
@@ -6650,17 +6650,17 @@
     <row r="222">
       <c r="A222" s="3" t="inlineStr">
         <is>
-          <t>Cooper Pratt</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D222" s="3" t="inlineStr">
@@ -6671,14 +6671,14 @@
       <c r="E222" s="3" t="inlineStr"/>
       <c r="F222" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B223" s="3" t="inlineStr">
@@ -6706,7 +6706,7 @@
     <row r="224">
       <c r="A224" s="3" t="inlineStr">
         <is>
-          <t>Garrett Stubbs</t>
+          <t>Drew Gilbert</t>
         </is>
       </c>
       <c r="B224" s="3" t="inlineStr">
@@ -6734,7 +6734,7 @@
     <row r="225">
       <c r="A225" s="3" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Garrett Stubbs</t>
         </is>
       </c>
       <c r="B225" s="3" t="inlineStr">
@@ -6762,7 +6762,7 @@
     <row r="226">
       <c r="A226" s="3" t="inlineStr">
         <is>
-          <t>Justin Crawford</t>
+          <t>David Hamilton</t>
         </is>
       </c>
       <c r="B226" s="3" t="inlineStr">
@@ -6818,7 +6818,7 @@
     <row r="228">
       <c r="A228" s="3" t="inlineStr">
         <is>
-          <t>Drew Gilbert</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B228" s="3" t="inlineStr">
@@ -6846,17 +6846,17 @@
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Christian Vazquez</t>
         </is>
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -6867,14 +6867,14 @@
       <c r="E229" s="3" t="inlineStr"/>
       <c r="F229" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="3" t="inlineStr">
         <is>
-          <t>Jake Meyers</t>
+          <t>Justin Crawford</t>
         </is>
       </c>
       <c r="B230" s="3" t="inlineStr">
@@ -6958,7 +6958,7 @@
     <row r="233">
       <c r="A233" s="3" t="inlineStr">
         <is>
-          <t>Edgar Quero</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B233" s="3" t="inlineStr">
@@ -6986,7 +6986,7 @@
     <row r="234">
       <c r="A234" s="3" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Edgar Quero</t>
         </is>
       </c>
       <c r="B234" s="3" t="inlineStr">
@@ -7019,12 +7019,12 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -7035,14 +7035,14 @@
       <c r="E235" s="3" t="inlineStr"/>
       <c r="F235" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="3" t="inlineStr">
         <is>
-          <t>Myles Straw</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B236" s="3" t="inlineStr">
@@ -7070,7 +7070,7 @@
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Myles Straw</t>
         </is>
       </c>
       <c r="B237" s="3" t="inlineStr">
@@ -7098,7 +7098,7 @@
     <row r="238">
       <c r="A238" s="3" t="inlineStr">
         <is>
-          <t>Jose Trevino</t>
+          <t>Taylor Walls</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr">
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -7175,14 +7175,14 @@
       <c r="E240" s="3" t="inlineStr"/>
       <c r="F240" s="3" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.6%</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
         <is>
-          <t>Taylor Walls</t>
+          <t>Jose Trevino</t>
         </is>
       </c>
       <c r="B241" s="3" t="inlineStr">
@@ -7238,7 +7238,7 @@
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B243" s="3" t="inlineStr">
@@ -7266,17 +7266,17 @@
     <row r="244">
       <c r="A244" s="3" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1280</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.2%</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
@@ -7287,7 +7287,7 @@
       <c r="E244" s="3" t="inlineStr"/>
       <c r="F244" s="3" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
@@ -7322,7 +7322,7 @@
     <row r="246">
       <c r="A246" s="3" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B246" s="3" t="inlineStr">
@@ -7350,7 +7350,7 @@
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
         <is>
-          <t>Jacob Wilson</t>
+          <t>Luisangel Acuna</t>
         </is>
       </c>
       <c r="B247" s="3" t="inlineStr">
@@ -7378,7 +7378,7 @@
     <row r="248">
       <c r="A248" s="3" t="inlineStr">
         <is>
-          <t>Luisangel Acuna</t>
+          <t>Jacob Wilson</t>
         </is>
       </c>
       <c r="B248" s="3" t="inlineStr">
@@ -7406,17 +7406,17 @@
     <row r="249">
       <c r="A249" s="3" t="inlineStr">
         <is>
-          <t>Nasim Nunez</t>
+          <t>Chandler Simpson</t>
         </is>
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>+1440</t>
+          <t>+1400</t>
         </is>
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>6.7%</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
@@ -7427,24 +7427,24 @@
       <c r="E249" s="3" t="inlineStr"/>
       <c r="F249" s="3" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>6.7%</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="3" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Nasim Nunez</t>
         </is>
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>+1480</t>
+          <t>+1440</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="D250" s="3" t="inlineStr">
@@ -7455,24 +7455,24 @@
       <c r="E250" s="3" t="inlineStr"/>
       <c r="F250" s="3" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>6.5%</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="3" t="inlineStr">
         <is>
-          <t>Miles Mastrobuoni</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>+1500</t>
+          <t>+1480</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
@@ -7483,24 +7483,24 @@
       <c r="E251" s="3" t="inlineStr"/>
       <c r="F251" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.3%</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="3" t="inlineStr">
         <is>
-          <t>Chandler Simpson</t>
+          <t>Miles Mastrobuoni</t>
         </is>
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>+1540</t>
+          <t>+1500</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
@@ -7511,7 +7511,7 @@
       <c r="E252" s="3" t="inlineStr"/>
       <c r="F252" s="3" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.2%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun 18 14:12:13 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+210</t>
+          <t>+203</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>32.3%</t>
+          <t>33.0%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -511,7 +511,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>32.3%</t>
+          <t>33.0%</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>+269</t>
+          <t>+255</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>28.2%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Miguel Vargas</t>
+          <t>Randal Grichuk</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>+284</t>
+          <t>+279</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -623,24 +623,24 @@
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>26.4%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+287</t>
+          <t>+280</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.3%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -651,7 +651,7 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.3%</t>
         </is>
       </c>
     </row>
@@ -686,17 +686,17 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Randal Grichuk</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>+292</t>
+          <t>+293</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -707,24 +707,24 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.4%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Cal Raleigh</t>
+          <t>Nick Kurtz</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>+299</t>
+          <t>+300</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -735,24 +735,24 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Nick Kurtz</t>
+          <t>Cal Raleigh</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+307</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>24.6%</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -763,7 +763,7 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>24.6%</t>
         </is>
       </c>
     </row>
@@ -824,75 +824,75 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Cody Bellinger</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>+343</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>22.6%</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>22.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Kody Clemens</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>+332</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>23.1%</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>23.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Cody Bellinger</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>+340</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>22.7%</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>22.7%</t>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>+344</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>22.5%</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>+340</t>
+          <t>+348</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>22.7%</t>
+          <t>22.3%</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -903,7 +903,7 @@
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>22.7%</t>
+          <t>22.3%</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+344</t>
+          <t>+349</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.3%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.3%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+367</t>
+          <t>+352</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>22.1%</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -959,24 +959,24 @@
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Colson Montgomery</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>+372</t>
+          <t>+355</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -987,80 +987,80 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>22.0%</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Ryan McMahon</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>+380</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>20.8%</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>20.8%</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Gunnar Henderson</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>+379</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>20.9%</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Willson Contreras</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>+380</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>20.8%</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>20.8%</t>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pete Alonso</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>+386</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>20.6%</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>20.6%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Pete Alonso</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>+394</t>
+          <t>+390</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1071,24 +1071,24 @@
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Bobby Witt Jr.</t>
+          <t>Willson Contreras</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>+397</t>
+          <t>+390</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1099,52 +1099,52 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Gunnar Henderson</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>+399</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>20.0%</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Ryan McMahon</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>+395</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>20.2%</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Julio Rodriguez</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>+406</t>
+          <t>+401</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1155,14 +1155,14 @@
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Nelson Velazquez</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1190,12 +1190,12 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Spencer Jones</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>+408</t>
+          <t>+407</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1216,47 +1216,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Joc Pederson</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>+418</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>19.3%</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>19.3%</t>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>+409</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>19.6%</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Julio Rodriguez</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>+418</t>
+          <t>+420</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1267,7 +1267,7 @@
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
@@ -1300,42 +1300,42 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>+437</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>18.6%</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>18.6%</t>
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Joc Pederson</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>+432</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>18.8%</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Samuel Basallo</t>
+          <t>Bryce Harper</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+439</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1356,47 +1356,47 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Nelson Velazquez</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>+440</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>18.5%</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>18.5%</t>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Samuel Basallo</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>+439</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>+455</t>
+          <t>+447</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1407,24 +1407,24 @@
       <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>MJ Melendez</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>+457</t>
+          <t>+453</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>+455</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Dominic Canzone</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>+469</t>
+          <t>+459</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1491,24 +1491,24 @@
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>+469</t>
+          <t>+461</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1519,24 +1519,24 @@
       <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Everson Pereira</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1547,24 +1547,24 @@
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Royce Lewis</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1575,24 +1575,24 @@
       <c r="E40" s="3" t="inlineStr"/>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Francisco Alvarez</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+471</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1603,52 +1603,52 @@
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>+489</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>17.0%</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>17.0%</t>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Kazuma Okamoto</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>+474</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>17.4%</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>MJ Melendez</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+477</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1659,24 +1659,24 @@
       <c r="E43" s="3" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Everson Pereira</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+477</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Matt Olson</t>
+          <t>Gary Sanchez</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>+496</t>
+          <t>+484</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1715,24 +1715,24 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+484</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1743,14 +1743,14 @@
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Gary Sanchez</t>
+          <t>Matt Olson</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1806,17 +1806,17 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>+502</t>
+          <t>+500</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1827,33 +1827,33 @@
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr">
         <is>
+          <t>16.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Royce Lewis</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>+501</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
           <t>16.6%</t>
         </is>
       </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Salvador Perez</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>+503</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>16.6%</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr">
         <is>
           <t>16.6%</t>
         </is>
@@ -1862,17 +1862,17 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Luke Raley</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>+505</t>
+          <t>+503</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -1883,7 +1883,7 @@
       <c r="E51" s="3" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1918,17 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>+517</t>
+          <t>+507</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -1939,52 +1939,52 @@
       <c r="E53" s="3" t="inlineStr"/>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>Zack Gelof</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>+520</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>16.1%</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr"/>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>16.1%</t>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>+510</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>16.4%</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1995,24 +1995,24 @@
       <c r="E55" s="3" t="inlineStr"/>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Rhys Hoskins</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+520</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2023,24 +2023,24 @@
       <c r="E56" s="3" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+526</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -2051,14 +2051,14 @@
       <c r="E57" s="3" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.0%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -2086,12 +2086,12 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>+530</t>
+          <t>+529</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -2114,17 +2114,17 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>+535</t>
+          <t>+530</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2135,24 +2135,24 @@
       <c r="E60" s="3" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>+537</t>
+          <t>+531</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2163,47 +2163,47 @@
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>Alec Burleson</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>+537</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>15.7%</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr"/>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>15.7%</t>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>+533</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>+538</t>
+          <t>+537</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2226,17 +2226,17 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>+542</t>
+          <t>+537</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2247,19 +2247,19 @@
       <c r="E64" s="3" t="inlineStr"/>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>+546</t>
+          <t>+547</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -2282,17 +2282,17 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>+547</t>
+          <t>+549</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -2303,24 +2303,24 @@
       <c r="E66" s="3" t="inlineStr"/>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Jesus Sanchez</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+553</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2331,24 +2331,24 @@
       <c r="E67" s="3" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+555</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -2359,24 +2359,24 @@
       <c r="E68" s="3" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Braden Montgomery</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+555</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2387,24 +2387,24 @@
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>+562</t>
+          <t>+556</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2415,19 +2415,19 @@
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>+563</t>
+          <t>+562</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -2450,17 +2450,17 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>+566</t>
+          <t>+563</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2471,24 +2471,24 @@
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>+567</t>
+          <t>+564</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2499,19 +2499,19 @@
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>+568</t>
+          <t>+567</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -2534,7 +2534,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -2562,7 +2562,7 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Jesus Sanchez</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -2590,12 +2590,12 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Denzer Guzman</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+572</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -2618,12 +2618,12 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Denzer Guzman</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>+572</t>
+          <t>+573</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -2646,17 +2646,17 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Braden Montgomery</t>
+          <t>Andrew Vaughn</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>+573</t>
+          <t>+581</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -2667,24 +2667,24 @@
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>+578</t>
+          <t>+584</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -2695,24 +2695,24 @@
       <c r="E80" s="3" t="inlineStr"/>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Vaughn Grissom</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -2723,19 +2723,19 @@
       <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Edmundo Sosa</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>+583</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -2758,17 +2758,17 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Vaughn Grissom</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>+585</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2779,24 +2779,24 @@
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+593</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2807,14 +2807,14 @@
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -2842,17 +2842,17 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Edmundo Sosa</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2863,7 +2863,7 @@
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -2926,17 +2926,17 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2947,24 +2947,24 @@
       <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -2975,14 +2975,14 @@
       <c r="E90" s="3" t="inlineStr"/>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -3010,17 +3010,17 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -3031,7 +3031,7 @@
       <c r="E92" s="3" t="inlineStr"/>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
@@ -3043,12 +3043,12 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -3059,7 +3059,7 @@
       <c r="E93" s="3" t="inlineStr"/>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3071,12 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -3087,24 +3087,24 @@
       <c r="E94" s="3" t="inlineStr"/>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -3115,24 +3115,24 @@
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Austin Riley</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -3143,24 +3143,24 @@
       <c r="E96" s="3" t="inlineStr"/>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Austin Riley</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -3171,24 +3171,24 @@
       <c r="E97" s="3" t="inlineStr"/>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -3199,24 +3199,24 @@
       <c r="E98" s="3" t="inlineStr"/>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Lane Thomas</t>
+          <t>Starling Marte</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -3227,24 +3227,24 @@
       <c r="E99" s="3" t="inlineStr"/>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -3255,14 +3255,14 @@
       <c r="E100" s="3" t="inlineStr"/>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Starling Marte</t>
+          <t>Derek Hill</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -3290,7 +3290,7 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Lane Thomas</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -3318,7 +3318,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Kyle Higashioka</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -3374,7 +3374,7 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Kyle Higashioka</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -3402,7 +3402,7 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Connor Wong</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Arias</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -3458,17 +3458,17 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -3479,24 +3479,24 @@
       <c r="E108" s="3" t="inlineStr"/>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Derek Hill</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       <c r="E109" s="3" t="inlineStr"/>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
@@ -3542,17 +3542,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Blaze Jordan</t>
+          <t>Brandon Valenzuela</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -3563,24 +3563,24 @@
       <c r="E111" s="3" t="inlineStr"/>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>Brandon Valenzuela</t>
+          <t>Edgar Quero</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -3591,14 +3591,14 @@
       <c r="E112" s="3" t="inlineStr"/>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Blaze Jordan</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -3654,17 +3654,17 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -3675,14 +3675,14 @@
       <c r="E115" s="3" t="inlineStr"/>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>Edgar Quero</t>
+          <t>J.C. Escarra</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -3710,17 +3710,17 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>J.C. Escarra</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -3731,24 +3731,24 @@
       <c r="E117" s="3" t="inlineStr"/>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -3759,14 +3759,14 @@
       <c r="E118" s="3" t="inlineStr"/>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Pedro Pages</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -3794,17 +3794,17 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -3815,24 +3815,24 @@
       <c r="E120" s="3" t="inlineStr"/>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3843,14 +3843,14 @@
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -3878,17 +3878,17 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -3899,24 +3899,24 @@
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -3927,7 +3927,7 @@
       <c r="E124" s="3" t="inlineStr"/>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
@@ -3939,12 +3939,12 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -3955,24 +3955,24 @@
       <c r="E125" s="3" t="inlineStr"/>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -3983,14 +3983,14 @@
       <c r="E126" s="3" t="inlineStr"/>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Josh Smith</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -4018,7 +4018,7 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Andruw Monasterio</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
@@ -4046,7 +4046,7 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>Pedro Pages</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -4074,17 +4074,17 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>+910</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
@@ -4095,14 +4095,14 @@
       <c r="E130" s="3" t="inlineStr"/>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Josh Smith</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -4130,17 +4130,17 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
@@ -4151,24 +4151,24 @@
       <c r="E132" s="3" t="inlineStr"/>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Luisangel Acuna</t>
+          <t>Stuart Fairchild</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -4179,14 +4179,14 @@
       <c r="E133" s="3" t="inlineStr"/>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>Blaze Alexander</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -4214,7 +4214,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Luisangel Acuna</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -4242,12 +4242,12 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -4270,17 +4270,17 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Alejandro Osuna</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -4291,24 +4291,24 @@
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>Marcelo Mayer</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
@@ -4319,24 +4319,24 @@
       <c r="E138" s="3" t="inlineStr"/>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>Alejandro Osuna</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -4347,24 +4347,24 @@
       <c r="E139" s="3" t="inlineStr"/>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -4375,24 +4375,24 @@
       <c r="E140" s="3" t="inlineStr"/>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Blaze Alexander</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
@@ -4403,14 +4403,14 @@
       <c r="E141" s="3" t="inlineStr"/>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>Masataka Yoshida</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -4438,17 +4438,17 @@
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Daniel Susac</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
@@ -4459,24 +4459,24 @@
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>Stuart Fairchild</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
@@ -4487,7 +4487,7 @@
       <c r="E144" s="3" t="inlineStr"/>
       <c r="F144" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
@@ -4499,12 +4499,12 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
@@ -4515,14 +4515,14 @@
       <c r="E145" s="3" t="inlineStr"/>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -4550,17 +4550,17 @@
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Austin Hedges</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -4571,24 +4571,24 @@
       <c r="E147" s="3" t="inlineStr"/>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Blake Perkins</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
@@ -4599,7 +4599,7 @@
       <c r="E148" s="3" t="inlineStr"/>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
@@ -4611,12 +4611,12 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -4627,24 +4627,24 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>Austin Hedges</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -4655,24 +4655,24 @@
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -4683,24 +4683,24 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>Blake Perkins</t>
+          <t>David Hamilton</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -4711,7 +4711,7 @@
       <c r="E152" s="3" t="inlineStr"/>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
@@ -4723,12 +4723,12 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4739,24 +4739,24 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -4767,14 +4767,14 @@
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Isiah Kiner-Falefa</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -4858,17 +4858,17 @@
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>Isiah Kiner-Falefa</t>
+          <t>Jacob Wilson</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1300</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -4879,24 +4879,24 @@
       <c r="E158" s="3" t="inlineStr"/>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.1%</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>Jacob Wilson</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1380</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -4907,24 +4907,24 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+1520</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -4935,7 +4935,7 @@
       <c r="E160" s="3" t="inlineStr"/>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.2%</t>
         </is>
       </c>
     </row>
@@ -4947,12 +4947,12 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>+1500</t>
+          <t>+1580</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -4963,24 +4963,24 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.0%</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>+1520</t>
+          <t>+1600</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4991,7 +4991,7 @@
       <c r="E162" s="3" t="inlineStr"/>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>5.9%</t>
         </is>
       </c>
     </row>
@@ -5003,12 +5003,12 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>+1860</t>
+          <t>+2000</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -5019,7 +5019,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>4.8%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun 18 15:37:36 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -579,12 +579,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>+255</t>
+          <t>+259</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -595,52 +595,52 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>27.9%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Randal Grichuk</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>+279</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>26.4%</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>26.4%</t>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>+282</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>26.2%</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>26.2%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+280</t>
+          <t>+282</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>26.3%</t>
+          <t>26.2%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -651,24 +651,24 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>26.3%</t>
+          <t>26.2%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>+289</t>
+          <t>+282</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>26.2%</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -679,24 +679,24 @@
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>25.7%</t>
+          <t>26.2%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>+293</t>
+          <t>+289</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.7%</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -707,7 +707,7 @@
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.7%</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+290</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>25.6%</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -735,24 +735,24 @@
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>25.6%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Cal Raleigh</t>
+          <t>Mike Trout</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>+307</t>
+          <t>+309</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>24.6%</t>
+          <t>24.4%</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -763,24 +763,24 @@
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>24.6%</t>
+          <t>24.4%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Mike Trout</t>
+          <t>Cal Raleigh</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>+313</t>
+          <t>+316</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -791,7 +791,7 @@
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>24.0%</t>
         </is>
       </c>
     </row>
@@ -826,17 +826,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>+343</t>
+          <t>+327</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -847,80 +847,80 @@
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3" t="inlineStr">
         <is>
+          <t>23.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Jordan Walker</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>+343</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
           <t>22.6%</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>22.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Kody Clemens</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>+344</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>22.5%</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>22.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Colson Montgomery</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>+348</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>22.3%</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>22.3%</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>+347</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>22.4%</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+349</t>
+          <t>+350</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+352</t>
+          <t>+356</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.9%</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -959,24 +959,24 @@
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>+355</t>
+          <t>+356</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>21.9%</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>+379</t>
+          <t>+363</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1015,24 +1015,24 @@
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.6%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Pete Alonso</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>+386</t>
+          <t>+379</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1043,24 +1043,24 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>+390</t>
+          <t>+388</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1071,24 +1071,24 @@
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.5%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Willson Contreras</t>
+          <t>Ryan McMahon</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>+390</t>
+          <t>+395</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1099,80 +1099,80 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Ryan McMahon</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>+395</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>20.2%</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>20.2%</t>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Spencer Jones</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>+405</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Julio Rodriguez</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>+401</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>20.0%</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Willson Contreras</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>+408</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>19.7%</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>19.7%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Nelson Velazquez</t>
+          <t>Julio Rodriguez</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>+407</t>
+          <t>+413</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1183,24 +1183,24 @@
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>+407</t>
+          <t>+420</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1211,24 +1211,24 @@
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>19.2%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Bobby Witt Jr.</t>
+          <t>Nelson Velazquez</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>+409</t>
+          <t>+428</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1239,24 +1239,24 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Jasson Dominguez</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+429</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1267,24 +1267,24 @@
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Jasson Dominguez</t>
+          <t>Joc Pederson</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>+429</t>
+          <t>+432</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1295,61 +1295,61 @@
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>18.8%</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>Joc Pederson</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>+432</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>18.8%</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>18.8%</t>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Bryce Harper</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>+437</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Bryce Harper</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Dominic Canzone</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>+437</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>18.6%</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>18.6%</t>
         </is>
@@ -1384,47 +1384,47 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>George Springer</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>+447</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>18.3%</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>18.3%</t>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>+440</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>MJ Melendez</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>+453</t>
+          <t>+447</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Dominic Canzone</t>
+          <t>MJ Melendez</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>+455</t>
+          <t>+453</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1463,7 +1463,7 @@
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
@@ -1582,17 +1582,17 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Luke Raley</t>
+          <t>Matt Olson</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>+471</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1603,19 +1603,19 @@
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Everson Pereira</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+479</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -1666,17 +1666,17 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Everson Pereira</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+486</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Gary Sanchez</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+495</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1715,24 +1715,24 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+500</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1743,19 +1743,19 @@
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Matt Olson</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>+499</t>
+          <t>+500</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1778,17 +1778,17 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Royce Lewis</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+501</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="3" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Francisco Alvarez</t>
+          <t>Gary Sanchez</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+501</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1827,14 +1827,14 @@
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Royce Lewis</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1862,12 +1862,12 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Rhys Hoskins</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>+503</t>
+          <t>+504</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -1918,17 +1918,17 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>+507</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -1939,42 +1939,42 @@
       <c r="E53" s="3" t="inlineStr"/>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.4%</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Salvador Perez</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>+510</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>16.4%</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>16.4%</t>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Oswald Peraza</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>+519</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Zack Gelof</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -2002,12 +2002,12 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>Zack Gelof</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+523</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -2030,7 +2030,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -2058,17 +2058,17 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Josh Naylor</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>+529</t>
+          <t>+526</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2079,33 +2079,33 @@
       <c r="E58" s="3" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr">
         <is>
+          <t>16.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>+528</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
           <t>15.9%</t>
         </is>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>Oswald Peraza</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>+529</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>15.9%</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr"/>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>15.9%</t>
         </is>
@@ -2114,12 +2114,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>+530</t>
+          <t>+529</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2142,17 +2142,17 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>+531</t>
+          <t>+530</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2163,33 +2163,33 @@
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3" t="inlineStr">
         <is>
+          <t>15.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Brett Baty</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>+531</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
           <t>15.8%</t>
         </is>
       </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>+533</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>15.8%</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr"/>
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>15.8%</t>
         </is>
@@ -2198,17 +2198,17 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Braden Montgomery</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>+537</t>
+          <t>+533</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2219,24 +2219,24 @@
       <c r="E63" s="3" t="inlineStr"/>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>+537</t>
+          <t>+541</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2247,24 +2247,24 @@
       <c r="E64" s="3" t="inlineStr"/>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>+547</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -2275,33 +2275,33 @@
       <c r="E65" s="3" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>Colton Cowser</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>+549</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>15.4%</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr"/>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>15.4%</t>
         </is>
@@ -2310,17 +2310,17 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Jesus Sanchez</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>+553</t>
+          <t>+549</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2331,19 +2331,19 @@
       <c r="E67" s="3" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>Jesus Sanchez</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>+555</t>
+          <t>+553</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -2366,7 +2366,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Braden Montgomery</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+557</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -2422,17 +2422,17 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>+562</t>
+          <t>+558</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2443,19 +2443,19 @@
       <c r="E71" s="3" t="inlineStr"/>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>+563</t>
+          <t>+562</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -2478,12 +2478,12 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>+564</t>
+          <t>+563</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -2534,17 +2534,17 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+568</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2555,7 +2555,7 @@
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
@@ -2590,17 +2590,17 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Denzer Guzman</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>+572</t>
+          <t>+577</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -2611,24 +2611,24 @@
       <c r="E77" s="3" t="inlineStr"/>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Vaughn Grissom</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>+573</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -2639,24 +2639,24 @@
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Edmundo Sosa</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -2667,19 +2667,19 @@
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>+584</t>
+          <t>+586</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -2702,12 +2702,12 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Vaughn Grissom</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>+585</t>
+          <t>+587</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -2730,17 +2730,17 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Edmundo Sosa</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>+585</t>
+          <t>+588</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -2751,19 +2751,19 @@
       <c r="E82" s="3" t="inlineStr"/>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Denzer Guzman</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>+592</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -2791,12 +2791,12 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>+593</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2807,24 +2807,24 @@
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+594</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2835,24 +2835,24 @@
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+596</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2863,24 +2863,24 @@
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+599</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -2891,24 +2891,24 @@
       <c r="E87" s="3" t="inlineStr"/>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+599</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2919,24 +2919,24 @@
       <c r="E88" s="3" t="inlineStr"/>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Andrew Vaughn</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2947,24 +2947,24 @@
       <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -2975,24 +2975,24 @@
       <c r="E90" s="3" t="inlineStr"/>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -3003,24 +3003,24 @@
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -3031,24 +3031,24 @@
       <c r="E92" s="3" t="inlineStr"/>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>David Fry</t>
+          <t>Tristan Gray</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -3059,24 +3059,24 @@
       <c r="E93" s="3" t="inlineStr"/>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>Tristan Gray</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -3087,7 +3087,7 @@
       <c r="E94" s="3" t="inlineStr"/>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
@@ -3099,12 +3099,12 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -3115,24 +3115,24 @@
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>Austin Riley</t>
+          <t>David Fry</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -3143,14 +3143,14 @@
       <c r="E96" s="3" t="inlineStr"/>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -3178,17 +3178,17 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Austin Riley</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -3199,24 +3199,24 @@
       <c r="E98" s="3" t="inlineStr"/>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Starling Marte</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -3227,14 +3227,14 @@
       <c r="E99" s="3" t="inlineStr"/>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Lane Thomas</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -3262,7 +3262,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Derek Hill</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -3290,7 +3290,7 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Lane Thomas</t>
+          <t>Derek Hill</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -3318,17 +3318,17 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+720</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -3339,24 +3339,24 @@
       <c r="E103" s="3" t="inlineStr"/>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.2%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+730</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
@@ -3367,14 +3367,14 @@
       <c r="E104" s="3" t="inlineStr"/>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.0%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Kyle Higashioka</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -3402,7 +3402,7 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Connor Wong</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Brandon Valenzuela</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -3486,17 +3486,17 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Kyle Higashioka</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -3507,14 +3507,14 @@
       <c r="E109" s="3" t="inlineStr"/>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Starling Marte</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -3542,7 +3542,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Brandon Valenzuela</t>
+          <t>Edgar Quero</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
@@ -3570,17 +3570,17 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>Edgar Quero</t>
+          <t>J.C. Escarra</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -3591,24 +3591,24 @@
       <c r="E112" s="3" t="inlineStr"/>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Blaze Jordan</t>
+          <t>Pedro Pages</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -3619,24 +3619,24 @@
       <c r="E113" s="3" t="inlineStr"/>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -3647,24 +3647,24 @@
       <c r="E114" s="3" t="inlineStr"/>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -3675,24 +3675,24 @@
       <c r="E115" s="3" t="inlineStr"/>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>J.C. Escarra</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -3703,24 +3703,24 @@
       <c r="E116" s="3" t="inlineStr"/>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Blaze Jordan</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -3731,24 +3731,24 @@
       <c r="E117" s="3" t="inlineStr"/>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -3759,24 +3759,24 @@
       <c r="E118" s="3" t="inlineStr"/>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>Pedro Pages</t>
+          <t>Colt Emerson</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -3787,24 +3787,24 @@
       <c r="E119" s="3" t="inlineStr"/>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Connor Wong</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -3815,24 +3815,24 @@
       <c r="E120" s="3" t="inlineStr"/>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Colt Emerson</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+820</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3843,24 +3843,24 @@
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Andruw Monasterio</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+830</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
@@ -3871,24 +3871,24 @@
       <c r="E122" s="3" t="inlineStr"/>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.8%</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+840</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -3899,24 +3899,24 @@
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -3927,14 +3927,14 @@
       <c r="E124" s="3" t="inlineStr"/>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -3962,17 +3962,17 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -3983,24 +3983,24 @@
       <c r="E126" s="3" t="inlineStr"/>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -4011,24 +4011,24 @@
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>Andruw Monasterio</t>
+          <t>Josh Smith</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
@@ -4039,24 +4039,24 @@
       <c r="E128" s="3" t="inlineStr"/>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
@@ -4067,14 +4067,14 @@
       <c r="E129" s="3" t="inlineStr"/>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -4102,17 +4102,17 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>Josh Smith</t>
+          <t>Stuart Fairchild</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -4123,14 +4123,14 @@
       <c r="E131" s="3" t="inlineStr"/>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.7%</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Luisangel Acuna</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -4158,17 +4158,17 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Stuart Fairchild</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -4179,24 +4179,24 @@
       <c r="E133" s="3" t="inlineStr"/>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
@@ -4207,24 +4207,24 @@
       <c r="E134" s="3" t="inlineStr"/>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>Luisangel Acuna</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="E135" s="3" t="inlineStr"/>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.5%</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
@@ -4263,19 +4263,19 @@
       <c r="E136" s="3" t="inlineStr"/>
       <c r="F136" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -4298,7 +4298,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -4326,7 +4326,7 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Alejandro Osuna</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -4354,17 +4354,17 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -4375,14 +4375,14 @@
       <c r="E140" s="3" t="inlineStr"/>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>Blaze Alexander</t>
+          <t>Alejandro Osuna</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -4410,17 +4410,17 @@
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
@@ -4431,24 +4431,24 @@
       <c r="E142" s="3" t="inlineStr"/>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Blaze Alexander</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
@@ -4459,14 +4459,14 @@
       <c r="E143" s="3" t="inlineStr"/>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Victor Robles</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -4494,17 +4494,17 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>Victor Robles</t>
+          <t>Daniel Susac</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1040</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
@@ -4515,7 +4515,7 @@
       <c r="E145" s="3" t="inlineStr"/>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
@@ -4583,12 +4583,12 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
@@ -4599,24 +4599,24 @@
       <c r="E148" s="3" t="inlineStr"/>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -4627,7 +4627,7 @@
       <c r="E149" s="3" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
@@ -4639,12 +4639,12 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -4655,24 +4655,24 @@
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -4683,7 +4683,7 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
@@ -4695,12 +4695,12 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -4711,7 +4711,7 @@
       <c r="E152" s="3" t="inlineStr"/>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
@@ -4723,12 +4723,12 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1140</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4739,7 +4739,7 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
@@ -4751,12 +4751,12 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1160</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -4767,7 +4767,7 @@
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>Ha-Seong Kim</t>
+          <t>Jacob Wilson</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
@@ -4835,12 +4835,12 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>+1240</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -4851,24 +4851,24 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.0%</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>Jacob Wilson</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1340</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -4879,14 +4879,14 @@
       <c r="E158" s="3" t="inlineStr"/>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.9%</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Ha-Seong Kim</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -4914,17 +4914,17 @@
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>+1520</t>
+          <t>+1480</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -4935,7 +4935,7 @@
       <c r="E160" s="3" t="inlineStr"/>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.3%</t>
         </is>
       </c>
     </row>
@@ -4970,17 +4970,17 @@
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>+1600</t>
+          <t>+1620</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4991,7 +4991,7 @@
       <c r="E162" s="3" t="inlineStr"/>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.8%</t>
         </is>
       </c>
     </row>
@@ -5003,12 +5003,12 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>+2000</t>
+          <t>+1780</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>5.3%</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -5019,7 +5019,7 @@
       <c r="E163" s="3" t="inlineStr"/>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>5.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Thu Jun 18 16:26:22 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -579,12 +579,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>+259</t>
+          <t>+263</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>27.5%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -595,52 +595,52 @@
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>27.5%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Randal Grichuk</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>+282</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>26.2%</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>26.2%</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Byron Buxton</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>+285</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>26.0%</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>26.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Shea Langeliers</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>+282</t>
+          <t>+289</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>25.7%</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -651,24 +651,24 @@
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>25.7%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>Shea Langeliers</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>+282</t>
+          <t>+289</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>25.7%</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -679,35 +679,35 @@
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>25.7%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Jazz Chisholm</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>+289</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>25.7%</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>25.7%</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Randal Grichuk</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>+290</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>25.6%</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>25.6%</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>+309</t>
+          <t>+310</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>+316</t>
+          <t>+317</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>+327</t>
+          <t>+324</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -847,19 +847,19 @@
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.6%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Cody Bellinger</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>+343</t>
+          <t>+342</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -880,47 +880,47 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>+347</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>22.4%</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>22.4%</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Jordan Walker</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>+343</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>22.6%</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>22.6%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+344</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Colson Montgomery</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>+356</t>
+          <t>+346</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -959,52 +959,52 @@
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Colson Montgomery</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>+356</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>21.9%</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>21.9%</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>+347</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>22.4%</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>+363</t>
+          <t>+361</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1015,108 +1015,108 @@
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.7%</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Gunnar Henderson</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Willson Contreras</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>+373</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>21.1%</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>21.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Ryan McMahon</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>+377</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>21.0%</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>21.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Pete Alonso</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>+379</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>20.9%</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>20.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Pete Alonso</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>+388</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>20.5%</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>20.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Ryan McMahon</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>+395</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>20.2%</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>+405</t>
+          <t>+384</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1127,61 +1127,61 @@
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3" t="inlineStr">
         <is>
+          <t>20.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Spencer Jones</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>+405</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
           <t>19.8%</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Willson Contreras</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>+408</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>19.7%</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>19.7%</t>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>19.8%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Julio Rodriguez</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>+413</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Jake Bauers</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>+414</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>19.5%</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>19.5%</t>
         </is>
@@ -1190,17 +1190,17 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Jasson Dominguez</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+414</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1211,52 +1211,52 @@
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Nelson Velazquez</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>+428</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>18.9%</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>18.9%</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>MJ Melendez</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>+424</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>19.1%</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Jasson Dominguez</t>
+          <t>Julio Rodriguez</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>+429</t>
+          <t>+425</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1267,89 +1267,89 @@
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
         <is>
+          <t>19.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Nelson Velazquez</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>+428</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>18.9%</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>18.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Joc Pederson</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>+432</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>18.8%</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>18.8%</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Bryce Harper</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>+437</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>18.6%</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>18.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Dominic Canzone</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>+437</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>18.6%</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>18.6%</t>
         </is>
@@ -1384,47 +1384,47 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Bobby Witt Jr.</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>+440</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>18.5%</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>18.5%</t>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>George Springer</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>+447</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>18.3%</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>George Springer</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>+447</t>
+          <t>+449</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>MJ Melendez</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>+453</t>
+          <t>+459</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1463,14 +1463,14 @@
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Dominic Canzone</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1496,47 +1496,47 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Jose Siri</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>+461</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>17.8%</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>17.8%</t>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Bobby Witt Jr.</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>17.9%</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>+469</t>
+          <t>+461</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1547,14 +1547,14 @@
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Logan O'Hoppe</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1582,17 +1582,17 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Matt Olson</t>
+          <t>Logan O'Hoppe</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>+476</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1603,24 +1603,24 @@
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Everson Pereira</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>+476</t>
+          <t>+469</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1631,24 +1631,24 @@
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>+479</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1659,24 +1659,24 @@
       <c r="E43" s="3" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.5%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Luke Raley</t>
+          <t>Everson Pereira</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>+486</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="3" t="inlineStr"/>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Luke Raley</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>+495</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1715,24 +1715,24 @@
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>Francisco Alvarez</t>
+          <t>Matt Olson</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+492</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1743,14 +1743,14 @@
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1806,7 +1806,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Gary Sanchez</t>
+          <t>Tyler Soderstrom</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1834,12 +1834,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Tyler Soderstrom</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>+501</t>
+          <t>+504</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -1862,17 +1862,17 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>JJ Wetherholt</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>+504</t>
+          <t>+505</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -1883,7 +1883,7 @@
       <c r="E51" s="3" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1918,17 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Jesus Sanchez</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>+508</t>
+          <t>+507</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -1939,24 +1939,24 @@
       <c r="E53" s="3" t="inlineStr"/>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.5%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Oswald Peraza</t>
+          <t>Brett Baty</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>+519</t>
+          <t>+513</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1967,35 +1967,35 @@
       <c r="E54" s="3" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr">
         <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>+518</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
           <t>16.2%</t>
         </is>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>Rhys Hoskins</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>+520</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>16.1%</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr"/>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>16.1%</t>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
@@ -2030,12 +2030,12 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Matt Chapman</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+524</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -2058,7 +2058,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Josh Naylor</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -2084,28 +2084,28 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Salvador Perez</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Adley Rutschman</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>+528</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>15.9%</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>15.9%</t>
         </is>
@@ -2114,12 +2114,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>+529</t>
+          <t>+530</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2142,17 +2142,17 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Oswald Peraza</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>+530</t>
+          <t>+541</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2163,24 +2163,24 @@
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Brett Baty</t>
+          <t>Gary Sanchez</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>+531</t>
+          <t>+542</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2191,24 +2191,24 @@
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Braden Montgomery</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+543</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2219,24 +2219,24 @@
       <c r="E63" s="3" t="inlineStr"/>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>+541</t>
+          <t>+549</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -2247,61 +2247,61 @@
       <c r="E64" s="3" t="inlineStr"/>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>Brooks Lee</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>+548</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>15.4%</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr"/>
-      <c r="F65" s="3" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Jac Caglianone</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>+549</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Josh Naylor</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>15.4%</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr"/>
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>15.4%</t>
         </is>
@@ -2310,17 +2310,17 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Colton Cowser</t>
+          <t>Matt Chapman</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>+549</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2331,19 +2331,19 @@
       <c r="E67" s="3" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Jesus Sanchez</t>
+          <t>Braden Montgomery</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>+553</t>
+          <t>+552</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -2366,17 +2366,17 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>+555</t>
+          <t>+562</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2387,24 +2387,24 @@
       <c r="E69" s="3" t="inlineStr"/>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>+557</t>
+          <t>+563</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2415,24 +2415,24 @@
       <c r="E70" s="3" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>+558</t>
+          <t>+567</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2443,24 +2443,24 @@
       <c r="E71" s="3" t="inlineStr"/>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>+562</t>
+          <t>+567</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2471,24 +2471,24 @@
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>+563</t>
+          <t>+568</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2499,19 +2499,19 @@
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>+567</t>
+          <t>+568</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -2534,17 +2534,17 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Vladimir Guerrero Jr.</t>
+          <t>Trea Turner</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>+568</t>
+          <t>+570</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2555,19 +2555,19 @@
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Trea Turner</t>
+          <t>Ceddanne Rafaela</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+571</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -2590,17 +2590,17 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Rafael Devers</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>+577</t>
+          <t>+573</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -2611,24 +2611,24 @@
       <c r="E77" s="3" t="inlineStr"/>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Vaughn Grissom</t>
+          <t>David Fry</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>+585</t>
+          <t>+574</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -2639,24 +2639,24 @@
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Edmundo Sosa</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>+585</t>
+          <t>+577</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -2667,24 +2667,24 @@
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>+586</t>
+          <t>+580</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -2695,24 +2695,24 @@
       <c r="E80" s="3" t="inlineStr"/>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+580</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -2723,24 +2723,24 @@
       <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Wyatt Langford</t>
+          <t>Edmundo Sosa</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>+588</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -2751,24 +2751,24 @@
       <c r="E82" s="3" t="inlineStr"/>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Denzer Guzman</t>
+          <t>Vaughn Grissom</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -2779,24 +2779,24 @@
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>+592</t>
+          <t>+586</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -2807,24 +2807,24 @@
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Ceddanne Rafaela</t>
+          <t>Wyatt Langford</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>+594</t>
+          <t>+588</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -2835,24 +2835,24 @@
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Denzer Guzman</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>+596</t>
+          <t>+590</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2863,24 +2863,24 @@
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Brandon Marsh</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -2891,24 +2891,24 @@
       <c r="E87" s="3" t="inlineStr"/>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Yohendrick Pinango</t>
+          <t>Andrew Vaughn</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2919,24 +2919,24 @@
       <c r="E88" s="3" t="inlineStr"/>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Andrew Vaughn</t>
+          <t>Lawrence Butler</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
@@ -2947,14 +2947,14 @@
       <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Brandon Marsh</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -2982,17 +2982,17 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Lawrence Butler</t>
+          <t>Rafael Devers</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -3003,24 +3003,24 @@
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -3031,24 +3031,24 @@
       <c r="E92" s="3" t="inlineStr"/>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Tristan Gray</t>
+          <t>Yohendrick Pinango</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -3059,14 +3059,14 @@
       <c r="E93" s="3" t="inlineStr"/>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Tristan Gray</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -3094,17 +3094,17 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -3115,24 +3115,24 @@
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>David Fry</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
@@ -3143,24 +3143,24 @@
       <c r="E96" s="3" t="inlineStr"/>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -3171,24 +3171,24 @@
       <c r="E97" s="3" t="inlineStr"/>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>Austin Riley</t>
+          <t>Jose Caballero</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -3199,7 +3199,7 @@
       <c r="E98" s="3" t="inlineStr"/>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
     </row>
@@ -3211,12 +3211,12 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -3227,24 +3227,24 @@
       <c r="E99" s="3" t="inlineStr"/>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>Lane Thomas</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -3255,24 +3255,24 @@
       <c r="E100" s="3" t="inlineStr"/>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Austin Riley</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+690</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -3283,24 +3283,24 @@
       <c r="E101" s="3" t="inlineStr"/>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>Derek Hill</t>
+          <t>Kahlil Watson</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
@@ -3311,24 +3311,24 @@
       <c r="E102" s="3" t="inlineStr"/>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -3339,24 +3339,24 @@
       <c r="E103" s="3" t="inlineStr"/>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Lane Thomas</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
@@ -3367,24 +3367,24 @@
       <c r="E104" s="3" t="inlineStr"/>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Derek Hill</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
@@ -3395,14 +3395,14 @@
       <c r="E105" s="3" t="inlineStr"/>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -3458,7 +3458,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Gabriel Arias</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -3486,7 +3486,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>Kyle Higashioka</t>
+          <t>J.C. Escarra</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -3514,7 +3514,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>Starling Marte</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -3570,17 +3570,17 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>J.C. Escarra</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -3591,24 +3591,24 @@
       <c r="E112" s="3" t="inlineStr"/>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.8%</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Pedro Pages</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+760</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -3619,24 +3619,24 @@
       <c r="E113" s="3" t="inlineStr"/>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.6%</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Starling Marte</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -3647,14 +3647,14 @@
       <c r="E114" s="3" t="inlineStr"/>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>11.5%</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Kyle Higashioka</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -3682,17 +3682,17 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+780</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -3703,24 +3703,24 @@
       <c r="E116" s="3" t="inlineStr"/>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.4%</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>Blaze Jordan</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+790</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -3731,24 +3731,24 @@
       <c r="E117" s="3" t="inlineStr"/>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Connor Wong</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -3759,7 +3759,7 @@
       <c r="E118" s="3" t="inlineStr"/>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
@@ -3771,12 +3771,12 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -3787,24 +3787,24 @@
       <c r="E119" s="3" t="inlineStr"/>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>Connor Wong</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+800</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -3815,24 +3815,24 @@
       <c r="E120" s="3" t="inlineStr"/>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Blaze Jordan</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -3843,24 +3843,24 @@
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Andruw Monasterio</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
@@ -3871,24 +3871,24 @@
       <c r="E122" s="3" t="inlineStr"/>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Pedro Pages</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -3899,24 +3899,24 @@
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Andruw Monasterio</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+810</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
@@ -3927,24 +3927,24 @@
       <c r="E124" s="3" t="inlineStr"/>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -3955,24 +3955,24 @@
       <c r="E125" s="3" t="inlineStr"/>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Maikel Garcia</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
@@ -3983,24 +3983,24 @@
       <c r="E126" s="3" t="inlineStr"/>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Maikel Garcia</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
@@ -4011,7 +4011,7 @@
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
@@ -4023,12 +4023,12 @@
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
@@ -4039,24 +4039,24 @@
       <c r="E128" s="3" t="inlineStr"/>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>Masyn Winn</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
@@ -4067,14 +4067,14 @@
       <c r="E129" s="3" t="inlineStr"/>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>Dominic Smith</t>
+          <t>Cooper Pratt</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -4102,17 +4102,17 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>Stuart Fairchild</t>
+          <t>Masyn Winn</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -4123,14 +4123,14 @@
       <c r="E131" s="3" t="inlineStr"/>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>Luisangel Acuna</t>
+          <t>Dominic Smith</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -4158,17 +4158,17 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -4179,24 +4179,24 @@
       <c r="E133" s="3" t="inlineStr"/>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Blaze Alexander</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
@@ -4207,24 +4207,24 @@
       <c r="E134" s="3" t="inlineStr"/>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Brayan Rocchio</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -4235,24 +4235,24 @@
       <c r="E135" s="3" t="inlineStr"/>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+970</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
@@ -4263,19 +4263,19 @@
       <c r="E136" s="3" t="inlineStr"/>
       <c r="F136" s="3" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.3%</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+980</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -4303,12 +4303,12 @@
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
@@ -4319,24 +4319,24 @@
       <c r="E138" s="3" t="inlineStr"/>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>Luisangel Acuna</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+990</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -4347,24 +4347,24 @@
       <c r="E139" s="3" t="inlineStr"/>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Alejandro Osuna</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>+990</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -4375,14 +4375,14 @@
       <c r="E140" s="3" t="inlineStr"/>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>Alejandro Osuna</t>
+          <t>Stuart Fairchild</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -4438,7 +4438,7 @@
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>Blaze Alexander</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
@@ -4466,7 +4466,7 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>Victor Robles</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -4494,7 +4494,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>Daniel Susac</t>
+          <t>Austin Hedges</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -4522,7 +4522,7 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -4550,17 +4550,17 @@
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>Austin Hedges</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -4571,24 +4571,24 @@
       <c r="E147" s="3" t="inlineStr"/>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>Blake Perkins</t>
+          <t>Daniel Susac</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1080</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
@@ -4599,14 +4599,14 @@
       <c r="E148" s="3" t="inlineStr"/>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.5%</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Blake Perkins</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -4634,7 +4634,7 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Nick Loftin</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
@@ -4662,17 +4662,17 @@
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>Nick Loftin</t>
+          <t>Victor Robles</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -4683,24 +4683,24 @@
       <c r="E151" s="3" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>David Hamilton</t>
+          <t>Isiah Kiner-Falefa</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1100</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -4711,24 +4711,24 @@
       <c r="E152" s="3" t="inlineStr"/>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.3%</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>Joey Ortiz</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -4739,24 +4739,24 @@
       <c r="E153" s="3" t="inlineStr"/>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1120</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -4767,24 +4767,24 @@
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.2%</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>Isiah Kiner-Falefa</t>
+          <t>Joey Ortiz</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
@@ -4795,7 +4795,7 @@
       <c r="E155" s="3" t="inlineStr"/>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
@@ -4830,17 +4830,17 @@
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>Nick Madrigal</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1240</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>7.5%</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -4851,24 +4851,24 @@
       <c r="E157" s="3" t="inlineStr"/>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>7.0%</t>
+          <t>7.5%</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>Mauricio Dubon</t>
+          <t>Nick Madrigal</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -4879,24 +4879,24 @@
       <c r="E158" s="3" t="inlineStr"/>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.0%</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>Ha-Seong Kim</t>
+          <t>Mauricio Dubon</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1340</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -4907,24 +4907,24 @@
       <c r="E159" s="3" t="inlineStr"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.9%</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>Jung Hoo Lee</t>
+          <t>Ha-Seong Kim</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>+1480</t>
+          <t>+1440</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
@@ -4935,24 +4935,24 @@
       <c r="E160" s="3" t="inlineStr"/>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>6.5%</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>Drew Gilbert</t>
+          <t>Jung Hoo Lee</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>+1580</t>
+          <t>+1480</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
@@ -4963,24 +4963,24 @@
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.3%</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Drew Gilbert</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>+1620</t>
+          <t>+1680</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
@@ -4991,7 +4991,7 @@
       <c r="E162" s="3" t="inlineStr"/>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>5.6%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Fri Jun 19 03:49:26 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -518,17 +518,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Ben Rice</t>
+          <t>Hunter Goodman</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+278</t>
+          <t>+218</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>31.4%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -539,24 +539,24 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>31.4%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Yordan Alvarez</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+279</t>
+          <t>+278</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -567,24 +567,24 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>26.5%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hunter Goodman</t>
+          <t>Yordan Alvarez</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+297</t>
+          <t>+279</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>25.2%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -595,24 +595,24 @@
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>25.2%</t>
+          <t>26.4%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Jazz Chisholm</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+309</t>
+          <t>+287</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
@@ -635,12 +635,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+310</t>
+          <t>+297</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>25.2%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -651,24 +651,24 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>25.2%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Byron Buxton</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+318</t>
+          <t>+303</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>24.8%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -679,24 +679,24 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>24.8%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Max Muncy (LAD)</t>
+          <t>Jazz Chisholm</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+326</t>
+          <t>+309</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>24.4%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -707,24 +707,24 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>24.4%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Pete Alonso</t>
+          <t>Byron Buxton</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>+346</t>
+          <t>+318</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>23.9%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -735,24 +735,24 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Cody Bellinger</t>
+          <t>Max Muncy (LAD)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>+348</t>
+          <t>+327</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -763,24 +763,24 @@
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>23.4%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Junior Caminero</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+346</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -791,24 +791,24 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+358</t>
+          <t>+346</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -819,52 +819,52 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Samuel Basallo</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>+366</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>21.5%</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>21.5%</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Cody Bellinger</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>+348</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>22.3%</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>22.3%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Paul Goldschmidt</t>
+          <t>Marcell Ozuna</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>+372</t>
+          <t>+349</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>22.3%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -875,24 +875,24 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>22.3%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Marcell Ozuna</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+375</t>
+          <t>+350</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -903,24 +903,24 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Gunnar Henderson</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+375</t>
+          <t>+358</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -931,24 +931,24 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+379</t>
+          <t>+359</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -959,24 +959,24 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Kyle Manzardo</t>
+          <t>Gunnar Henderson</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+386</t>
+          <t>+367</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -987,24 +987,24 @@
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Rhys Hoskins</t>
+          <t>Paul Goldschmidt</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+388</t>
+          <t>+372</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>21.2%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1015,24 +1015,24 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>21.2%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Ryan McMahon</t>
+          <t>Samuel Basallo</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>+401</t>
+          <t>+383</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1043,52 +1043,52 @@
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Dalton Rushing</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>+402</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>19.9%</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>19.9%</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>+386</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>20.6%</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>20.6%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Ketel Marte</t>
+          <t>Kyle Manzardo</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>+416</t>
+          <t>+386</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>20.6%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1099,24 +1099,24 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>20.6%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Rhys Hoskins</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>+416</t>
+          <t>+388</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1127,24 +1127,24 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>20.5%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Gavin Sheets</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+423</t>
+          <t>+396</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1155,24 +1155,24 @@
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>20.2%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Esmerlyn Valdez</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1183,52 +1183,52 @@
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Troy Johnston</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>+434</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>18.7%</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>18.7%</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Ryan McMahon</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>+401</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>20.0%</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Freddie Freeman</t>
+          <t>Dalton Rushing</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>+437</t>
+          <t>+402</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1239,24 +1239,24 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>+439</t>
+          <t>+403</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1267,52 +1267,52 @@
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>19.9%</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>+441</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>18.5%</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>18.5%</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Colson Montgomery</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>+414</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Adley Rutschman</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>+459</t>
+          <t>+416</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>19.4%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1323,24 +1323,24 @@
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>19.4%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Dillon Dingler</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+460</t>
+          <t>+419</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1351,24 +1351,24 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>19.3%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Jasson Dominguez</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+423</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1379,24 +1379,24 @@
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Randal Grichuk</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>+478</t>
+          <t>+424</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1407,24 +1407,24 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Eugenio Suarez</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>+504</t>
+          <t>+426</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1435,24 +1435,24 @@
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Taylor Ward</t>
+          <t>Corbin Carroll</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+439</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1463,24 +1463,24 @@
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+439</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1491,24 +1491,24 @@
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>18.6%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Esmerlyn Valdez</t>
+          <t>Manny Machado</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+533</t>
+          <t>+440</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1519,52 +1519,52 @@
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Colton Cowser</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>+540</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>15.6%</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>15.6%</t>
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>+441</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>18.5%</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>18.5%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+548</t>
+          <t>+446</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1575,24 +1575,24 @@
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>18.3%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Carter Jensen</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+560</t>
+          <t>+450</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1603,24 +1603,24 @@
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>+565</t>
+          <t>+452</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1631,52 +1631,52 @@
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Jose Altuve</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>+577</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>14.8%</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>14.8%</t>
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Willson Contreras</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>+453</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>18.1%</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>18.1%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+455</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1687,24 +1687,24 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Nick Gonzales</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>+583</t>
+          <t>+460</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1715,24 +1715,24 @@
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Jasson Dominguez</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1743,24 +1743,24 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Jared Triolo</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>+587</t>
+          <t>+478</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1771,24 +1771,24 @@
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>17.3%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Adley Rutschman</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>+589</t>
+          <t>+485</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1799,24 +1799,24 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>17.1%</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Nick Gonzales</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>+591</t>
+          <t>+492</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1827,24 +1827,24 @@
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Endy Rodriguez</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>+594</t>
+          <t>+492</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1855,24 +1855,24 @@
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>16.9%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Nathaniel Lowe</t>
+          <t>Kerry Carpenter</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+497</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1883,24 +1883,24 @@
       <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Spencer Horwitz</t>
+          <t>Eugenio Suarez</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+596</t>
+          <t>+504</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1911,24 +1911,24 @@
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Daniel Schneemann</t>
+          <t>Colton Cowser</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>+597</t>
+          <t>+514</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1939,52 +1939,52 @@
       <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Travis Bazzana</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>+597</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>14.3%</t>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Salvador Perez</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>+515</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>16.3%</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>16.3%</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Henry Davis</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>+598</t>
+          <t>+517</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -1995,24 +1995,24 @@
       <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Jonathan Aranda</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+521</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2023,52 +2023,52 @@
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>16.1%</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>+610</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>14.1%</t>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Jones</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>+528</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>15.9%</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Lourdes Gurriel Jr.</t>
+          <t>JJ Wetherholt</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>+610</t>
+          <t>+534</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2079,52 +2079,52 @@
       <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>14.1%</t>
+          <t>15.8%</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Billy Cook</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>+610</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>14.1%</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>14.1%</t>
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Jac Caglianone</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>+538</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>15.7%</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>15.7%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Arias</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+540</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2135,24 +2135,24 @@
       <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Jeremy Pena</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+548</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2163,24 +2163,24 @@
       <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Kahlil Watson</t>
+          <t>Taylor Ward</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>+640</t>
+          <t>+553</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -2191,24 +2191,24 @@
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>15.3%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Yainer Diaz</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+559</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -2219,24 +2219,24 @@
       <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Ryan Ward</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+560</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2247,24 +2247,24 @@
       <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Taylor Trammell</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+561</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2275,24 +2275,24 @@
       <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Cole Carrigg</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+564</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2303,24 +2303,24 @@
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Brayan Rocchio</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+565</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -2331,52 +2331,52 @@
       <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>J.C. Escarra</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>+720</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>12.2%</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>12.2%</t>
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>+567</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr"/>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Cam Smith</t>
+          <t>Billy Cook</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+571</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -2387,24 +2387,24 @@
       <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Spencer Steer</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+576</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2415,24 +2415,24 @@
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Jordan Lawlar</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+577</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -2443,24 +2443,24 @@
       <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+580</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2471,24 +2471,24 @@
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Lane Thomas</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+582</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2499,24 +2499,24 @@
       <c r="E73" s="2" t="inlineStr"/>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Xander Bogaerts</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+585</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -2527,24 +2527,24 @@
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Royce Lewis</t>
+          <t>Michael Massey</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+586</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2555,24 +2555,24 @@
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Joey Loperfido</t>
+          <t>Tyler Stephenson</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+589</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2583,24 +2583,24 @@
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>14.5%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Tyler Freeman</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+594</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2611,24 +2611,24 @@
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Ildemaro Vargas</t>
+          <t>Nathaniel Lowe</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+595</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -2639,24 +2639,24 @@
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>14.4%</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Blaze Alexander</t>
+          <t>Daniel Schneemann</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+597</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2667,24 +2667,24 @@
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Jose Caballero</t>
+          <t>Hao-Yu Lee</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+597</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -2695,24 +2695,24 @@
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+597</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -2723,24 +2723,24 @@
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Tristan Gray</t>
+          <t>CJ Abrams</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+599</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2751,24 +2751,24 @@
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+600</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -2779,24 +2779,24 @@
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Lourdes Gurriel Jr.</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+610</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -2807,52 +2807,52 @@
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>14.1%</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>Alex Freeland</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>+890</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>10.1%</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr"/>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>10.1%</t>
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Kevin McGonigle</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr"/>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Patrick Bailey</t>
+          <t>Gabriel Arias</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -2863,24 +2863,24 @@
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Noelvi Marte</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+620</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -2891,24 +2891,24 @@
       <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>13.9%</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Blake Dunn</t>
+          <t>Jeremy Pena</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+630</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -2919,24 +2919,24 @@
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>13.7%</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>LuJames Groover</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -2947,24 +2947,24 @@
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Kahlil Watson</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+640</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -2975,24 +2975,24 @@
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>7.8%</t>
+          <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Troy Johnston</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>+1520</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -3003,7 +3003,2023 @@
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr">
         <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Luis Garcia (WAS)</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Braden Montgomery</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Yainer Diaz</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Trammell</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Nathan Church</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Colt Keith</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>+670</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>13.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Ceddanne Rafaela</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel Moreno</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Curtis Mead</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Brayan Rocchio</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>J.C. Escarra</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>12.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>John Rave</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Cam Smith</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Steer</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Jordan Lawlar</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Nolan Arenado</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Victor Mesa Jr.</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Daylen Lile</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Yandy Diaz</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Royce Lewis</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Brooks Lee</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Jared Triolo</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Cedric Mullins</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr"/>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Joey Loperfido</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Michael Gasper</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr"/>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Ildemaro Vargas</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>+780</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Spencer Horwitz</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>+780</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>11.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Blaze Alexander</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Jose Caballero</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr"/>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Geraldo Perdomo</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr"/>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Karros</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr"/>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>James Outman</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr"/>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>11.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Tyler Freeman</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr"/>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Keibert Ruiz</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>+830</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr"/>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Rodolfo Duran</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr"/>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Jimmy Crooks</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr"/>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Lars Nootbaar</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr"/>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Isaac Collins</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr"/>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Blaze Jordan</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>+870</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr"/>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>10.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Tristan Gray</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>10.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Patrick Bailey</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr"/>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Trevor Larnach</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Alex Freeland</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr"/>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Leody Taveras</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr"/>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>Jake McCarthy</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr"/>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Maikel Garcia</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr"/>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Junior Perez</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr"/>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Marcelo Mayer</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr"/>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Masyn Winn</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr"/>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Narvaez</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Noelvi Marte</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Will Wagner</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>9.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Chase Meidroth</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr"/>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Edgar Quero</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr"/>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Jacob Young</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr"/>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Blake Dunn</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr"/>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Richie Palacios</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr"/>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Nick Loftin</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr"/>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>8.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>LuJames Groover</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr"/>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>8.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Caleb Durbin</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr"/>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>Samad Taylor</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr"/>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Walls</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>+1160</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr"/>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>Victor Caratini</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>+1160</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr"/>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>7.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Zach McKinstry</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>+1180</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>7.8%</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr"/>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>7.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Sam Antonacci</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>7.7%</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr"/>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>7.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Hunter Feduccia</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>+1220</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr"/>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>Luisangel Acuna</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>7.1%</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr"/>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>7.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>Nasim Nunez</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
           <t>6.2%</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr"/>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>Luke Keaschall</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>+1520</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr"/>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>Isiah Kiner-Falefa</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>+1520</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr"/>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>6.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>Chandler Simpson</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>+1600</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>5.9%</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr"/>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>5.9%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update odds files - Fri Jun 19 05:13:04 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -803,12 +803,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>+330</t>
+          <t>+332</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
@@ -1216,28 +1216,28 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Esmerlyn Valdez</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>+400</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>20.0%</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>20.0%</t>
         </is>
@@ -1468,28 +1468,28 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Randal Grichuk</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>+424</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>19.1%</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>19.1%</t>
         </is>
@@ -2506,12 +2506,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Ryan Ward</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>+559</t>
+          <t>+560</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -2534,17 +2534,17 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Ryan Ward</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>+560</t>
+          <t>+561</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2555,19 +2555,19 @@
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.1%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Cole Carrigg</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>+561</t>
+          <t>+564</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -2590,17 +2590,17 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Cole Carrigg</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>+564</t>
+          <t>+565</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -2611,19 +2611,19 @@
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Cam Smith</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>+565</t>
+          <t>+567</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -2644,56 +2644,56 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>Cam Smith</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>+567</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr"/>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr"/>
+      <c r="F79" s="3" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>+567</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Alec Burleson</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr"/>
-      <c r="F80" s="3" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>
@@ -2702,17 +2702,17 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Billy Cook</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>+568</t>
+          <t>+571</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -2723,24 +2723,24 @@
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Billy Cook</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>+571</t>
+          <t>+576</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2751,24 +2751,24 @@
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>+576</t>
+          <t>+580</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -2779,19 +2779,19 @@
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+581</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -3122,7 +3122,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3148,28 +3148,28 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>Kevin McGonigle</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Dylan Crews</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
         <is>
           <t>+620</t>
         </is>
       </c>
-      <c r="C97" s="3" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>13.9%</t>
         </is>
       </c>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E97" s="3" t="inlineStr"/>
-      <c r="F97" s="3" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
         <is>
           <t>13.9%</t>
         </is>
@@ -3178,7 +3178,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Kevin McGonigle</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3234,7 +3234,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Jackson Holliday</t>
+          <t>Seiya Suzuki</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3262,7 +3262,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Seiya Suzuki</t>
+          <t>Jackson Holliday</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -3290,7 +3290,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Luis Garcia (WAS)</t>
+          <t>Troy Johnston</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -3318,7 +3318,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Troy Johnston</t>
+          <t>Luis Garcia (WAS)</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Rob Refsnyder</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Rob Refsnyder</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -4606,17 +4606,17 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Rodolfo Duran</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+850</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -4627,14 +4627,14 @@
       <c r="E149" s="2" t="inlineStr"/>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.5%</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Dansby Swanson</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -4662,17 +4662,17 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Dansby Swanson</t>
+          <t>Jimmy Crooks</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -4683,14 +4683,14 @@
       <c r="E151" s="2" t="inlineStr"/>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Crooks</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -4718,7 +4718,7 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Rodolfo Duran</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -4856,28 +4856,28 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="3" t="inlineStr">
+      <c r="A158" s="2" t="inlineStr">
         <is>
           <t>Jake McCarthy</t>
         </is>
       </c>
-      <c r="B158" s="3" t="inlineStr">
+      <c r="B158" s="2" t="inlineStr">
         <is>
           <t>+900</t>
         </is>
       </c>
-      <c r="C158" s="3" t="inlineStr">
+      <c r="C158" s="2" t="inlineStr">
         <is>
           <t>10.0%</t>
         </is>
       </c>
-      <c r="D158" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E158" s="3" t="inlineStr"/>
-      <c r="F158" s="3" t="inlineStr">
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr"/>
+      <c r="F158" s="2" t="inlineStr">
         <is>
           <t>10.0%</t>
         </is>

</xml_diff>

<commit_message>
Update odds files - Sun Jun 21 04:48:28 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -600,47 +600,47 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Max Muncy (LAD)</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>+265</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>27.4%</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>27.4%</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Schwarber</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>+264</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>27.5%</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>27.5%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Max Muncy (LAD)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+288</t>
+          <t>+265</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>27.4%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -651,35 +651,35 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>27.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>James Wood</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>+288</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>25.8%</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Kyle Schwarber</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>+290</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>25.6%</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>25.6%</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>25.8%</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Christian Walker</t>
+          <t>Jordan Walker</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -994,17 +994,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Jordan Walker</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>+373</t>
+          <t>+384</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1015,7 +1015,7 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
@@ -1048,28 +1048,28 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Austin Wells</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>+386</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>20.6%</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>20.6%</t>
         </is>
@@ -1524,28 +1524,28 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Ryan Ward</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>+445</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>18.3%</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>18.3%</t>
         </is>
@@ -1608,42 +1608,42 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Austin Riley</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>+458</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>17.9%</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>17.9%</t>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Tyler Callihan</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>+461</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>17.8%</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Tyler Callihan</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+461</t>
+          <t>+462</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1666,17 +1666,17 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+462</t>
+          <t>+464</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1687,126 +1687,126 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.7%</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Mookie Betts</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>+464</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>17.7%</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>17.7%</t>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Paredes</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>+468</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>17.6%</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>Isaac Paredes</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>+468</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>17.6%</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>17.6%</t>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Alec Burleson</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>+475</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>17.4%</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Alec Burleson</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-   